<commit_message>
Roll Upstart and Google One forward to Sep 7
Both came out of the account on Aug 7 alongside the Compunnel paycheck, so
they are already reflected in the $71.17 beginning balance. Confirmed with
the user. Week 1 now shows only what is genuinely still ahead: Central Maine
Power on Aug 10, Bruno's paycheck on Aug 12, and Apple: iCloud on Aug 13.

Every Next Due Date on the Recurring tab now falls on or after the Aug 7
start date, so no transaction is counted twice.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0171RmRt5NEruH3aRWtNMF8Q
</commit_message>
<xml_diff>
--- a/Weekly_Cash_Flow_Survival.xlsx
+++ b/Weekly_Cash_Flow_Survival.xlsx
@@ -189,7 +189,7 @@
     <t xml:space="preserve">Amounts are entered as positive numbers. The Type column (Income or Expense) decides the sign, so a $90 paycheck is Type = Income, amount 90.</t>
   </si>
   <si>
-    <t xml:space="preserve">The sheet opens on Fri Aug 7, 2026 with $71.17 already in hand. The Aug 7 Compunnel paycheck had already landed by then, so its Next Due Date is Aug 14 — the first one still to come. Bruno's, Apple: Claude, OpenAI and Obsidian were rolled forward for the same reason. Google One ($4.99) and Upstart ($500) are still shown as due on Aug 7; if those already came out of the account, roll them forward to Sep 7 too.</t>
+    <t xml:space="preserve">The sheet opens on Fri Aug 7, 2026 with $71.17 already in hand. Everything that had already moved by that morning was rolled forward to its next occurrence, so the projection never counts the same money twice: the Compunnel paycheck (now Aug 14), Upstart and Google One (now Sep 7), and Bruno's, Apple: Claude, OpenAI and Obsidian. Confirmed with the user on Aug 7, 2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Progressive Insurance ($143.37) was cut off at the bottom of the third screenshot, so its due date is set to Aug 31, 2026. Correct it on the Recurring tab if that is wrong.</t>
@@ -1886,7 +1886,7 @@
         <v>42</v>
       </c>
       <c r="F10" s="22" t="n">
-        <v>46241</v>
+        <v>46272</v>
       </c>
       <c r="G10" s="20" t="s">
         <v>72</v>
@@ -1916,7 +1916,7 @@
         <v>42</v>
       </c>
       <c r="F11" s="17" t="n">
-        <v>46241</v>
+        <v>46272</v>
       </c>
       <c r="G11" s="15" t="s">
         <v>72</v>
@@ -2601,11 +2601,11 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="9" t="str">
         <f aca="false">IFERROR(INDEX(Schedule!$C$4:$C$483,MATCH(1001,Schedule!$K$4:$K$483,0)),"")</f>
-        <v>Google One</v>
+        <v>Central Maine Power Co.</v>
       </c>
       <c r="C15" s="34" t="n">
         <f aca="false">IF($B15="","",INDEX(Schedule!$G$4:$G$483,MATCH(1001,Schedule!$K$4:$K$483,0)))</f>
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="D15" s="35" t="str">
         <f aca="false">IF($B15="","",INDEX(Schedule!$D$4:$D$483,MATCH(1001,Schedule!$K$4:$K$483,0)))</f>
@@ -2613,20 +2613,20 @@
       </c>
       <c r="E15" s="36" t="n">
         <f aca="false">IF($B15="","",INDEX(Schedule!$E$4:$E$483,MATCH(1001,Schedule!$K$4:$K$483,0)))</f>
-        <v>4.99</v>
+        <v>163.5</v>
       </c>
       <c r="F15" s="16"/>
       <c r="G15" s="36" t="n">
         <f aca="false">IF($B15="","",IF($F15&lt;&gt;"",$F15,$E15))</f>
-        <v>4.99</v>
+        <v>163.5</v>
       </c>
       <c r="H15" s="36" t="n">
         <f aca="false">IF($B15="",0,IF($D15="Income",$G15,-$G15))</f>
-        <v>-4.99</v>
+        <v>-163.5</v>
       </c>
       <c r="I15" s="37" t="n">
         <f aca="false">IF($B15="","",$I$13+SUM($H$15:$H15))</f>
-        <v>66.18</v>
+        <v>-92.33</v>
       </c>
       <c r="J15" s="38" t="str">
         <f aca="true">IF($B15="","",IF($F15&lt;&gt;"","PAID",IF($C15&lt;TODAY(),"PAST DUE",IF($C15&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -2636,32 +2636,32 @@
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="9" t="str">
         <f aca="false">IFERROR(INDEX(Schedule!$C$4:$C$483,MATCH(1002,Schedule!$K$4:$K$483,0)),"")</f>
-        <v>Upstart (loan)</v>
+        <v>Bruno's Restaurant (paycheck)</v>
       </c>
       <c r="C16" s="34" t="n">
         <f aca="false">IF($B16="","",INDEX(Schedule!$G$4:$G$483,MATCH(1002,Schedule!$K$4:$K$483,0)))</f>
-        <v>46241</v>
+        <v>46246</v>
       </c>
       <c r="D16" s="35" t="str">
         <f aca="false">IF($B16="","",INDEX(Schedule!$D$4:$D$483,MATCH(1002,Schedule!$K$4:$K$483,0)))</f>
-        <v>Expense</v>
+        <v>Income</v>
       </c>
       <c r="E16" s="36" t="n">
         <f aca="false">IF($B16="","",INDEX(Schedule!$E$4:$E$483,MATCH(1002,Schedule!$K$4:$K$483,0)))</f>
-        <v>500</v>
+        <v>90</v>
       </c>
       <c r="F16" s="16"/>
       <c r="G16" s="36" t="n">
         <f aca="false">IF($B16="","",IF($F16&lt;&gt;"",$F16,$E16))</f>
-        <v>500</v>
+        <v>90</v>
       </c>
       <c r="H16" s="36" t="n">
         <f aca="false">IF($B16="",0,IF($D16="Income",$G16,-$G16))</f>
-        <v>-500</v>
+        <v>90</v>
       </c>
       <c r="I16" s="37" t="n">
         <f aca="false">IF($B16="","",$I$13+SUM($H$15:$H16))</f>
-        <v>-433.82</v>
+        <v>-2.33</v>
       </c>
       <c r="J16" s="38" t="str">
         <f aca="true">IF($B16="","",IF($F16&lt;&gt;"","PAID",IF($C16&lt;TODAY(),"PAST DUE",IF($C16&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -2671,11 +2671,11 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="9" t="str">
         <f aca="false">IFERROR(INDEX(Schedule!$C$4:$C$483,MATCH(1003,Schedule!$K$4:$K$483,0)),"")</f>
-        <v>Central Maine Power Co.</v>
+        <v>Apple: iCloud</v>
       </c>
       <c r="C17" s="34" t="n">
         <f aca="false">IF($B17="","",INDEX(Schedule!$G$4:$G$483,MATCH(1003,Schedule!$K$4:$K$483,0)))</f>
-        <v>46244</v>
+        <v>46247</v>
       </c>
       <c r="D17" s="35" t="str">
         <f aca="false">IF($B17="","",INDEX(Schedule!$D$4:$D$483,MATCH(1003,Schedule!$K$4:$K$483,0)))</f>
@@ -2683,20 +2683,20 @@
       </c>
       <c r="E17" s="36" t="n">
         <f aca="false">IF($B17="","",INDEX(Schedule!$E$4:$E$483,MATCH(1003,Schedule!$K$4:$K$483,0)))</f>
-        <v>163.5</v>
+        <v>2.99</v>
       </c>
       <c r="F17" s="16"/>
       <c r="G17" s="36" t="n">
         <f aca="false">IF($B17="","",IF($F17&lt;&gt;"",$F17,$E17))</f>
-        <v>163.5</v>
+        <v>2.99</v>
       </c>
       <c r="H17" s="36" t="n">
         <f aca="false">IF($B17="",0,IF($D17="Income",$G17,-$G17))</f>
-        <v>-163.5</v>
+        <v>-2.99</v>
       </c>
       <c r="I17" s="37" t="n">
         <f aca="false">IF($B17="","",$I$13+SUM($H$15:$H17))</f>
-        <v>-597.32</v>
+        <v>-5.31999999999999</v>
       </c>
       <c r="J17" s="38" t="str">
         <f aca="true">IF($B17="","",IF($F17&lt;&gt;"","PAID",IF($C17&lt;TODAY(),"PAST DUE",IF($C17&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -2706,71 +2706,71 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="9" t="str">
         <f aca="false">IFERROR(INDEX(Schedule!$C$4:$C$483,MATCH(1004,Schedule!$K$4:$K$483,0)),"")</f>
-        <v>Bruno's Restaurant (paycheck)</v>
-      </c>
-      <c r="C18" s="34" t="n">
+        <v/>
+      </c>
+      <c r="C18" s="34" t="str">
         <f aca="false">IF($B18="","",INDEX(Schedule!$G$4:$G$483,MATCH(1004,Schedule!$K$4:$K$483,0)))</f>
-        <v>46246</v>
+        <v/>
       </c>
       <c r="D18" s="35" t="str">
         <f aca="false">IF($B18="","",INDEX(Schedule!$D$4:$D$483,MATCH(1004,Schedule!$K$4:$K$483,0)))</f>
-        <v>Income</v>
-      </c>
-      <c r="E18" s="36" t="n">
+        <v/>
+      </c>
+      <c r="E18" s="36" t="str">
         <f aca="false">IF($B18="","",INDEX(Schedule!$E$4:$E$483,MATCH(1004,Schedule!$K$4:$K$483,0)))</f>
-        <v>90</v>
+        <v/>
       </c>
       <c r="F18" s="16"/>
-      <c r="G18" s="36" t="n">
+      <c r="G18" s="36" t="str">
         <f aca="false">IF($B18="","",IF($F18&lt;&gt;"",$F18,$E18))</f>
-        <v>90</v>
+        <v/>
       </c>
       <c r="H18" s="36" t="n">
         <f aca="false">IF($B18="",0,IF($D18="Income",$G18,-$G18))</f>
-        <v>90</v>
-      </c>
-      <c r="I18" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="37" t="str">
         <f aca="false">IF($B18="","",$I$13+SUM($H$15:$H18))</f>
-        <v>-507.32</v>
+        <v/>
       </c>
       <c r="J18" s="38" t="str">
         <f aca="true">IF($B18="","",IF($F18&lt;&gt;"","PAID",IF($C18&lt;TODAY(),"PAST DUE",IF($C18&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
-        <v>DUE</v>
+        <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="9" t="str">
         <f aca="false">IFERROR(INDEX(Schedule!$C$4:$C$483,MATCH(1005,Schedule!$K$4:$K$483,0)),"")</f>
-        <v>Apple: iCloud</v>
-      </c>
-      <c r="C19" s="34" t="n">
+        <v/>
+      </c>
+      <c r="C19" s="34" t="str">
         <f aca="false">IF($B19="","",INDEX(Schedule!$G$4:$G$483,MATCH(1005,Schedule!$K$4:$K$483,0)))</f>
-        <v>46247</v>
+        <v/>
       </c>
       <c r="D19" s="35" t="str">
         <f aca="false">IF($B19="","",INDEX(Schedule!$D$4:$D$483,MATCH(1005,Schedule!$K$4:$K$483,0)))</f>
-        <v>Expense</v>
-      </c>
-      <c r="E19" s="36" t="n">
+        <v/>
+      </c>
+      <c r="E19" s="36" t="str">
         <f aca="false">IF($B19="","",INDEX(Schedule!$E$4:$E$483,MATCH(1005,Schedule!$K$4:$K$483,0)))</f>
-        <v>2.99</v>
+        <v/>
       </c>
       <c r="F19" s="16"/>
-      <c r="G19" s="36" t="n">
+      <c r="G19" s="36" t="str">
         <f aca="false">IF($B19="","",IF($F19&lt;&gt;"",$F19,$E19))</f>
-        <v>2.99</v>
+        <v/>
       </c>
       <c r="H19" s="36" t="n">
         <f aca="false">IF($B19="",0,IF($D19="Income",$G19,-$G19))</f>
-        <v>-2.99</v>
-      </c>
-      <c r="I19" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="37" t="str">
         <f aca="false">IF($B19="","",$I$13+SUM($H$15:$H19))</f>
-        <v>-510.31</v>
+        <v/>
       </c>
       <c r="J19" s="38" t="str">
         <f aca="true">IF($B19="","",IF($F19&lt;&gt;"","PAID",IF($C19&lt;TODAY(),"PAST DUE",IF($C19&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
-        <v>DUE</v>
+        <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3107,7 +3107,7 @@
       <c r="D32" s="42"/>
       <c r="E32" s="43" t="n">
         <f aca="false">SUM($E$15:$E$31)</f>
-        <v>761.48</v>
+        <v>256.49</v>
       </c>
       <c r="F32" s="43" t="n">
         <f aca="false">SUM($F$15:$F$24)</f>
@@ -3115,15 +3115,15 @@
       </c>
       <c r="G32" s="43" t="n">
         <f aca="false">SUM($G$15:$G$31)</f>
-        <v>761.48</v>
+        <v>256.49</v>
       </c>
       <c r="H32" s="43" t="n">
         <f aca="false">SUM($H$15:$H$31)</f>
-        <v>-581.48</v>
+        <v>-76.49</v>
       </c>
       <c r="I32" s="44" t="n">
         <f aca="false">$I$13+SUM($H$15:$H$31)</f>
-        <v>-510.31</v>
+        <v>-5.31999999999999</v>
       </c>
       <c r="J32" s="45" t="str">
         <f aca="false">IF($I$32&lt;0,"SHORTFALL",IF($I$32&lt;$E$7,"TIGHT","OK"))</f>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="K32" s="23" t="str">
         <f aca="false">"Income "&amp;TEXT(SUMIF($D$15:$D$31,"Income",$G$15:$G$31),"$#,##0.00")&amp;"   less expenses "&amp;TEXT(SUMIF($D$15:$D$31,"Expense",$G$15:$G$31),"$#,##0.00")&amp;"   =  net "&amp;TEXT($H$32,"$#,##0.00")</f>
-        <v>Income $90.00   less expenses $671.48   =  net -$581.48</v>
+        <v>Income $90.00   less expenses $166.49   =  net -$76.49</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3149,7 +3149,7 @@
       <c r="H34" s="30"/>
       <c r="I34" s="32" t="n">
         <f aca="false">$I$32</f>
-        <v>-510.31</v>
+        <v>-5.31999999999999</v>
       </c>
       <c r="J34" s="30"/>
       <c r="K34" s="26" t="str">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="I36" s="37" t="n">
         <f aca="false">IF($B36="","",$I$34+SUM($H$36:$H36))</f>
-        <v>279.69</v>
+        <v>784.68</v>
       </c>
       <c r="J36" s="38" t="str">
         <f aca="true">IF($B36="","",IF($F36&lt;&gt;"","PAID",IF($C36&lt;TODAY(),"PAST DUE",IF($C36&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -3249,7 +3249,7 @@
       </c>
       <c r="I37" s="37" t="n">
         <f aca="false">IF($B37="","",$I$34+SUM($H$36:$H37))</f>
-        <v>-70.31</v>
+        <v>434.68</v>
       </c>
       <c r="J37" s="38" t="str">
         <f aca="true">IF($B37="","",IF($F37&lt;&gt;"","PAID",IF($C37&lt;TODAY(),"PAST DUE",IF($C37&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -3284,7 +3284,7 @@
       </c>
       <c r="I38" s="37" t="n">
         <f aca="false">IF($B38="","",$I$34+SUM($H$36:$H38))</f>
-        <v>-241.41</v>
+        <v>263.58</v>
       </c>
       <c r="J38" s="38" t="str">
         <f aca="true">IF($B38="","",IF($F38&lt;&gt;"","PAID",IF($C38&lt;TODAY(),"PAST DUE",IF($C38&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -3319,7 +3319,7 @@
       </c>
       <c r="I39" s="37" t="n">
         <f aca="false">IF($B39="","",$I$34+SUM($H$36:$H39))</f>
-        <v>-286.41</v>
+        <v>218.58</v>
       </c>
       <c r="J39" s="38" t="str">
         <f aca="true">IF($B39="","",IF($F39&lt;&gt;"","PAID",IF($C39&lt;TODAY(),"PAST DUE",IF($C39&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -3354,7 +3354,7 @@
       </c>
       <c r="I40" s="37" t="n">
         <f aca="false">IF($B40="","",$I$34+SUM($H$36:$H40))</f>
-        <v>-303.4</v>
+        <v>201.59</v>
       </c>
       <c r="J40" s="38" t="str">
         <f aca="true">IF($B40="","",IF($F40&lt;&gt;"","PAID",IF($C40&lt;TODAY(),"PAST DUE",IF($C40&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -3389,7 +3389,7 @@
       </c>
       <c r="I41" s="37" t="n">
         <f aca="false">IF($B41="","",$I$34+SUM($H$36:$H41))</f>
-        <v>-213.4</v>
+        <v>291.59</v>
       </c>
       <c r="J41" s="38" t="str">
         <f aca="true">IF($B41="","",IF($F41&lt;&gt;"","PAID",IF($C41&lt;TODAY(),"PAST DUE",IF($C41&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -3711,11 +3711,11 @@
       </c>
       <c r="I53" s="44" t="n">
         <f aca="false">$I$34+SUM($H$36:$H$52)</f>
-        <v>-213.4</v>
+        <v>291.59</v>
       </c>
       <c r="J53" s="45" t="str">
         <f aca="false">IF($I$53&lt;0,"SHORTFALL",IF($I$53&lt;$E$7,"TIGHT","OK"))</f>
-        <v>SHORTFALL</v>
+        <v>OK</v>
       </c>
       <c r="K53" s="23" t="str">
         <f aca="false">"Income "&amp;TEXT(SUMIF($D$36:$D$52,"Income",$G$36:$G$52),"$#,##0.00")&amp;"   less expenses "&amp;TEXT(SUMIF($D$36:$D$52,"Expense",$G$36:$G$52),"$#,##0.00")&amp;"   =  net "&amp;TEXT($H$53,"$#,##0.00")</f>
@@ -3737,7 +3737,7 @@
       <c r="H55" s="30"/>
       <c r="I55" s="32" t="n">
         <f aca="false">$I$53</f>
-        <v>-213.4</v>
+        <v>291.59</v>
       </c>
       <c r="J55" s="30"/>
       <c r="K55" s="26" t="str">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="I57" s="37" t="n">
         <f aca="false">IF($B57="","",$I$55+SUM($H$57:$H57))</f>
-        <v>576.6</v>
+        <v>1081.59</v>
       </c>
       <c r="J57" s="38" t="str">
         <f aca="true">IF($B57="","",IF($F57&lt;&gt;"","PAID",IF($C57&lt;TODAY(),"PAST DUE",IF($C57&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -3837,7 +3837,7 @@
       </c>
       <c r="I58" s="37" t="n">
         <f aca="false">IF($B58="","",$I$55+SUM($H$57:$H58))</f>
-        <v>562.9</v>
+        <v>1067.89</v>
       </c>
       <c r="J58" s="38" t="str">
         <f aca="true">IF($B58="","",IF($F58&lt;&gt;"","PAID",IF($C58&lt;TODAY(),"PAST DUE",IF($C58&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -3872,7 +3872,7 @@
       </c>
       <c r="I59" s="37" t="n">
         <f aca="false">IF($B59="","",$I$55+SUM($H$57:$H59))</f>
-        <v>519.03</v>
+        <v>1024.02</v>
       </c>
       <c r="J59" s="38" t="str">
         <f aca="true">IF($B59="","",IF($F59&lt;&gt;"","PAID",IF($C59&lt;TODAY(),"PAST DUE",IF($C59&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -3907,7 +3907,7 @@
       </c>
       <c r="I60" s="37" t="n">
         <f aca="false">IF($B60="","",$I$55+SUM($H$57:$H60))</f>
-        <v>609.03</v>
+        <v>1114.02</v>
       </c>
       <c r="J60" s="38" t="str">
         <f aca="true">IF($B60="","",IF($F60&lt;&gt;"","PAID",IF($C60&lt;TODAY(),"PAST DUE",IF($C60&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -4299,7 +4299,7 @@
       </c>
       <c r="I74" s="44" t="n">
         <f aca="false">$I$55+SUM($H$57:$H$73)</f>
-        <v>609.03</v>
+        <v>1114.02</v>
       </c>
       <c r="J74" s="45" t="str">
         <f aca="false">IF($I$74&lt;0,"SHORTFALL",IF($I$74&lt;$E$7,"TIGHT","OK"))</f>
@@ -4325,7 +4325,7 @@
       <c r="H76" s="30"/>
       <c r="I76" s="32" t="n">
         <f aca="false">$I$74</f>
-        <v>609.03</v>
+        <v>1114.02</v>
       </c>
       <c r="J76" s="30"/>
       <c r="K76" s="26" t="str">
@@ -4390,7 +4390,7 @@
       </c>
       <c r="I78" s="37" t="n">
         <f aca="false">IF($B78="","",$I$76+SUM($H$78:$H78))</f>
-        <v>1399.03</v>
+        <v>1904.02</v>
       </c>
       <c r="J78" s="38" t="str">
         <f aca="true">IF($B78="","",IF($F78&lt;&gt;"","PAID",IF($C78&lt;TODAY(),"PAST DUE",IF($C78&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -4425,7 +4425,7 @@
       </c>
       <c r="I79" s="37" t="n">
         <f aca="false">IF($B79="","",$I$76+SUM($H$78:$H79))</f>
-        <v>1249.03</v>
+        <v>1754.02</v>
       </c>
       <c r="J79" s="38" t="str">
         <f aca="true">IF($B79="","",IF($F79&lt;&gt;"","PAID",IF($C79&lt;TODAY(),"PAST DUE",IF($C79&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -4460,7 +4460,7 @@
       </c>
       <c r="I80" s="37" t="n">
         <f aca="false">IF($B80="","",$I$76+SUM($H$78:$H80))</f>
-        <v>899.03</v>
+        <v>1404.02</v>
       </c>
       <c r="J80" s="38" t="str">
         <f aca="true">IF($B80="","",IF($F80&lt;&gt;"","PAID",IF($C80&lt;TODAY(),"PAST DUE",IF($C80&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -4495,7 +4495,7 @@
       </c>
       <c r="I81" s="37" t="n">
         <f aca="false">IF($B81="","",$I$76+SUM($H$78:$H81))</f>
-        <v>755.66</v>
+        <v>1260.65</v>
       </c>
       <c r="J81" s="38" t="str">
         <f aca="true">IF($B81="","",IF($F81&lt;&gt;"","PAID",IF($C81&lt;TODAY(),"PAST DUE",IF($C81&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -4530,7 +4530,7 @@
       </c>
       <c r="I82" s="37" t="n">
         <f aca="false">IF($B82="","",$I$76+SUM($H$78:$H82))</f>
-        <v>845.66</v>
+        <v>1350.65</v>
       </c>
       <c r="J82" s="38" t="str">
         <f aca="true">IF($B82="","",IF($F82&lt;&gt;"","PAID",IF($C82&lt;TODAY(),"PAST DUE",IF($C82&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -4887,7 +4887,7 @@
       </c>
       <c r="I95" s="44" t="n">
         <f aca="false">$I$76+SUM($H$78:$H$94)</f>
-        <v>845.66</v>
+        <v>1350.65</v>
       </c>
       <c r="J95" s="45" t="str">
         <f aca="false">IF($I$95&lt;0,"SHORTFALL",IF($I$95&lt;$E$7,"TIGHT","OK"))</f>
@@ -4913,7 +4913,7 @@
       <c r="H97" s="30"/>
       <c r="I97" s="32" t="n">
         <f aca="false">$I$95</f>
-        <v>845.66</v>
+        <v>1350.65</v>
       </c>
       <c r="J97" s="30"/>
       <c r="K97" s="26" t="str">
@@ -4978,7 +4978,7 @@
       </c>
       <c r="I99" s="37" t="n">
         <f aca="false">IF($B99="","",$I$97+SUM($H$99:$H99))</f>
-        <v>1635.66</v>
+        <v>2140.65</v>
       </c>
       <c r="J99" s="38" t="str">
         <f aca="true">IF($B99="","",IF($F99&lt;&gt;"","PAID",IF($C99&lt;TODAY(),"PAST DUE",IF($C99&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5013,7 +5013,7 @@
       </c>
       <c r="I100" s="37" t="n">
         <f aca="false">IF($B100="","",$I$97+SUM($H$99:$H100))</f>
-        <v>1614.56</v>
+        <v>2119.55</v>
       </c>
       <c r="J100" s="38" t="str">
         <f aca="true">IF($B100="","",IF($F100&lt;&gt;"","PAID",IF($C100&lt;TODAY(),"PAST DUE",IF($C100&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5048,7 +5048,7 @@
       </c>
       <c r="I101" s="37" t="n">
         <f aca="false">IF($B101="","",$I$97+SUM($H$99:$H101))</f>
-        <v>1594.56</v>
+        <v>2099.55</v>
       </c>
       <c r="J101" s="38" t="str">
         <f aca="true">IF($B101="","",IF($F101&lt;&gt;"","PAID",IF($C101&lt;TODAY(),"PAST DUE",IF($C101&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5083,7 +5083,7 @@
       </c>
       <c r="I102" s="37" t="n">
         <f aca="false">IF($B102="","",$I$97+SUM($H$99:$H102))</f>
-        <v>1584.56</v>
+        <v>2089.55</v>
       </c>
       <c r="J102" s="38" t="str">
         <f aca="true">IF($B102="","",IF($F102&lt;&gt;"","PAID",IF($C102&lt;TODAY(),"PAST DUE",IF($C102&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5118,7 +5118,7 @@
       </c>
       <c r="I103" s="37" t="n">
         <f aca="false">IF($B103="","",$I$97+SUM($H$99:$H103))</f>
-        <v>1579.57</v>
+        <v>2084.56</v>
       </c>
       <c r="J103" s="38" t="str">
         <f aca="true">IF($B103="","",IF($F103&lt;&gt;"","PAID",IF($C103&lt;TODAY(),"PAST DUE",IF($C103&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5153,7 +5153,7 @@
       </c>
       <c r="I104" s="37" t="n">
         <f aca="false">IF($B104="","",$I$97+SUM($H$99:$H104))</f>
-        <v>1079.57</v>
+        <v>1584.56</v>
       </c>
       <c r="J104" s="38" t="str">
         <f aca="true">IF($B104="","",IF($F104&lt;&gt;"","PAID",IF($C104&lt;TODAY(),"PAST DUE",IF($C104&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5188,7 +5188,7 @@
       </c>
       <c r="I105" s="37" t="n">
         <f aca="false">IF($B105="","",$I$97+SUM($H$99:$H105))</f>
-        <v>1169.57</v>
+        <v>1674.56</v>
       </c>
       <c r="J105" s="38" t="str">
         <f aca="true">IF($B105="","",IF($F105&lt;&gt;"","PAID",IF($C105&lt;TODAY(),"PAST DUE",IF($C105&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5223,7 +5223,7 @@
       </c>
       <c r="I106" s="37" t="n">
         <f aca="false">IF($B106="","",$I$97+SUM($H$99:$H106))</f>
-        <v>1006.07</v>
+        <v>1511.06</v>
       </c>
       <c r="J106" s="38" t="str">
         <f aca="true">IF($B106="","",IF($F106&lt;&gt;"","PAID",IF($C106&lt;TODAY(),"PAST DUE",IF($C106&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5475,7 +5475,7 @@
       </c>
       <c r="I116" s="44" t="n">
         <f aca="false">$I$97+SUM($H$99:$H$115)</f>
-        <v>1006.07</v>
+        <v>1511.06</v>
       </c>
       <c r="J116" s="45" t="str">
         <f aca="false">IF($I$116&lt;0,"SHORTFALL",IF($I$116&lt;$E$7,"TIGHT","OK"))</f>
@@ -5501,7 +5501,7 @@
       <c r="H118" s="30"/>
       <c r="I118" s="32" t="n">
         <f aca="false">$I$116</f>
-        <v>1006.07</v>
+        <v>1511.06</v>
       </c>
       <c r="J118" s="30"/>
       <c r="K118" s="26" t="str">
@@ -5566,7 +5566,7 @@
       </c>
       <c r="I120" s="37" t="n">
         <f aca="false">IF($B120="","",$I$118+SUM($H$120:$H120))</f>
-        <v>1796.07</v>
+        <v>2301.06</v>
       </c>
       <c r="J120" s="38" t="str">
         <f aca="true">IF($B120="","",IF($F120&lt;&gt;"","PAID",IF($C120&lt;TODAY(),"PAST DUE",IF($C120&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5601,7 +5601,7 @@
       </c>
       <c r="I121" s="37" t="n">
         <f aca="false">IF($B121="","",$I$118+SUM($H$120:$H121))</f>
-        <v>1793.08</v>
+        <v>2298.07</v>
       </c>
       <c r="J121" s="38" t="str">
         <f aca="true">IF($B121="","",IF($F121&lt;&gt;"","PAID",IF($C121&lt;TODAY(),"PAST DUE",IF($C121&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5636,7 +5636,7 @@
       </c>
       <c r="I122" s="37" t="n">
         <f aca="false">IF($B122="","",$I$118+SUM($H$120:$H122))</f>
-        <v>1443.08</v>
+        <v>1948.07</v>
       </c>
       <c r="J122" s="38" t="str">
         <f aca="true">IF($B122="","",IF($F122&lt;&gt;"","PAID",IF($C122&lt;TODAY(),"PAST DUE",IF($C122&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5671,7 +5671,7 @@
       </c>
       <c r="I123" s="37" t="n">
         <f aca="false">IF($B123="","",$I$118+SUM($H$120:$H123))</f>
-        <v>1533.08</v>
+        <v>2038.07</v>
       </c>
       <c r="J123" s="38" t="str">
         <f aca="true">IF($B123="","",IF($F123&lt;&gt;"","PAID",IF($C123&lt;TODAY(),"PAST DUE",IF($C123&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5706,7 +5706,7 @@
       </c>
       <c r="I124" s="37" t="n">
         <f aca="false">IF($B124="","",$I$118+SUM($H$120:$H124))</f>
-        <v>1361.98</v>
+        <v>1866.97</v>
       </c>
       <c r="J124" s="38" t="str">
         <f aca="true">IF($B124="","",IF($F124&lt;&gt;"","PAID",IF($C124&lt;TODAY(),"PAST DUE",IF($C124&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5741,7 +5741,7 @@
       </c>
       <c r="I125" s="37" t="n">
         <f aca="false">IF($B125="","",$I$118+SUM($H$120:$H125))</f>
-        <v>1316.98</v>
+        <v>1821.97</v>
       </c>
       <c r="J125" s="38" t="str">
         <f aca="true">IF($B125="","",IF($F125&lt;&gt;"","PAID",IF($C125&lt;TODAY(),"PAST DUE",IF($C125&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6063,7 +6063,7 @@
       </c>
       <c r="I137" s="44" t="n">
         <f aca="false">$I$118+SUM($H$120:$H$136)</f>
-        <v>1316.98</v>
+        <v>1821.97</v>
       </c>
       <c r="J137" s="45" t="str">
         <f aca="false">IF($I$137&lt;0,"SHORTFALL",IF($I$137&lt;$E$7,"TIGHT","OK"))</f>
@@ -6089,7 +6089,7 @@
       <c r="H139" s="30"/>
       <c r="I139" s="32" t="n">
         <f aca="false">$I$137</f>
-        <v>1316.98</v>
+        <v>1821.97</v>
       </c>
       <c r="J139" s="30"/>
       <c r="K139" s="26" t="str">
@@ -6154,7 +6154,7 @@
       </c>
       <c r="I141" s="37" t="n">
         <f aca="false">IF($B141="","",$I$139+SUM($H$141:$H141))</f>
-        <v>2106.98</v>
+        <v>2611.97</v>
       </c>
       <c r="J141" s="38" t="str">
         <f aca="true">IF($B141="","",IF($F141&lt;&gt;"","PAID",IF($C141&lt;TODAY(),"PAST DUE",IF($C141&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6189,7 +6189,7 @@
       </c>
       <c r="I142" s="37" t="n">
         <f aca="false">IF($B142="","",$I$139+SUM($H$141:$H142))</f>
-        <v>2089.99</v>
+        <v>2594.98</v>
       </c>
       <c r="J142" s="38" t="str">
         <f aca="true">IF($B142="","",IF($F142&lt;&gt;"","PAID",IF($C142&lt;TODAY(),"PAST DUE",IF($C142&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6224,7 +6224,7 @@
       </c>
       <c r="I143" s="37" t="n">
         <f aca="false">IF($B143="","",$I$139+SUM($H$141:$H143))</f>
-        <v>2179.99</v>
+        <v>2684.98</v>
       </c>
       <c r="J143" s="38" t="str">
         <f aca="true">IF($B143="","",IF($F143&lt;&gt;"","PAID",IF($C143&lt;TODAY(),"PAST DUE",IF($C143&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6651,7 +6651,7 @@
       </c>
       <c r="I158" s="44" t="n">
         <f aca="false">$I$139+SUM($H$141:$H$157)</f>
-        <v>2179.99</v>
+        <v>2684.98</v>
       </c>
       <c r="J158" s="45" t="str">
         <f aca="false">IF($I$158&lt;0,"SHORTFALL",IF($I$158&lt;$E$7,"TIGHT","OK"))</f>
@@ -6677,7 +6677,7 @@
       <c r="H160" s="30"/>
       <c r="I160" s="32" t="n">
         <f aca="false">$I$158</f>
-        <v>2179.99</v>
+        <v>2684.98</v>
       </c>
       <c r="J160" s="30"/>
       <c r="K160" s="26" t="str">
@@ -6742,7 +6742,7 @@
       </c>
       <c r="I162" s="37" t="n">
         <f aca="false">IF($B162="","",$I$160+SUM($H$162:$H162))</f>
-        <v>2969.99</v>
+        <v>3474.98</v>
       </c>
       <c r="J162" s="38" t="str">
         <f aca="true">IF($B162="","",IF($F162&lt;&gt;"","PAID",IF($C162&lt;TODAY(),"PAST DUE",IF($C162&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6777,7 +6777,7 @@
       </c>
       <c r="I163" s="37" t="n">
         <f aca="false">IF($B163="","",$I$160+SUM($H$162:$H163))</f>
-        <v>2956.29</v>
+        <v>3461.28</v>
       </c>
       <c r="J163" s="38" t="str">
         <f aca="true">IF($B163="","",IF($F163&lt;&gt;"","PAID",IF($C163&lt;TODAY(),"PAST DUE",IF($C163&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6812,7 +6812,7 @@
       </c>
       <c r="I164" s="37" t="n">
         <f aca="false">IF($B164="","",$I$160+SUM($H$162:$H164))</f>
-        <v>2912.42</v>
+        <v>3417.41</v>
       </c>
       <c r="J164" s="38" t="str">
         <f aca="true">IF($B164="","",IF($F164&lt;&gt;"","PAID",IF($C164&lt;TODAY(),"PAST DUE",IF($C164&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6847,7 +6847,7 @@
       </c>
       <c r="I165" s="37" t="n">
         <f aca="false">IF($B165="","",$I$160+SUM($H$162:$H165))</f>
-        <v>3002.42</v>
+        <v>3507.41</v>
       </c>
       <c r="J165" s="38" t="str">
         <f aca="true">IF($B165="","",IF($F165&lt;&gt;"","PAID",IF($C165&lt;TODAY(),"PAST DUE",IF($C165&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6882,7 +6882,7 @@
       </c>
       <c r="I166" s="37" t="n">
         <f aca="false">IF($B166="","",$I$160+SUM($H$162:$H166))</f>
-        <v>2652.42</v>
+        <v>3157.41</v>
       </c>
       <c r="J166" s="38" t="str">
         <f aca="true">IF($B166="","",IF($F166&lt;&gt;"","PAID",IF($C166&lt;TODAY(),"PAST DUE",IF($C166&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6917,7 +6917,7 @@
       </c>
       <c r="I167" s="37" t="n">
         <f aca="false">IF($B167="","",$I$160+SUM($H$162:$H167))</f>
-        <v>2502.42</v>
+        <v>3007.41</v>
       </c>
       <c r="J167" s="38" t="str">
         <f aca="true">IF($B167="","",IF($F167&lt;&gt;"","PAID",IF($C167&lt;TODAY(),"PAST DUE",IF($C167&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6952,7 +6952,7 @@
       </c>
       <c r="I168" s="37" t="n">
         <f aca="false">IF($B168="","",$I$160+SUM($H$162:$H168))</f>
-        <v>2359.05</v>
+        <v>2864.04</v>
       </c>
       <c r="J168" s="38" t="str">
         <f aca="true">IF($B168="","",IF($F168&lt;&gt;"","PAID",IF($C168&lt;TODAY(),"PAST DUE",IF($C168&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7239,7 +7239,7 @@
       </c>
       <c r="I179" s="44" t="n">
         <f aca="false">$I$160+SUM($H$162:$H$178)</f>
-        <v>2359.05</v>
+        <v>2864.04</v>
       </c>
       <c r="J179" s="45" t="str">
         <f aca="false">IF($I$179&lt;0,"SHORTFALL",IF($I$179&lt;$E$7,"TIGHT","OK"))</f>
@@ -7265,7 +7265,7 @@
       <c r="H181" s="30"/>
       <c r="I181" s="32" t="n">
         <f aca="false">$I$179</f>
-        <v>2359.05</v>
+        <v>2864.04</v>
       </c>
       <c r="J181" s="30"/>
       <c r="K181" s="26" t="str">
@@ -7330,7 +7330,7 @@
       </c>
       <c r="I183" s="37" t="n">
         <f aca="false">IF($B183="","",$I$181+SUM($H$183:$H183))</f>
-        <v>3149.05</v>
+        <v>3654.04</v>
       </c>
       <c r="J183" s="38" t="str">
         <f aca="true">IF($B183="","",IF($F183&lt;&gt;"","PAID",IF($C183&lt;TODAY(),"PAST DUE",IF($C183&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7365,7 +7365,7 @@
       </c>
       <c r="I184" s="37" t="n">
         <f aca="false">IF($B184="","",$I$181+SUM($H$183:$H184))</f>
-        <v>3127.95</v>
+        <v>3632.94</v>
       </c>
       <c r="J184" s="38" t="str">
         <f aca="true">IF($B184="","",IF($F184&lt;&gt;"","PAID",IF($C184&lt;TODAY(),"PAST DUE",IF($C184&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7400,7 +7400,7 @@
       </c>
       <c r="I185" s="37" t="n">
         <f aca="false">IF($B185="","",$I$181+SUM($H$183:$H185))</f>
-        <v>3107.95</v>
+        <v>3612.94</v>
       </c>
       <c r="J185" s="38" t="str">
         <f aca="true">IF($B185="","",IF($F185&lt;&gt;"","PAID",IF($C185&lt;TODAY(),"PAST DUE",IF($C185&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7435,7 +7435,7 @@
       </c>
       <c r="I186" s="37" t="n">
         <f aca="false">IF($B186="","",$I$181+SUM($H$183:$H186))</f>
-        <v>3097.95</v>
+        <v>3602.94</v>
       </c>
       <c r="J186" s="38" t="str">
         <f aca="true">IF($B186="","",IF($F186&lt;&gt;"","PAID",IF($C186&lt;TODAY(),"PAST DUE",IF($C186&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7470,7 +7470,7 @@
       </c>
       <c r="I187" s="37" t="n">
         <f aca="false">IF($B187="","",$I$181+SUM($H$183:$H187))</f>
-        <v>3187.95</v>
+        <v>3692.94</v>
       </c>
       <c r="J187" s="38" t="str">
         <f aca="true">IF($B187="","",IF($F187&lt;&gt;"","PAID",IF($C187&lt;TODAY(),"PAST DUE",IF($C187&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7505,7 +7505,7 @@
       </c>
       <c r="I188" s="37" t="n">
         <f aca="false">IF($B188="","",$I$181+SUM($H$183:$H188))</f>
-        <v>3182.96</v>
+        <v>3687.95</v>
       </c>
       <c r="J188" s="38" t="str">
         <f aca="true">IF($B188="","",IF($F188&lt;&gt;"","PAID",IF($C188&lt;TODAY(),"PAST DUE",IF($C188&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7540,7 +7540,7 @@
       </c>
       <c r="I189" s="37" t="n">
         <f aca="false">IF($B189="","",$I$181+SUM($H$183:$H189))</f>
-        <v>2682.96</v>
+        <v>3187.95</v>
       </c>
       <c r="J189" s="38" t="str">
         <f aca="true">IF($B189="","",IF($F189&lt;&gt;"","PAID",IF($C189&lt;TODAY(),"PAST DUE",IF($C189&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7827,7 +7827,7 @@
       </c>
       <c r="I200" s="44" t="n">
         <f aca="false">$I$181+SUM($H$183:$H$199)</f>
-        <v>2682.96</v>
+        <v>3187.95</v>
       </c>
       <c r="J200" s="45" t="str">
         <f aca="false">IF($I$200&lt;0,"SHORTFALL",IF($I$200&lt;$E$7,"TIGHT","OK"))</f>
@@ -7853,7 +7853,7 @@
       <c r="H202" s="30"/>
       <c r="I202" s="32" t="n">
         <f aca="false">$I$200</f>
-        <v>2682.96</v>
+        <v>3187.95</v>
       </c>
       <c r="J202" s="30"/>
       <c r="K202" s="26" t="str">
@@ -7918,7 +7918,7 @@
       </c>
       <c r="I204" s="37" t="n">
         <f aca="false">IF($B204="","",$I$202+SUM($H$204:$H204))</f>
-        <v>3472.96</v>
+        <v>3977.95</v>
       </c>
       <c r="J204" s="38" t="str">
         <f aca="true">IF($B204="","",IF($F204&lt;&gt;"","PAID",IF($C204&lt;TODAY(),"PAST DUE",IF($C204&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7953,7 +7953,7 @@
       </c>
       <c r="I205" s="37" t="n">
         <f aca="false">IF($B205="","",$I$202+SUM($H$204:$H205))</f>
-        <v>3309.46</v>
+        <v>3814.45</v>
       </c>
       <c r="J205" s="38" t="str">
         <f aca="true">IF($B205="","",IF($F205&lt;&gt;"","PAID",IF($C205&lt;TODAY(),"PAST DUE",IF($C205&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7988,7 +7988,7 @@
       </c>
       <c r="I206" s="37" t="n">
         <f aca="false">IF($B206="","",$I$202+SUM($H$204:$H206))</f>
-        <v>3306.47</v>
+        <v>3811.46</v>
       </c>
       <c r="J206" s="38" t="str">
         <f aca="true">IF($B206="","",IF($F206&lt;&gt;"","PAID",IF($C206&lt;TODAY(),"PAST DUE",IF($C206&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -8023,7 +8023,7 @@
       </c>
       <c r="I207" s="37" t="n">
         <f aca="false">IF($B207="","",$I$202+SUM($H$204:$H207))</f>
-        <v>3396.47</v>
+        <v>3901.46</v>
       </c>
       <c r="J207" s="38" t="str">
         <f aca="true">IF($B207="","",IF($F207&lt;&gt;"","PAID",IF($C207&lt;TODAY(),"PAST DUE",IF($C207&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -8058,7 +8058,7 @@
       </c>
       <c r="I208" s="37" t="n">
         <f aca="false">IF($B208="","",$I$202+SUM($H$204:$H208))</f>
-        <v>3046.47</v>
+        <v>3551.46</v>
       </c>
       <c r="J208" s="38" t="str">
         <f aca="true">IF($B208="","",IF($F208&lt;&gt;"","PAID",IF($C208&lt;TODAY(),"PAST DUE",IF($C208&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -8415,7 +8415,7 @@
       </c>
       <c r="I221" s="44" t="n">
         <f aca="false">$I$202+SUM($H$204:$H$220)</f>
-        <v>3046.47</v>
+        <v>3551.46</v>
       </c>
       <c r="J221" s="45" t="str">
         <f aca="false">IF($I$221&lt;0,"SHORTFALL",IF($I$221&lt;$E$7,"TIGHT","OK"))</f>
@@ -8441,7 +8441,7 @@
       <c r="H223" s="30"/>
       <c r="I223" s="32" t="n">
         <f aca="false">$I$221</f>
-        <v>3046.47</v>
+        <v>3551.46</v>
       </c>
       <c r="J223" s="30"/>
       <c r="K223" s="26" t="str">
@@ -8506,7 +8506,7 @@
       </c>
       <c r="I225" s="37" t="n">
         <f aca="false">IF($B225="","",$I$223+SUM($H$225:$H225))</f>
-        <v>3836.47</v>
+        <v>4341.46</v>
       </c>
       <c r="J225" s="38" t="str">
         <f aca="true">IF($B225="","",IF($F225&lt;&gt;"","PAID",IF($C225&lt;TODAY(),"PAST DUE",IF($C225&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -8541,7 +8541,7 @@
       </c>
       <c r="I226" s="37" t="n">
         <f aca="false">IF($B226="","",$I$223+SUM($H$225:$H226))</f>
-        <v>3665.37</v>
+        <v>4170.36</v>
       </c>
       <c r="J226" s="38" t="str">
         <f aca="true">IF($B226="","",IF($F226&lt;&gt;"","PAID",IF($C226&lt;TODAY(),"PAST DUE",IF($C226&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -8576,7 +8576,7 @@
       </c>
       <c r="I227" s="37" t="n">
         <f aca="false">IF($B227="","",$I$223+SUM($H$225:$H227))</f>
-        <v>3620.37</v>
+        <v>4125.36</v>
       </c>
       <c r="J227" s="38" t="str">
         <f aca="true">IF($B227="","",IF($F227&lt;&gt;"","PAID",IF($C227&lt;TODAY(),"PAST DUE",IF($C227&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -8611,7 +8611,7 @@
       </c>
       <c r="I228" s="37" t="n">
         <f aca="false">IF($B228="","",$I$223+SUM($H$225:$H228))</f>
-        <v>3603.38</v>
+        <v>4108.37</v>
       </c>
       <c r="J228" s="38" t="str">
         <f aca="true">IF($B228="","",IF($F228&lt;&gt;"","PAID",IF($C228&lt;TODAY(),"PAST DUE",IF($C228&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -8646,7 +8646,7 @@
       </c>
       <c r="I229" s="37" t="n">
         <f aca="false">IF($B229="","",$I$223+SUM($H$225:$H229))</f>
-        <v>3693.38</v>
+        <v>4198.37</v>
       </c>
       <c r="J229" s="38" t="str">
         <f aca="true">IF($B229="","",IF($F229&lt;&gt;"","PAID",IF($C229&lt;TODAY(),"PAST DUE",IF($C229&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9003,7 +9003,7 @@
       </c>
       <c r="I242" s="44" t="n">
         <f aca="false">$I$223+SUM($H$225:$H$241)</f>
-        <v>3693.38</v>
+        <v>4198.37</v>
       </c>
       <c r="J242" s="45" t="str">
         <f aca="false">IF($I$242&lt;0,"SHORTFALL",IF($I$242&lt;$E$7,"TIGHT","OK"))</f>
@@ -9029,7 +9029,7 @@
       <c r="H244" s="30"/>
       <c r="I244" s="32" t="n">
         <f aca="false">$I$242</f>
-        <v>3693.38</v>
+        <v>4198.37</v>
       </c>
       <c r="J244" s="30"/>
       <c r="K244" s="26" t="str">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="I246" s="37" t="n">
         <f aca="false">IF($B246="","",$I$244+SUM($H$246:$H246))</f>
-        <v>4483.38</v>
+        <v>4988.37</v>
       </c>
       <c r="J246" s="38" t="str">
         <f aca="true">IF($B246="","",IF($F246&lt;&gt;"","PAID",IF($C246&lt;TODAY(),"PAST DUE",IF($C246&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9129,7 +9129,7 @@
       </c>
       <c r="I247" s="37" t="n">
         <f aca="false">IF($B247="","",$I$244+SUM($H$246:$H247))</f>
-        <v>4469.68</v>
+        <v>4974.67</v>
       </c>
       <c r="J247" s="38" t="str">
         <f aca="true">IF($B247="","",IF($F247&lt;&gt;"","PAID",IF($C247&lt;TODAY(),"PAST DUE",IF($C247&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9164,7 +9164,7 @@
       </c>
       <c r="I248" s="37" t="n">
         <f aca="false">IF($B248="","",$I$244+SUM($H$246:$H248))</f>
-        <v>4425.81</v>
+        <v>4930.8</v>
       </c>
       <c r="J248" s="38" t="str">
         <f aca="true">IF($B248="","",IF($F248&lt;&gt;"","PAID",IF($C248&lt;TODAY(),"PAST DUE",IF($C248&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9199,7 +9199,7 @@
       </c>
       <c r="I249" s="37" t="n">
         <f aca="false">IF($B249="","",$I$244+SUM($H$246:$H249))</f>
-        <v>4515.81</v>
+        <v>5020.8</v>
       </c>
       <c r="J249" s="38" t="str">
         <f aca="true">IF($B249="","",IF($F249&lt;&gt;"","PAID",IF($C249&lt;TODAY(),"PAST DUE",IF($C249&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9591,7 +9591,7 @@
       </c>
       <c r="I263" s="44" t="n">
         <f aca="false">$I$244+SUM($H$246:$H$262)</f>
-        <v>4515.81</v>
+        <v>5020.8</v>
       </c>
       <c r="J263" s="45" t="str">
         <f aca="false">IF($I$263&lt;0,"SHORTFALL",IF($I$263&lt;$E$7,"TIGHT","OK"))</f>
@@ -9617,7 +9617,7 @@
       <c r="H265" s="30"/>
       <c r="I265" s="32" t="n">
         <f aca="false">$I$263</f>
-        <v>4515.81</v>
+        <v>5020.8</v>
       </c>
       <c r="J265" s="30"/>
       <c r="K265" s="26" t="str">
@@ -9682,7 +9682,7 @@
       </c>
       <c r="I267" s="37" t="n">
         <f aca="false">IF($B267="","",$I$265+SUM($H$267:$H267))</f>
-        <v>5305.81</v>
+        <v>5810.8</v>
       </c>
       <c r="J267" s="38" t="str">
         <f aca="true">IF($B267="","",IF($F267&lt;&gt;"","PAID",IF($C267&lt;TODAY(),"PAST DUE",IF($C267&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9717,7 +9717,7 @@
       </c>
       <c r="I268" s="37" t="n">
         <f aca="false">IF($B268="","",$I$265+SUM($H$267:$H268))</f>
-        <v>4955.81</v>
+        <v>5460.8</v>
       </c>
       <c r="J268" s="38" t="str">
         <f aca="true">IF($B268="","",IF($F268&lt;&gt;"","PAID",IF($C268&lt;TODAY(),"PAST DUE",IF($C268&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9752,7 +9752,7 @@
       </c>
       <c r="I269" s="37" t="n">
         <f aca="false">IF($B269="","",$I$265+SUM($H$267:$H269))</f>
-        <v>4805.81</v>
+        <v>5310.8</v>
       </c>
       <c r="J269" s="38" t="str">
         <f aca="true">IF($B269="","",IF($F269&lt;&gt;"","PAID",IF($C269&lt;TODAY(),"PAST DUE",IF($C269&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9787,7 +9787,7 @@
       </c>
       <c r="I270" s="37" t="n">
         <f aca="false">IF($B270="","",$I$265+SUM($H$267:$H270))</f>
-        <v>4662.44</v>
+        <v>5167.43</v>
       </c>
       <c r="J270" s="38" t="str">
         <f aca="true">IF($B270="","",IF($F270&lt;&gt;"","PAID",IF($C270&lt;TODAY(),"PAST DUE",IF($C270&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9822,7 +9822,7 @@
       </c>
       <c r="I271" s="37" t="n">
         <f aca="false">IF($B271="","",$I$265+SUM($H$267:$H271))</f>
-        <v>4752.44</v>
+        <v>5257.43</v>
       </c>
       <c r="J271" s="38" t="str">
         <f aca="true">IF($B271="","",IF($F271&lt;&gt;"","PAID",IF($C271&lt;TODAY(),"PAST DUE",IF($C271&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9857,7 +9857,7 @@
       </c>
       <c r="I272" s="37" t="n">
         <f aca="false">IF($B272="","",$I$265+SUM($H$267:$H272))</f>
-        <v>4731.34</v>
+        <v>5236.33</v>
       </c>
       <c r="J272" s="38" t="str">
         <f aca="true">IF($B272="","",IF($F272&lt;&gt;"","PAID",IF($C272&lt;TODAY(),"PAST DUE",IF($C272&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9892,7 +9892,7 @@
       </c>
       <c r="I273" s="37" t="n">
         <f aca="false">IF($B273="","",$I$265+SUM($H$267:$H273))</f>
-        <v>4711.34</v>
+        <v>5216.33</v>
       </c>
       <c r="J273" s="38" t="str">
         <f aca="true">IF($B273="","",IF($F273&lt;&gt;"","PAID",IF($C273&lt;TODAY(),"PAST DUE",IF($C273&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9927,7 +9927,7 @@
       </c>
       <c r="I274" s="37" t="n">
         <f aca="false">IF($B274="","",$I$265+SUM($H$267:$H274))</f>
-        <v>4701.34</v>
+        <v>5206.33</v>
       </c>
       <c r="J274" s="38" t="str">
         <f aca="true">IF($B274="","",IF($F274&lt;&gt;"","PAID",IF($C274&lt;TODAY(),"PAST DUE",IF($C274&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -10179,7 +10179,7 @@
       </c>
       <c r="I284" s="44" t="n">
         <f aca="false">$I$265+SUM($H$267:$H$283)</f>
-        <v>4701.34</v>
+        <v>5206.33</v>
       </c>
       <c r="J284" s="45" t="str">
         <f aca="false">IF($I$284&lt;0,"SHORTFALL",IF($I$284&lt;$E$7,"TIGHT","OK"))</f>
@@ -10260,7 +10260,7 @@
       <c r="D4" s="46"/>
       <c r="E4" s="47" t="n">
         <f aca="false">MIN($I$13:$I$25)</f>
-        <v>-510.31</v>
+        <v>-5.31999999999999</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10312,7 +10312,7 @@
       <c r="D8" s="46"/>
       <c r="E8" s="49" t="n">
         <f aca="false">SUM($F$13:$F$25)+SUM($G$13:$G$25)</f>
-        <v>6019.83</v>
+        <v>5514.84</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10323,7 +10323,7 @@
       <c r="D9" s="46"/>
       <c r="E9" s="47" t="n">
         <f aca="false">SUM($H$13:$H$25)</f>
-        <v>4630.17</v>
+        <v>5135.16</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10334,7 +10334,7 @@
       <c r="D10" s="46"/>
       <c r="E10" s="47" t="n">
         <f aca="false">$I$25</f>
-        <v>4701.34</v>
+        <v>5206.33</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10387,7 +10387,7 @@
       </c>
       <c r="F13" s="52" t="n">
         <f aca="false">SUMIF('Cash Flow'!$D$15:$D$24,"Expense",'Cash Flow'!$G$15:$G$24)</f>
-        <v>671.48</v>
+        <v>166.49</v>
       </c>
       <c r="G13" s="52" t="n">
         <f aca="false">SUMIF('Cash Flow'!$D$26:$D$31,"Expense",'Cash Flow'!$G$26:$G$31)</f>
@@ -10395,11 +10395,11 @@
       </c>
       <c r="H13" s="53" t="n">
         <f aca="false">$E13-$F13-$G13</f>
-        <v>-581.48</v>
+        <v>-76.49</v>
       </c>
       <c r="I13" s="53" t="n">
         <f aca="false">'Cash Flow'!$I$32</f>
-        <v>-510.31</v>
+        <v>-5.31999999999999</v>
       </c>
       <c r="J13" s="54" t="str">
         <f aca="false">IF($I13&lt;0,"SHORTFALL",IF($I13&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10420,7 +10420,7 @@
       </c>
       <c r="D14" s="56" t="n">
         <f aca="false">'Cash Flow'!$I$34</f>
-        <v>-510.31</v>
+        <v>-5.31999999999999</v>
       </c>
       <c r="E14" s="57" t="n">
         <f aca="false">SUMIF('Cash Flow'!$D$36:$D$45,"Income",'Cash Flow'!$G$36:$G$45)</f>
@@ -10440,15 +10440,15 @@
       </c>
       <c r="I14" s="58" t="n">
         <f aca="false">'Cash Flow'!$I$53</f>
-        <v>-213.4</v>
+        <v>291.59</v>
       </c>
       <c r="J14" s="59" t="str">
         <f aca="false">IF($I14&lt;0,"SHORTFALL",IF($I14&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
-        <v>SHORTFALL</v>
+        <v>OK</v>
       </c>
       <c r="K14" s="27" t="n">
         <f aca="false">IF($I14&lt;0,$B14,999)</f>
-        <v>2</v>
+        <v>999</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10461,7 +10461,7 @@
       </c>
       <c r="D15" s="51" t="n">
         <f aca="false">'Cash Flow'!$I$55</f>
-        <v>-213.4</v>
+        <v>291.59</v>
       </c>
       <c r="E15" s="52" t="n">
         <f aca="false">SUMIF('Cash Flow'!$D$57:$D$66,"Income",'Cash Flow'!$G$57:$G$66)</f>
@@ -10481,7 +10481,7 @@
       </c>
       <c r="I15" s="53" t="n">
         <f aca="false">'Cash Flow'!$I$74</f>
-        <v>609.03</v>
+        <v>1114.02</v>
       </c>
       <c r="J15" s="54" t="str">
         <f aca="false">IF($I15&lt;0,"SHORTFALL",IF($I15&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10502,7 +10502,7 @@
       </c>
       <c r="D16" s="56" t="n">
         <f aca="false">'Cash Flow'!$I$76</f>
-        <v>609.03</v>
+        <v>1114.02</v>
       </c>
       <c r="E16" s="57" t="n">
         <f aca="false">SUMIF('Cash Flow'!$D$78:$D$87,"Income",'Cash Flow'!$G$78:$G$87)</f>
@@ -10522,7 +10522,7 @@
       </c>
       <c r="I16" s="58" t="n">
         <f aca="false">'Cash Flow'!$I$95</f>
-        <v>845.66</v>
+        <v>1350.65</v>
       </c>
       <c r="J16" s="59" t="str">
         <f aca="false">IF($I16&lt;0,"SHORTFALL",IF($I16&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10543,7 +10543,7 @@
       </c>
       <c r="D17" s="51" t="n">
         <f aca="false">'Cash Flow'!$I$97</f>
-        <v>845.66</v>
+        <v>1350.65</v>
       </c>
       <c r="E17" s="52" t="n">
         <f aca="false">SUMIF('Cash Flow'!$D$99:$D$108,"Income",'Cash Flow'!$G$99:$G$108)</f>
@@ -10563,7 +10563,7 @@
       </c>
       <c r="I17" s="53" t="n">
         <f aca="false">'Cash Flow'!$I$116</f>
-        <v>1006.07</v>
+        <v>1511.06</v>
       </c>
       <c r="J17" s="54" t="str">
         <f aca="false">IF($I17&lt;0,"SHORTFALL",IF($I17&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10584,7 +10584,7 @@
       </c>
       <c r="D18" s="56" t="n">
         <f aca="false">'Cash Flow'!$I$118</f>
-        <v>1006.07</v>
+        <v>1511.06</v>
       </c>
       <c r="E18" s="57" t="n">
         <f aca="false">SUMIF('Cash Flow'!$D$120:$D$129,"Income",'Cash Flow'!$G$120:$G$129)</f>
@@ -10604,7 +10604,7 @@
       </c>
       <c r="I18" s="58" t="n">
         <f aca="false">'Cash Flow'!$I$137</f>
-        <v>1316.98</v>
+        <v>1821.97</v>
       </c>
       <c r="J18" s="59" t="str">
         <f aca="false">IF($I18&lt;0,"SHORTFALL",IF($I18&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10625,7 +10625,7 @@
       </c>
       <c r="D19" s="51" t="n">
         <f aca="false">'Cash Flow'!$I$139</f>
-        <v>1316.98</v>
+        <v>1821.97</v>
       </c>
       <c r="E19" s="52" t="n">
         <f aca="false">SUMIF('Cash Flow'!$D$141:$D$150,"Income",'Cash Flow'!$G$141:$G$150)</f>
@@ -10645,7 +10645,7 @@
       </c>
       <c r="I19" s="53" t="n">
         <f aca="false">'Cash Flow'!$I$158</f>
-        <v>2179.99</v>
+        <v>2684.98</v>
       </c>
       <c r="J19" s="54" t="str">
         <f aca="false">IF($I19&lt;0,"SHORTFALL",IF($I19&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10666,7 +10666,7 @@
       </c>
       <c r="D20" s="56" t="n">
         <f aca="false">'Cash Flow'!$I$160</f>
-        <v>2179.99</v>
+        <v>2684.98</v>
       </c>
       <c r="E20" s="57" t="n">
         <f aca="false">SUMIF('Cash Flow'!$D$162:$D$171,"Income",'Cash Flow'!$G$162:$G$171)</f>
@@ -10686,7 +10686,7 @@
       </c>
       <c r="I20" s="58" t="n">
         <f aca="false">'Cash Flow'!$I$179</f>
-        <v>2359.05</v>
+        <v>2864.04</v>
       </c>
       <c r="J20" s="59" t="str">
         <f aca="false">IF($I20&lt;0,"SHORTFALL",IF($I20&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10707,7 +10707,7 @@
       </c>
       <c r="D21" s="51" t="n">
         <f aca="false">'Cash Flow'!$I$181</f>
-        <v>2359.05</v>
+        <v>2864.04</v>
       </c>
       <c r="E21" s="52" t="n">
         <f aca="false">SUMIF('Cash Flow'!$D$183:$D$192,"Income",'Cash Flow'!$G$183:$G$192)</f>
@@ -10727,7 +10727,7 @@
       </c>
       <c r="I21" s="53" t="n">
         <f aca="false">'Cash Flow'!$I$200</f>
-        <v>2682.96</v>
+        <v>3187.95</v>
       </c>
       <c r="J21" s="54" t="str">
         <f aca="false">IF($I21&lt;0,"SHORTFALL",IF($I21&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10748,7 +10748,7 @@
       </c>
       <c r="D22" s="56" t="n">
         <f aca="false">'Cash Flow'!$I$202</f>
-        <v>2682.96</v>
+        <v>3187.95</v>
       </c>
       <c r="E22" s="57" t="n">
         <f aca="false">SUMIF('Cash Flow'!$D$204:$D$213,"Income",'Cash Flow'!$G$204:$G$213)</f>
@@ -10768,7 +10768,7 @@
       </c>
       <c r="I22" s="58" t="n">
         <f aca="false">'Cash Flow'!$I$221</f>
-        <v>3046.47</v>
+        <v>3551.46</v>
       </c>
       <c r="J22" s="59" t="str">
         <f aca="false">IF($I22&lt;0,"SHORTFALL",IF($I22&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10789,7 +10789,7 @@
       </c>
       <c r="D23" s="51" t="n">
         <f aca="false">'Cash Flow'!$I$223</f>
-        <v>3046.47</v>
+        <v>3551.46</v>
       </c>
       <c r="E23" s="52" t="n">
         <f aca="false">SUMIF('Cash Flow'!$D$225:$D$234,"Income",'Cash Flow'!$G$225:$G$234)</f>
@@ -10809,7 +10809,7 @@
       </c>
       <c r="I23" s="53" t="n">
         <f aca="false">'Cash Flow'!$I$242</f>
-        <v>3693.38</v>
+        <v>4198.37</v>
       </c>
       <c r="J23" s="54" t="str">
         <f aca="false">IF($I23&lt;0,"SHORTFALL",IF($I23&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10830,7 +10830,7 @@
       </c>
       <c r="D24" s="56" t="n">
         <f aca="false">'Cash Flow'!$I$244</f>
-        <v>3693.38</v>
+        <v>4198.37</v>
       </c>
       <c r="E24" s="57" t="n">
         <f aca="false">SUMIF('Cash Flow'!$D$246:$D$255,"Income",'Cash Flow'!$G$246:$G$255)</f>
@@ -10850,7 +10850,7 @@
       </c>
       <c r="I24" s="58" t="n">
         <f aca="false">'Cash Flow'!$I$263</f>
-        <v>4515.81</v>
+        <v>5020.8</v>
       </c>
       <c r="J24" s="59" t="str">
         <f aca="false">IF($I24&lt;0,"SHORTFALL",IF($I24&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10871,7 +10871,7 @@
       </c>
       <c r="D25" s="51" t="n">
         <f aca="false">'Cash Flow'!$I$265</f>
-        <v>4515.81</v>
+        <v>5020.8</v>
       </c>
       <c r="E25" s="52" t="n">
         <f aca="false">SUMIF('Cash Flow'!$D$267:$D$276,"Income",'Cash Flow'!$G$267:$G$276)</f>
@@ -10891,7 +10891,7 @@
       </c>
       <c r="I25" s="53" t="n">
         <f aca="false">'Cash Flow'!$I$284</f>
-        <v>4701.34</v>
+        <v>5206.33</v>
       </c>
       <c r="J25" s="54" t="str">
         <f aca="false">IF($I25&lt;0,"SHORTFALL",IF($I25&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10919,7 +10919,7 @@
       </c>
       <c r="F26" s="43" t="n">
         <f aca="false">SUM($F$13:$F$25)</f>
-        <v>6019.83</v>
+        <v>5514.84</v>
       </c>
       <c r="G26" s="43" t="n">
         <f aca="false">SUM($G$13:$G$25)</f>
@@ -10927,11 +10927,11 @@
       </c>
       <c r="H26" s="61" t="n">
         <f aca="false">SUM($H$13:$H$25)</f>
-        <v>4630.17</v>
+        <v>5135.16</v>
       </c>
       <c r="I26" s="61" t="n">
         <f aca="false">$I$25</f>
-        <v>4701.34</v>
+        <v>5206.33</v>
       </c>
       <c r="J26" s="42"/>
     </row>
@@ -11091,7 +11091,7 @@
       </c>
       <c r="K4" s="66" t="n">
         <f aca="false">IF($H4=1,$I4*1000+COUNTIFS($I$4:$I$483,$I4,$J$4:$J$483,"&lt;"&amp;$J4)+1,"")</f>
-        <v>1004</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14591,11 +14591,11 @@
       </c>
       <c r="F84" s="68" t="n">
         <f aca="false">IF($C84="","",IF(Recurring!$E$10="Weekly",Recurring!$F$10+7*0,IF(Recurring!$E$10="Every 2 Weeks",Recurring!$F$10+14*0,IF(Recurring!$E$10="Monthly",EDATE(Recurring!$F$10,0),IF(Recurring!$E$10="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+0),2)=1,EOMONTH(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+0)/2)),DATE(YEAR(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+0)/2))),MONTH(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+0)/2))),15)),IF(Recurring!$E$10="One Time",IF(1=1,Recurring!$F$10,""),""))))))</f>
-        <v>46241</v>
+        <v>46272</v>
       </c>
       <c r="G84" s="68" t="n">
         <f aca="false">IF($F84="","",IF(Recurring!$G$10="Move Before",IF(WEEKDAY($F84,2)=6,$F84-1,IF(WEEKDAY($F84,2)=7,$F84-2,$F84)),IF(Recurring!$G$10="Move After",IF(WEEKDAY($F84,2)=6,$F84+2,IF(WEEKDAY($F84,2)=7,$F84+1,$F84)),$F84)))</f>
-        <v>46241</v>
+        <v>46272</v>
       </c>
       <c r="H84" s="69" t="n">
         <f aca="false">IF($G84="",0,IF(AND($G84&gt;='Cash Flow'!$E$6,$G84&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -14603,15 +14603,15 @@
       </c>
       <c r="I84" s="69" t="n">
         <f aca="false">IF($H84=1,INT(($G84-'Cash Flow'!$E$6)/7)+1,"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J84" s="66" t="n">
         <f aca="false">IF($H84=1,$G84*10000+ROW(),"")</f>
-        <v>462410084</v>
+        <v>462720084</v>
       </c>
       <c r="K84" s="66" t="n">
         <f aca="false">IF($H84=1,$I84*1000+COUNTIFS($I$4:$I$483,$I84,$J$4:$J$483,"&lt;"&amp;$J84)+1,"")</f>
-        <v>1001</v>
+        <v>5005</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14635,11 +14635,11 @@
       </c>
       <c r="F85" s="68" t="n">
         <f aca="false">IF($C85="","",IF(Recurring!$E$10="Weekly",Recurring!$F$10+7*1,IF(Recurring!$E$10="Every 2 Weeks",Recurring!$F$10+14*1,IF(Recurring!$E$10="Monthly",EDATE(Recurring!$F$10,1),IF(Recurring!$E$10="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+1),2)=1,EOMONTH(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+1)/2)),DATE(YEAR(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+1)/2))),MONTH(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+1)/2))),15)),IF(Recurring!$E$10="One Time",IF(2=1,Recurring!$F$10,""),""))))))</f>
-        <v>46272</v>
+        <v>46302</v>
       </c>
       <c r="G85" s="68" t="n">
         <f aca="false">IF($F85="","",IF(Recurring!$G$10="Move Before",IF(WEEKDAY($F85,2)=6,$F85-1,IF(WEEKDAY($F85,2)=7,$F85-2,$F85)),IF(Recurring!$G$10="Move After",IF(WEEKDAY($F85,2)=6,$F85+2,IF(WEEKDAY($F85,2)=7,$F85+1,$F85)),$F85)))</f>
-        <v>46272</v>
+        <v>46302</v>
       </c>
       <c r="H85" s="69" t="n">
         <f aca="false">IF($G85="",0,IF(AND($G85&gt;='Cash Flow'!$E$6,$G85&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -14647,15 +14647,15 @@
       </c>
       <c r="I85" s="69" t="n">
         <f aca="false">IF($H85=1,INT(($G85-'Cash Flow'!$E$6)/7)+1,"")</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J85" s="66" t="n">
         <f aca="false">IF($H85=1,$G85*10000+ROW(),"")</f>
-        <v>462720085</v>
+        <v>463020085</v>
       </c>
       <c r="K85" s="66" t="n">
         <f aca="false">IF($H85=1,$I85*1000+COUNTIFS($I$4:$I$483,$I85,$J$4:$J$483,"&lt;"&amp;$J85)+1,"")</f>
-        <v>5005</v>
+        <v>9006</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14679,27 +14679,27 @@
       </c>
       <c r="F86" s="68" t="n">
         <f aca="false">IF($C86="","",IF(Recurring!$E$10="Weekly",Recurring!$F$10+7*2,IF(Recurring!$E$10="Every 2 Weeks",Recurring!$F$10+14*2,IF(Recurring!$E$10="Monthly",EDATE(Recurring!$F$10,2),IF(Recurring!$E$10="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+2),2)=1,EOMONTH(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+2)/2)),DATE(YEAR(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+2)/2))),MONTH(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+2)/2))),15)),IF(Recurring!$E$10="One Time",IF(3=1,Recurring!$F$10,""),""))))))</f>
-        <v>46302</v>
+        <v>46333</v>
       </c>
       <c r="G86" s="68" t="n">
         <f aca="false">IF($F86="","",IF(Recurring!$G$10="Move Before",IF(WEEKDAY($F86,2)=6,$F86-1,IF(WEEKDAY($F86,2)=7,$F86-2,$F86)),IF(Recurring!$G$10="Move After",IF(WEEKDAY($F86,2)=6,$F86+2,IF(WEEKDAY($F86,2)=7,$F86+1,$F86)),$F86)))</f>
-        <v>46302</v>
+        <v>46333</v>
       </c>
       <c r="H86" s="69" t="n">
         <f aca="false">IF($G86="",0,IF(AND($G86&gt;='Cash Flow'!$E$6,$G86&lt;'Cash Flow'!$E$6+91),1,0))</f>
-        <v>1</v>
-      </c>
-      <c r="I86" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="69" t="str">
         <f aca="false">IF($H86=1,INT(($G86-'Cash Flow'!$E$6)/7)+1,"")</f>
-        <v>9</v>
-      </c>
-      <c r="J86" s="66" t="n">
+        <v/>
+      </c>
+      <c r="J86" s="66" t="str">
         <f aca="false">IF($H86=1,$G86*10000+ROW(),"")</f>
-        <v>463020086</v>
-      </c>
-      <c r="K86" s="66" t="n">
+        <v/>
+      </c>
+      <c r="K86" s="66" t="str">
         <f aca="false">IF($H86=1,$I86*1000+COUNTIFS($I$4:$I$483,$I86,$J$4:$J$483,"&lt;"&amp;$J86)+1,"")</f>
-        <v>9006</v>
+        <v/>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14723,11 +14723,11 @@
       </c>
       <c r="F87" s="68" t="n">
         <f aca="false">IF($C87="","",IF(Recurring!$E$10="Weekly",Recurring!$F$10+7*3,IF(Recurring!$E$10="Every 2 Weeks",Recurring!$F$10+14*3,IF(Recurring!$E$10="Monthly",EDATE(Recurring!$F$10,3),IF(Recurring!$E$10="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+3),2)=1,EOMONTH(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+3)/2)),DATE(YEAR(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+3)/2))),MONTH(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+3)/2))),15)),IF(Recurring!$E$10="One Time",IF(4=1,Recurring!$F$10,""),""))))))</f>
-        <v>46333</v>
+        <v>46363</v>
       </c>
       <c r="G87" s="68" t="n">
         <f aca="false">IF($F87="","",IF(Recurring!$G$10="Move Before",IF(WEEKDAY($F87,2)=6,$F87-1,IF(WEEKDAY($F87,2)=7,$F87-2,$F87)),IF(Recurring!$G$10="Move After",IF(WEEKDAY($F87,2)=6,$F87+2,IF(WEEKDAY($F87,2)=7,$F87+1,$F87)),$F87)))</f>
-        <v>46333</v>
+        <v>46363</v>
       </c>
       <c r="H87" s="69" t="n">
         <f aca="false">IF($G87="",0,IF(AND($G87&gt;='Cash Flow'!$E$6,$G87&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -14767,11 +14767,11 @@
       </c>
       <c r="F88" s="68" t="n">
         <f aca="false">IF($C88="","",IF(Recurring!$E$10="Weekly",Recurring!$F$10+7*4,IF(Recurring!$E$10="Every 2 Weeks",Recurring!$F$10+14*4,IF(Recurring!$E$10="Monthly",EDATE(Recurring!$F$10,4),IF(Recurring!$E$10="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+4),2)=1,EOMONTH(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+4)/2)),DATE(YEAR(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+4)/2))),MONTH(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+4)/2))),15)),IF(Recurring!$E$10="One Time",IF(5=1,Recurring!$F$10,""),""))))))</f>
-        <v>46363</v>
+        <v>46394</v>
       </c>
       <c r="G88" s="68" t="n">
         <f aca="false">IF($F88="","",IF(Recurring!$G$10="Move Before",IF(WEEKDAY($F88,2)=6,$F88-1,IF(WEEKDAY($F88,2)=7,$F88-2,$F88)),IF(Recurring!$G$10="Move After",IF(WEEKDAY($F88,2)=6,$F88+2,IF(WEEKDAY($F88,2)=7,$F88+1,$F88)),$F88)))</f>
-        <v>46363</v>
+        <v>46394</v>
       </c>
       <c r="H88" s="69" t="n">
         <f aca="false">IF($G88="",0,IF(AND($G88&gt;='Cash Flow'!$E$6,$G88&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -14811,11 +14811,11 @@
       </c>
       <c r="F89" s="68" t="n">
         <f aca="false">IF($C89="","",IF(Recurring!$E$10="Weekly",Recurring!$F$10+7*5,IF(Recurring!$E$10="Every 2 Weeks",Recurring!$F$10+14*5,IF(Recurring!$E$10="Monthly",EDATE(Recurring!$F$10,5),IF(Recurring!$E$10="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+5),2)=1,EOMONTH(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+5)/2)),DATE(YEAR(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+5)/2))),MONTH(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+5)/2))),15)),IF(Recurring!$E$10="One Time",IF(6=1,Recurring!$F$10,""),""))))))</f>
-        <v>46394</v>
+        <v>46425</v>
       </c>
       <c r="G89" s="68" t="n">
         <f aca="false">IF($F89="","",IF(Recurring!$G$10="Move Before",IF(WEEKDAY($F89,2)=6,$F89-1,IF(WEEKDAY($F89,2)=7,$F89-2,$F89)),IF(Recurring!$G$10="Move After",IF(WEEKDAY($F89,2)=6,$F89+2,IF(WEEKDAY($F89,2)=7,$F89+1,$F89)),$F89)))</f>
-        <v>46394</v>
+        <v>46425</v>
       </c>
       <c r="H89" s="69" t="n">
         <f aca="false">IF($G89="",0,IF(AND($G89&gt;='Cash Flow'!$E$6,$G89&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -14855,11 +14855,11 @@
       </c>
       <c r="F90" s="68" t="n">
         <f aca="false">IF($C90="","",IF(Recurring!$E$10="Weekly",Recurring!$F$10+7*6,IF(Recurring!$E$10="Every 2 Weeks",Recurring!$F$10+14*6,IF(Recurring!$E$10="Monthly",EDATE(Recurring!$F$10,6),IF(Recurring!$E$10="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+6),2)=1,EOMONTH(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+6)/2)),DATE(YEAR(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+6)/2))),MONTH(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+6)/2))),15)),IF(Recurring!$E$10="One Time",IF(7=1,Recurring!$F$10,""),""))))))</f>
-        <v>46425</v>
+        <v>46453</v>
       </c>
       <c r="G90" s="68" t="n">
         <f aca="false">IF($F90="","",IF(Recurring!$G$10="Move Before",IF(WEEKDAY($F90,2)=6,$F90-1,IF(WEEKDAY($F90,2)=7,$F90-2,$F90)),IF(Recurring!$G$10="Move After",IF(WEEKDAY($F90,2)=6,$F90+2,IF(WEEKDAY($F90,2)=7,$F90+1,$F90)),$F90)))</f>
-        <v>46425</v>
+        <v>46453</v>
       </c>
       <c r="H90" s="69" t="n">
         <f aca="false">IF($G90="",0,IF(AND($G90&gt;='Cash Flow'!$E$6,$G90&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -14899,11 +14899,11 @@
       </c>
       <c r="F91" s="68" t="n">
         <f aca="false">IF($C91="","",IF(Recurring!$E$10="Weekly",Recurring!$F$10+7*7,IF(Recurring!$E$10="Every 2 Weeks",Recurring!$F$10+14*7,IF(Recurring!$E$10="Monthly",EDATE(Recurring!$F$10,7),IF(Recurring!$E$10="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+7),2)=1,EOMONTH(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+7)/2)),DATE(YEAR(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+7)/2))),MONTH(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+7)/2))),15)),IF(Recurring!$E$10="One Time",IF(8=1,Recurring!$F$10,""),""))))))</f>
-        <v>46453</v>
+        <v>46484</v>
       </c>
       <c r="G91" s="68" t="n">
         <f aca="false">IF($F91="","",IF(Recurring!$G$10="Move Before",IF(WEEKDAY($F91,2)=6,$F91-1,IF(WEEKDAY($F91,2)=7,$F91-2,$F91)),IF(Recurring!$G$10="Move After",IF(WEEKDAY($F91,2)=6,$F91+2,IF(WEEKDAY($F91,2)=7,$F91+1,$F91)),$F91)))</f>
-        <v>46453</v>
+        <v>46484</v>
       </c>
       <c r="H91" s="69" t="n">
         <f aca="false">IF($G91="",0,IF(AND($G91&gt;='Cash Flow'!$E$6,$G91&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -14943,11 +14943,11 @@
       </c>
       <c r="F92" s="68" t="n">
         <f aca="false">IF($C92="","",IF(Recurring!$E$10="Weekly",Recurring!$F$10+7*8,IF(Recurring!$E$10="Every 2 Weeks",Recurring!$F$10+14*8,IF(Recurring!$E$10="Monthly",EDATE(Recurring!$F$10,8),IF(Recurring!$E$10="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+8),2)=1,EOMONTH(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+8)/2)),DATE(YEAR(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+8)/2))),MONTH(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+8)/2))),15)),IF(Recurring!$E$10="One Time",IF(9=1,Recurring!$F$10,""),""))))))</f>
-        <v>46484</v>
+        <v>46514</v>
       </c>
       <c r="G92" s="68" t="n">
         <f aca="false">IF($F92="","",IF(Recurring!$G$10="Move Before",IF(WEEKDAY($F92,2)=6,$F92-1,IF(WEEKDAY($F92,2)=7,$F92-2,$F92)),IF(Recurring!$G$10="Move After",IF(WEEKDAY($F92,2)=6,$F92+2,IF(WEEKDAY($F92,2)=7,$F92+1,$F92)),$F92)))</f>
-        <v>46484</v>
+        <v>46514</v>
       </c>
       <c r="H92" s="69" t="n">
         <f aca="false">IF($G92="",0,IF(AND($G92&gt;='Cash Flow'!$E$6,$G92&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -14987,11 +14987,11 @@
       </c>
       <c r="F93" s="68" t="n">
         <f aca="false">IF($C93="","",IF(Recurring!$E$10="Weekly",Recurring!$F$10+7*9,IF(Recurring!$E$10="Every 2 Weeks",Recurring!$F$10+14*9,IF(Recurring!$E$10="Monthly",EDATE(Recurring!$F$10,9),IF(Recurring!$E$10="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+9),2)=1,EOMONTH(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+9)/2)),DATE(YEAR(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+9)/2))),MONTH(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+9)/2))),15)),IF(Recurring!$E$10="One Time",IF(10=1,Recurring!$F$10,""),""))))))</f>
-        <v>46514</v>
+        <v>46545</v>
       </c>
       <c r="G93" s="68" t="n">
         <f aca="false">IF($F93="","",IF(Recurring!$G$10="Move Before",IF(WEEKDAY($F93,2)=6,$F93-1,IF(WEEKDAY($F93,2)=7,$F93-2,$F93)),IF(Recurring!$G$10="Move After",IF(WEEKDAY($F93,2)=6,$F93+2,IF(WEEKDAY($F93,2)=7,$F93+1,$F93)),$F93)))</f>
-        <v>46514</v>
+        <v>46545</v>
       </c>
       <c r="H93" s="69" t="n">
         <f aca="false">IF($G93="",0,IF(AND($G93&gt;='Cash Flow'!$E$6,$G93&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15031,11 +15031,11 @@
       </c>
       <c r="F94" s="68" t="n">
         <f aca="false">IF($C94="","",IF(Recurring!$E$10="Weekly",Recurring!$F$10+7*10,IF(Recurring!$E$10="Every 2 Weeks",Recurring!$F$10+14*10,IF(Recurring!$E$10="Monthly",EDATE(Recurring!$F$10,10),IF(Recurring!$E$10="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+10),2)=1,EOMONTH(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+10)/2)),DATE(YEAR(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+10)/2))),MONTH(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+10)/2))),15)),IF(Recurring!$E$10="One Time",IF(11=1,Recurring!$F$10,""),""))))))</f>
-        <v>46545</v>
+        <v>46575</v>
       </c>
       <c r="G94" s="68" t="n">
         <f aca="false">IF($F94="","",IF(Recurring!$G$10="Move Before",IF(WEEKDAY($F94,2)=6,$F94-1,IF(WEEKDAY($F94,2)=7,$F94-2,$F94)),IF(Recurring!$G$10="Move After",IF(WEEKDAY($F94,2)=6,$F94+2,IF(WEEKDAY($F94,2)=7,$F94+1,$F94)),$F94)))</f>
-        <v>46545</v>
+        <v>46575</v>
       </c>
       <c r="H94" s="69" t="n">
         <f aca="false">IF($G94="",0,IF(AND($G94&gt;='Cash Flow'!$E$6,$G94&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15075,11 +15075,11 @@
       </c>
       <c r="F95" s="68" t="n">
         <f aca="false">IF($C95="","",IF(Recurring!$E$10="Weekly",Recurring!$F$10+7*11,IF(Recurring!$E$10="Every 2 Weeks",Recurring!$F$10+14*11,IF(Recurring!$E$10="Monthly",EDATE(Recurring!$F$10,11),IF(Recurring!$E$10="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+11),2)=1,EOMONTH(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+11)/2)),DATE(YEAR(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+11)/2))),MONTH(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+11)/2))),15)),IF(Recurring!$E$10="One Time",IF(12=1,Recurring!$F$10,""),""))))))</f>
-        <v>46575</v>
+        <v>46606</v>
       </c>
       <c r="G95" s="68" t="n">
         <f aca="false">IF($F95="","",IF(Recurring!$G$10="Move Before",IF(WEEKDAY($F95,2)=6,$F95-1,IF(WEEKDAY($F95,2)=7,$F95-2,$F95)),IF(Recurring!$G$10="Move After",IF(WEEKDAY($F95,2)=6,$F95+2,IF(WEEKDAY($F95,2)=7,$F95+1,$F95)),$F95)))</f>
-        <v>46575</v>
+        <v>46606</v>
       </c>
       <c r="H95" s="69" t="n">
         <f aca="false">IF($G95="",0,IF(AND($G95&gt;='Cash Flow'!$E$6,$G95&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15119,11 +15119,11 @@
       </c>
       <c r="F96" s="68" t="n">
         <f aca="false">IF($C96="","",IF(Recurring!$E$10="Weekly",Recurring!$F$10+7*12,IF(Recurring!$E$10="Every 2 Weeks",Recurring!$F$10+14*12,IF(Recurring!$E$10="Monthly",EDATE(Recurring!$F$10,12),IF(Recurring!$E$10="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+12),2)=1,EOMONTH(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+12)/2)),DATE(YEAR(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+12)/2))),MONTH(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+12)/2))),15)),IF(Recurring!$E$10="One Time",IF(13=1,Recurring!$F$10,""),""))))))</f>
-        <v>46606</v>
+        <v>46637</v>
       </c>
       <c r="G96" s="68" t="n">
         <f aca="false">IF($F96="","",IF(Recurring!$G$10="Move Before",IF(WEEKDAY($F96,2)=6,$F96-1,IF(WEEKDAY($F96,2)=7,$F96-2,$F96)),IF(Recurring!$G$10="Move After",IF(WEEKDAY($F96,2)=6,$F96+2,IF(WEEKDAY($F96,2)=7,$F96+1,$F96)),$F96)))</f>
-        <v>46606</v>
+        <v>46637</v>
       </c>
       <c r="H96" s="69" t="n">
         <f aca="false">IF($G96="",0,IF(AND($G96&gt;='Cash Flow'!$E$6,$G96&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15163,11 +15163,11 @@
       </c>
       <c r="F97" s="68" t="n">
         <f aca="false">IF($C97="","",IF(Recurring!$E$10="Weekly",Recurring!$F$10+7*13,IF(Recurring!$E$10="Every 2 Weeks",Recurring!$F$10+14*13,IF(Recurring!$E$10="Monthly",EDATE(Recurring!$F$10,13),IF(Recurring!$E$10="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+13),2)=1,EOMONTH(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+13)/2)),DATE(YEAR(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+13)/2))),MONTH(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+13)/2))),15)),IF(Recurring!$E$10="One Time",IF(14=1,Recurring!$F$10,""),""))))))</f>
-        <v>46637</v>
+        <v>46667</v>
       </c>
       <c r="G97" s="68" t="n">
         <f aca="false">IF($F97="","",IF(Recurring!$G$10="Move Before",IF(WEEKDAY($F97,2)=6,$F97-1,IF(WEEKDAY($F97,2)=7,$F97-2,$F97)),IF(Recurring!$G$10="Move After",IF(WEEKDAY($F97,2)=6,$F97+2,IF(WEEKDAY($F97,2)=7,$F97+1,$F97)),$F97)))</f>
-        <v>46637</v>
+        <v>46667</v>
       </c>
       <c r="H97" s="69" t="n">
         <f aca="false">IF($G97="",0,IF(AND($G97&gt;='Cash Flow'!$E$6,$G97&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15207,11 +15207,11 @@
       </c>
       <c r="F98" s="68" t="n">
         <f aca="false">IF($C98="","",IF(Recurring!$E$10="Weekly",Recurring!$F$10+7*14,IF(Recurring!$E$10="Every 2 Weeks",Recurring!$F$10+14*14,IF(Recurring!$E$10="Monthly",EDATE(Recurring!$F$10,14),IF(Recurring!$E$10="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+14),2)=1,EOMONTH(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+14)/2)),DATE(YEAR(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+14)/2))),MONTH(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+14)/2))),15)),IF(Recurring!$E$10="One Time",IF(15=1,Recurring!$F$10,""),""))))))</f>
-        <v>46667</v>
+        <v>46698</v>
       </c>
       <c r="G98" s="68" t="n">
         <f aca="false">IF($F98="","",IF(Recurring!$G$10="Move Before",IF(WEEKDAY($F98,2)=6,$F98-1,IF(WEEKDAY($F98,2)=7,$F98-2,$F98)),IF(Recurring!$G$10="Move After",IF(WEEKDAY($F98,2)=6,$F98+2,IF(WEEKDAY($F98,2)=7,$F98+1,$F98)),$F98)))</f>
-        <v>46667</v>
+        <v>46698</v>
       </c>
       <c r="H98" s="69" t="n">
         <f aca="false">IF($G98="",0,IF(AND($G98&gt;='Cash Flow'!$E$6,$G98&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15251,11 +15251,11 @@
       </c>
       <c r="F99" s="68" t="n">
         <f aca="false">IF($C99="","",IF(Recurring!$E$10="Weekly",Recurring!$F$10+7*15,IF(Recurring!$E$10="Every 2 Weeks",Recurring!$F$10+14*15,IF(Recurring!$E$10="Monthly",EDATE(Recurring!$F$10,15),IF(Recurring!$E$10="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+15),2)=1,EOMONTH(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+15)/2)),DATE(YEAR(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+15)/2))),MONTH(EDATE(Recurring!$F$10,INT((IF(DAY(Recurring!$F$10)&lt;=20,0,1)+15)/2))),15)),IF(Recurring!$E$10="One Time",IF(16=1,Recurring!$F$10,""),""))))))</f>
-        <v>46698</v>
+        <v>46728</v>
       </c>
       <c r="G99" s="68" t="n">
         <f aca="false">IF($F99="","",IF(Recurring!$G$10="Move Before",IF(WEEKDAY($F99,2)=6,$F99-1,IF(WEEKDAY($F99,2)=7,$F99-2,$F99)),IF(Recurring!$G$10="Move After",IF(WEEKDAY($F99,2)=6,$F99+2,IF(WEEKDAY($F99,2)=7,$F99+1,$F99)),$F99)))</f>
-        <v>46698</v>
+        <v>46728</v>
       </c>
       <c r="H99" s="69" t="n">
         <f aca="false">IF($G99="",0,IF(AND($G99&gt;='Cash Flow'!$E$6,$G99&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15295,11 +15295,11 @@
       </c>
       <c r="F100" s="68" t="n">
         <f aca="false">IF($C100="","",IF(Recurring!$E$11="Weekly",Recurring!$F$11+7*0,IF(Recurring!$E$11="Every 2 Weeks",Recurring!$F$11+14*0,IF(Recurring!$E$11="Monthly",EDATE(Recurring!$F$11,0),IF(Recurring!$E$11="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+0),2)=1,EOMONTH(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+0)/2)),DATE(YEAR(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+0)/2))),MONTH(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+0)/2))),15)),IF(Recurring!$E$11="One Time",IF(1=1,Recurring!$F$11,""),""))))))</f>
-        <v>46241</v>
+        <v>46272</v>
       </c>
       <c r="G100" s="68" t="n">
         <f aca="false">IF($F100="","",IF(Recurring!$G$11="Move Before",IF(WEEKDAY($F100,2)=6,$F100-1,IF(WEEKDAY($F100,2)=7,$F100-2,$F100)),IF(Recurring!$G$11="Move After",IF(WEEKDAY($F100,2)=6,$F100+2,IF(WEEKDAY($F100,2)=7,$F100+1,$F100)),$F100)))</f>
-        <v>46241</v>
+        <v>46272</v>
       </c>
       <c r="H100" s="69" t="n">
         <f aca="false">IF($G100="",0,IF(AND($G100&gt;='Cash Flow'!$E$6,$G100&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15307,15 +15307,15 @@
       </c>
       <c r="I100" s="69" t="n">
         <f aca="false">IF($H100=1,INT(($G100-'Cash Flow'!$E$6)/7)+1,"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J100" s="66" t="n">
         <f aca="false">IF($H100=1,$G100*10000+ROW(),"")</f>
-        <v>462410100</v>
+        <v>462720100</v>
       </c>
       <c r="K100" s="66" t="n">
         <f aca="false">IF($H100=1,$I100*1000+COUNTIFS($I$4:$I$483,$I100,$J$4:$J$483,"&lt;"&amp;$J100)+1,"")</f>
-        <v>1002</v>
+        <v>5006</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15339,11 +15339,11 @@
       </c>
       <c r="F101" s="68" t="n">
         <f aca="false">IF($C101="","",IF(Recurring!$E$11="Weekly",Recurring!$F$11+7*1,IF(Recurring!$E$11="Every 2 Weeks",Recurring!$F$11+14*1,IF(Recurring!$E$11="Monthly",EDATE(Recurring!$F$11,1),IF(Recurring!$E$11="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+1),2)=1,EOMONTH(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+1)/2)),DATE(YEAR(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+1)/2))),MONTH(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+1)/2))),15)),IF(Recurring!$E$11="One Time",IF(2=1,Recurring!$F$11,""),""))))))</f>
-        <v>46272</v>
+        <v>46302</v>
       </c>
       <c r="G101" s="68" t="n">
         <f aca="false">IF($F101="","",IF(Recurring!$G$11="Move Before",IF(WEEKDAY($F101,2)=6,$F101-1,IF(WEEKDAY($F101,2)=7,$F101-2,$F101)),IF(Recurring!$G$11="Move After",IF(WEEKDAY($F101,2)=6,$F101+2,IF(WEEKDAY($F101,2)=7,$F101+1,$F101)),$F101)))</f>
-        <v>46272</v>
+        <v>46302</v>
       </c>
       <c r="H101" s="69" t="n">
         <f aca="false">IF($G101="",0,IF(AND($G101&gt;='Cash Flow'!$E$6,$G101&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15351,15 +15351,15 @@
       </c>
       <c r="I101" s="69" t="n">
         <f aca="false">IF($H101=1,INT(($G101-'Cash Flow'!$E$6)/7)+1,"")</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J101" s="66" t="n">
         <f aca="false">IF($H101=1,$G101*10000+ROW(),"")</f>
-        <v>462720101</v>
+        <v>463020101</v>
       </c>
       <c r="K101" s="66" t="n">
         <f aca="false">IF($H101=1,$I101*1000+COUNTIFS($I$4:$I$483,$I101,$J$4:$J$483,"&lt;"&amp;$J101)+1,"")</f>
-        <v>5006</v>
+        <v>9007</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15383,27 +15383,27 @@
       </c>
       <c r="F102" s="68" t="n">
         <f aca="false">IF($C102="","",IF(Recurring!$E$11="Weekly",Recurring!$F$11+7*2,IF(Recurring!$E$11="Every 2 Weeks",Recurring!$F$11+14*2,IF(Recurring!$E$11="Monthly",EDATE(Recurring!$F$11,2),IF(Recurring!$E$11="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+2),2)=1,EOMONTH(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+2)/2)),DATE(YEAR(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+2)/2))),MONTH(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+2)/2))),15)),IF(Recurring!$E$11="One Time",IF(3=1,Recurring!$F$11,""),""))))))</f>
-        <v>46302</v>
+        <v>46333</v>
       </c>
       <c r="G102" s="68" t="n">
         <f aca="false">IF($F102="","",IF(Recurring!$G$11="Move Before",IF(WEEKDAY($F102,2)=6,$F102-1,IF(WEEKDAY($F102,2)=7,$F102-2,$F102)),IF(Recurring!$G$11="Move After",IF(WEEKDAY($F102,2)=6,$F102+2,IF(WEEKDAY($F102,2)=7,$F102+1,$F102)),$F102)))</f>
-        <v>46302</v>
+        <v>46333</v>
       </c>
       <c r="H102" s="69" t="n">
         <f aca="false">IF($G102="",0,IF(AND($G102&gt;='Cash Flow'!$E$6,$G102&lt;'Cash Flow'!$E$6+91),1,0))</f>
-        <v>1</v>
-      </c>
-      <c r="I102" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="I102" s="69" t="str">
         <f aca="false">IF($H102=1,INT(($G102-'Cash Flow'!$E$6)/7)+1,"")</f>
-        <v>9</v>
-      </c>
-      <c r="J102" s="66" t="n">
+        <v/>
+      </c>
+      <c r="J102" s="66" t="str">
         <f aca="false">IF($H102=1,$G102*10000+ROW(),"")</f>
-        <v>463020102</v>
-      </c>
-      <c r="K102" s="66" t="n">
+        <v/>
+      </c>
+      <c r="K102" s="66" t="str">
         <f aca="false">IF($H102=1,$I102*1000+COUNTIFS($I$4:$I$483,$I102,$J$4:$J$483,"&lt;"&amp;$J102)+1,"")</f>
-        <v>9007</v>
+        <v/>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15427,11 +15427,11 @@
       </c>
       <c r="F103" s="68" t="n">
         <f aca="false">IF($C103="","",IF(Recurring!$E$11="Weekly",Recurring!$F$11+7*3,IF(Recurring!$E$11="Every 2 Weeks",Recurring!$F$11+14*3,IF(Recurring!$E$11="Monthly",EDATE(Recurring!$F$11,3),IF(Recurring!$E$11="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+3),2)=1,EOMONTH(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+3)/2)),DATE(YEAR(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+3)/2))),MONTH(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+3)/2))),15)),IF(Recurring!$E$11="One Time",IF(4=1,Recurring!$F$11,""),""))))))</f>
-        <v>46333</v>
+        <v>46363</v>
       </c>
       <c r="G103" s="68" t="n">
         <f aca="false">IF($F103="","",IF(Recurring!$G$11="Move Before",IF(WEEKDAY($F103,2)=6,$F103-1,IF(WEEKDAY($F103,2)=7,$F103-2,$F103)),IF(Recurring!$G$11="Move After",IF(WEEKDAY($F103,2)=6,$F103+2,IF(WEEKDAY($F103,2)=7,$F103+1,$F103)),$F103)))</f>
-        <v>46333</v>
+        <v>46363</v>
       </c>
       <c r="H103" s="69" t="n">
         <f aca="false">IF($G103="",0,IF(AND($G103&gt;='Cash Flow'!$E$6,$G103&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15471,11 +15471,11 @@
       </c>
       <c r="F104" s="68" t="n">
         <f aca="false">IF($C104="","",IF(Recurring!$E$11="Weekly",Recurring!$F$11+7*4,IF(Recurring!$E$11="Every 2 Weeks",Recurring!$F$11+14*4,IF(Recurring!$E$11="Monthly",EDATE(Recurring!$F$11,4),IF(Recurring!$E$11="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+4),2)=1,EOMONTH(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+4)/2)),DATE(YEAR(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+4)/2))),MONTH(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+4)/2))),15)),IF(Recurring!$E$11="One Time",IF(5=1,Recurring!$F$11,""),""))))))</f>
-        <v>46363</v>
+        <v>46394</v>
       </c>
       <c r="G104" s="68" t="n">
         <f aca="false">IF($F104="","",IF(Recurring!$G$11="Move Before",IF(WEEKDAY($F104,2)=6,$F104-1,IF(WEEKDAY($F104,2)=7,$F104-2,$F104)),IF(Recurring!$G$11="Move After",IF(WEEKDAY($F104,2)=6,$F104+2,IF(WEEKDAY($F104,2)=7,$F104+1,$F104)),$F104)))</f>
-        <v>46363</v>
+        <v>46394</v>
       </c>
       <c r="H104" s="69" t="n">
         <f aca="false">IF($G104="",0,IF(AND($G104&gt;='Cash Flow'!$E$6,$G104&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15515,11 +15515,11 @@
       </c>
       <c r="F105" s="68" t="n">
         <f aca="false">IF($C105="","",IF(Recurring!$E$11="Weekly",Recurring!$F$11+7*5,IF(Recurring!$E$11="Every 2 Weeks",Recurring!$F$11+14*5,IF(Recurring!$E$11="Monthly",EDATE(Recurring!$F$11,5),IF(Recurring!$E$11="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+5),2)=1,EOMONTH(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+5)/2)),DATE(YEAR(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+5)/2))),MONTH(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+5)/2))),15)),IF(Recurring!$E$11="One Time",IF(6=1,Recurring!$F$11,""),""))))))</f>
-        <v>46394</v>
+        <v>46425</v>
       </c>
       <c r="G105" s="68" t="n">
         <f aca="false">IF($F105="","",IF(Recurring!$G$11="Move Before",IF(WEEKDAY($F105,2)=6,$F105-1,IF(WEEKDAY($F105,2)=7,$F105-2,$F105)),IF(Recurring!$G$11="Move After",IF(WEEKDAY($F105,2)=6,$F105+2,IF(WEEKDAY($F105,2)=7,$F105+1,$F105)),$F105)))</f>
-        <v>46394</v>
+        <v>46425</v>
       </c>
       <c r="H105" s="69" t="n">
         <f aca="false">IF($G105="",0,IF(AND($G105&gt;='Cash Flow'!$E$6,$G105&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15559,11 +15559,11 @@
       </c>
       <c r="F106" s="68" t="n">
         <f aca="false">IF($C106="","",IF(Recurring!$E$11="Weekly",Recurring!$F$11+7*6,IF(Recurring!$E$11="Every 2 Weeks",Recurring!$F$11+14*6,IF(Recurring!$E$11="Monthly",EDATE(Recurring!$F$11,6),IF(Recurring!$E$11="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+6),2)=1,EOMONTH(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+6)/2)),DATE(YEAR(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+6)/2))),MONTH(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+6)/2))),15)),IF(Recurring!$E$11="One Time",IF(7=1,Recurring!$F$11,""),""))))))</f>
-        <v>46425</v>
+        <v>46453</v>
       </c>
       <c r="G106" s="68" t="n">
         <f aca="false">IF($F106="","",IF(Recurring!$G$11="Move Before",IF(WEEKDAY($F106,2)=6,$F106-1,IF(WEEKDAY($F106,2)=7,$F106-2,$F106)),IF(Recurring!$G$11="Move After",IF(WEEKDAY($F106,2)=6,$F106+2,IF(WEEKDAY($F106,2)=7,$F106+1,$F106)),$F106)))</f>
-        <v>46425</v>
+        <v>46453</v>
       </c>
       <c r="H106" s="69" t="n">
         <f aca="false">IF($G106="",0,IF(AND($G106&gt;='Cash Flow'!$E$6,$G106&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15603,11 +15603,11 @@
       </c>
       <c r="F107" s="68" t="n">
         <f aca="false">IF($C107="","",IF(Recurring!$E$11="Weekly",Recurring!$F$11+7*7,IF(Recurring!$E$11="Every 2 Weeks",Recurring!$F$11+14*7,IF(Recurring!$E$11="Monthly",EDATE(Recurring!$F$11,7),IF(Recurring!$E$11="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+7),2)=1,EOMONTH(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+7)/2)),DATE(YEAR(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+7)/2))),MONTH(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+7)/2))),15)),IF(Recurring!$E$11="One Time",IF(8=1,Recurring!$F$11,""),""))))))</f>
-        <v>46453</v>
+        <v>46484</v>
       </c>
       <c r="G107" s="68" t="n">
         <f aca="false">IF($F107="","",IF(Recurring!$G$11="Move Before",IF(WEEKDAY($F107,2)=6,$F107-1,IF(WEEKDAY($F107,2)=7,$F107-2,$F107)),IF(Recurring!$G$11="Move After",IF(WEEKDAY($F107,2)=6,$F107+2,IF(WEEKDAY($F107,2)=7,$F107+1,$F107)),$F107)))</f>
-        <v>46453</v>
+        <v>46484</v>
       </c>
       <c r="H107" s="69" t="n">
         <f aca="false">IF($G107="",0,IF(AND($G107&gt;='Cash Flow'!$E$6,$G107&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15647,11 +15647,11 @@
       </c>
       <c r="F108" s="68" t="n">
         <f aca="false">IF($C108="","",IF(Recurring!$E$11="Weekly",Recurring!$F$11+7*8,IF(Recurring!$E$11="Every 2 Weeks",Recurring!$F$11+14*8,IF(Recurring!$E$11="Monthly",EDATE(Recurring!$F$11,8),IF(Recurring!$E$11="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+8),2)=1,EOMONTH(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+8)/2)),DATE(YEAR(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+8)/2))),MONTH(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+8)/2))),15)),IF(Recurring!$E$11="One Time",IF(9=1,Recurring!$F$11,""),""))))))</f>
-        <v>46484</v>
+        <v>46514</v>
       </c>
       <c r="G108" s="68" t="n">
         <f aca="false">IF($F108="","",IF(Recurring!$G$11="Move Before",IF(WEEKDAY($F108,2)=6,$F108-1,IF(WEEKDAY($F108,2)=7,$F108-2,$F108)),IF(Recurring!$G$11="Move After",IF(WEEKDAY($F108,2)=6,$F108+2,IF(WEEKDAY($F108,2)=7,$F108+1,$F108)),$F108)))</f>
-        <v>46484</v>
+        <v>46514</v>
       </c>
       <c r="H108" s="69" t="n">
         <f aca="false">IF($G108="",0,IF(AND($G108&gt;='Cash Flow'!$E$6,$G108&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15691,11 +15691,11 @@
       </c>
       <c r="F109" s="68" t="n">
         <f aca="false">IF($C109="","",IF(Recurring!$E$11="Weekly",Recurring!$F$11+7*9,IF(Recurring!$E$11="Every 2 Weeks",Recurring!$F$11+14*9,IF(Recurring!$E$11="Monthly",EDATE(Recurring!$F$11,9),IF(Recurring!$E$11="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+9),2)=1,EOMONTH(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+9)/2)),DATE(YEAR(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+9)/2))),MONTH(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+9)/2))),15)),IF(Recurring!$E$11="One Time",IF(10=1,Recurring!$F$11,""),""))))))</f>
-        <v>46514</v>
+        <v>46545</v>
       </c>
       <c r="G109" s="68" t="n">
         <f aca="false">IF($F109="","",IF(Recurring!$G$11="Move Before",IF(WEEKDAY($F109,2)=6,$F109-1,IF(WEEKDAY($F109,2)=7,$F109-2,$F109)),IF(Recurring!$G$11="Move After",IF(WEEKDAY($F109,2)=6,$F109+2,IF(WEEKDAY($F109,2)=7,$F109+1,$F109)),$F109)))</f>
-        <v>46514</v>
+        <v>46545</v>
       </c>
       <c r="H109" s="69" t="n">
         <f aca="false">IF($G109="",0,IF(AND($G109&gt;='Cash Flow'!$E$6,$G109&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15735,11 +15735,11 @@
       </c>
       <c r="F110" s="68" t="n">
         <f aca="false">IF($C110="","",IF(Recurring!$E$11="Weekly",Recurring!$F$11+7*10,IF(Recurring!$E$11="Every 2 Weeks",Recurring!$F$11+14*10,IF(Recurring!$E$11="Monthly",EDATE(Recurring!$F$11,10),IF(Recurring!$E$11="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+10),2)=1,EOMONTH(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+10)/2)),DATE(YEAR(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+10)/2))),MONTH(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+10)/2))),15)),IF(Recurring!$E$11="One Time",IF(11=1,Recurring!$F$11,""),""))))))</f>
-        <v>46545</v>
+        <v>46575</v>
       </c>
       <c r="G110" s="68" t="n">
         <f aca="false">IF($F110="","",IF(Recurring!$G$11="Move Before",IF(WEEKDAY($F110,2)=6,$F110-1,IF(WEEKDAY($F110,2)=7,$F110-2,$F110)),IF(Recurring!$G$11="Move After",IF(WEEKDAY($F110,2)=6,$F110+2,IF(WEEKDAY($F110,2)=7,$F110+1,$F110)),$F110)))</f>
-        <v>46545</v>
+        <v>46575</v>
       </c>
       <c r="H110" s="69" t="n">
         <f aca="false">IF($G110="",0,IF(AND($G110&gt;='Cash Flow'!$E$6,$G110&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15779,11 +15779,11 @@
       </c>
       <c r="F111" s="68" t="n">
         <f aca="false">IF($C111="","",IF(Recurring!$E$11="Weekly",Recurring!$F$11+7*11,IF(Recurring!$E$11="Every 2 Weeks",Recurring!$F$11+14*11,IF(Recurring!$E$11="Monthly",EDATE(Recurring!$F$11,11),IF(Recurring!$E$11="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+11),2)=1,EOMONTH(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+11)/2)),DATE(YEAR(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+11)/2))),MONTH(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+11)/2))),15)),IF(Recurring!$E$11="One Time",IF(12=1,Recurring!$F$11,""),""))))))</f>
-        <v>46575</v>
+        <v>46606</v>
       </c>
       <c r="G111" s="68" t="n">
         <f aca="false">IF($F111="","",IF(Recurring!$G$11="Move Before",IF(WEEKDAY($F111,2)=6,$F111-1,IF(WEEKDAY($F111,2)=7,$F111-2,$F111)),IF(Recurring!$G$11="Move After",IF(WEEKDAY($F111,2)=6,$F111+2,IF(WEEKDAY($F111,2)=7,$F111+1,$F111)),$F111)))</f>
-        <v>46575</v>
+        <v>46606</v>
       </c>
       <c r="H111" s="69" t="n">
         <f aca="false">IF($G111="",0,IF(AND($G111&gt;='Cash Flow'!$E$6,$G111&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15823,11 +15823,11 @@
       </c>
       <c r="F112" s="68" t="n">
         <f aca="false">IF($C112="","",IF(Recurring!$E$11="Weekly",Recurring!$F$11+7*12,IF(Recurring!$E$11="Every 2 Weeks",Recurring!$F$11+14*12,IF(Recurring!$E$11="Monthly",EDATE(Recurring!$F$11,12),IF(Recurring!$E$11="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+12),2)=1,EOMONTH(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+12)/2)),DATE(YEAR(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+12)/2))),MONTH(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+12)/2))),15)),IF(Recurring!$E$11="One Time",IF(13=1,Recurring!$F$11,""),""))))))</f>
-        <v>46606</v>
+        <v>46637</v>
       </c>
       <c r="G112" s="68" t="n">
         <f aca="false">IF($F112="","",IF(Recurring!$G$11="Move Before",IF(WEEKDAY($F112,2)=6,$F112-1,IF(WEEKDAY($F112,2)=7,$F112-2,$F112)),IF(Recurring!$G$11="Move After",IF(WEEKDAY($F112,2)=6,$F112+2,IF(WEEKDAY($F112,2)=7,$F112+1,$F112)),$F112)))</f>
-        <v>46606</v>
+        <v>46637</v>
       </c>
       <c r="H112" s="69" t="n">
         <f aca="false">IF($G112="",0,IF(AND($G112&gt;='Cash Flow'!$E$6,$G112&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15867,11 +15867,11 @@
       </c>
       <c r="F113" s="68" t="n">
         <f aca="false">IF($C113="","",IF(Recurring!$E$11="Weekly",Recurring!$F$11+7*13,IF(Recurring!$E$11="Every 2 Weeks",Recurring!$F$11+14*13,IF(Recurring!$E$11="Monthly",EDATE(Recurring!$F$11,13),IF(Recurring!$E$11="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+13),2)=1,EOMONTH(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+13)/2)),DATE(YEAR(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+13)/2))),MONTH(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+13)/2))),15)),IF(Recurring!$E$11="One Time",IF(14=1,Recurring!$F$11,""),""))))))</f>
-        <v>46637</v>
+        <v>46667</v>
       </c>
       <c r="G113" s="68" t="n">
         <f aca="false">IF($F113="","",IF(Recurring!$G$11="Move Before",IF(WEEKDAY($F113,2)=6,$F113-1,IF(WEEKDAY($F113,2)=7,$F113-2,$F113)),IF(Recurring!$G$11="Move After",IF(WEEKDAY($F113,2)=6,$F113+2,IF(WEEKDAY($F113,2)=7,$F113+1,$F113)),$F113)))</f>
-        <v>46637</v>
+        <v>46667</v>
       </c>
       <c r="H113" s="69" t="n">
         <f aca="false">IF($G113="",0,IF(AND($G113&gt;='Cash Flow'!$E$6,$G113&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15911,11 +15911,11 @@
       </c>
       <c r="F114" s="68" t="n">
         <f aca="false">IF($C114="","",IF(Recurring!$E$11="Weekly",Recurring!$F$11+7*14,IF(Recurring!$E$11="Every 2 Weeks",Recurring!$F$11+14*14,IF(Recurring!$E$11="Monthly",EDATE(Recurring!$F$11,14),IF(Recurring!$E$11="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+14),2)=1,EOMONTH(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+14)/2)),DATE(YEAR(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+14)/2))),MONTH(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+14)/2))),15)),IF(Recurring!$E$11="One Time",IF(15=1,Recurring!$F$11,""),""))))))</f>
-        <v>46667</v>
+        <v>46698</v>
       </c>
       <c r="G114" s="68" t="n">
         <f aca="false">IF($F114="","",IF(Recurring!$G$11="Move Before",IF(WEEKDAY($F114,2)=6,$F114-1,IF(WEEKDAY($F114,2)=7,$F114-2,$F114)),IF(Recurring!$G$11="Move After",IF(WEEKDAY($F114,2)=6,$F114+2,IF(WEEKDAY($F114,2)=7,$F114+1,$F114)),$F114)))</f>
-        <v>46667</v>
+        <v>46698</v>
       </c>
       <c r="H114" s="69" t="n">
         <f aca="false">IF($G114="",0,IF(AND($G114&gt;='Cash Flow'!$E$6,$G114&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15955,11 +15955,11 @@
       </c>
       <c r="F115" s="68" t="n">
         <f aca="false">IF($C115="","",IF(Recurring!$E$11="Weekly",Recurring!$F$11+7*15,IF(Recurring!$E$11="Every 2 Weeks",Recurring!$F$11+14*15,IF(Recurring!$E$11="Monthly",EDATE(Recurring!$F$11,15),IF(Recurring!$E$11="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+15),2)=1,EOMONTH(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+15)/2)),DATE(YEAR(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+15)/2))),MONTH(EDATE(Recurring!$F$11,INT((IF(DAY(Recurring!$F$11)&lt;=20,0,1)+15)/2))),15)),IF(Recurring!$E$11="One Time",IF(16=1,Recurring!$F$11,""),""))))))</f>
-        <v>46698</v>
+        <v>46728</v>
       </c>
       <c r="G115" s="68" t="n">
         <f aca="false">IF($F115="","",IF(Recurring!$G$11="Move Before",IF(WEEKDAY($F115,2)=6,$F115-1,IF(WEEKDAY($F115,2)=7,$F115-2,$F115)),IF(Recurring!$G$11="Move After",IF(WEEKDAY($F115,2)=6,$F115+2,IF(WEEKDAY($F115,2)=7,$F115+1,$F115)),$F115)))</f>
-        <v>46698</v>
+        <v>46728</v>
       </c>
       <c r="H115" s="69" t="n">
         <f aca="false">IF($G115="",0,IF(AND($G115&gt;='Cash Flow'!$E$6,$G115&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -16019,7 +16019,7 @@
       </c>
       <c r="K116" s="66" t="n">
         <f aca="false">IF($H116=1,$I116*1000+COUNTIFS($I$4:$I$483,$I116,$J$4:$J$483,"&lt;"&amp;$J116)+1,"")</f>
-        <v>1003</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16723,7 +16723,7 @@
       </c>
       <c r="K132" s="66" t="n">
         <f aca="false">IF($H132=1,$I132*1000+COUNTIFS($I$4:$I$483,$I132,$J$4:$J$483,"&lt;"&amp;$J132)+1,"")</f>
-        <v>1005</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Correct the Central Maine Power entries
The $43.87 monthly charge is CMP's payment plan, not a property charge - the
name was transcribed from a truncated screenshot and is now corrected. That
plan covers usage through August, so the $163.50 regular bill does not resume
until Sep 10, 2026 rather than Aug 10.

This clears the only negative week in the projection. Week 1 now ends at
$158.18 and the balance never drops below zero across all 13 weeks.

Flagged as an open question on the Instructions tab: the $43.87 plan is still
set to repeat monthly from Aug 25, so if it ends once the $163.50 billing
resumes it needs to be marked inactive, or the sheet will charge both from
September onward.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0171RmRt5NEruH3aRWtNMF8Q
</commit_message>
<xml_diff>
--- a/Weekly_Cash_Flow_Survival.xlsx
+++ b/Weekly_Cash_Flow_Survival.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">'Cash Flow'!$A$1:$K$284</definedName>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Instructions!$A$1:$C$44</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Instructions!$A$1:$C$45</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">Recurring!$A$1:$J$38</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">Recurring!$4:$4</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Summary!$A$1:$J$28</definedName>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="166">
   <si>
     <t xml:space="preserve">WEEKLY CASH FLOW SURVIVAL WORKSHEET</t>
   </si>
@@ -207,6 +207,9 @@
     <t xml:space="preserve">Progressive Insurance ($143.37) was cut off at the bottom of the third screenshot, so its due date is set to Aug 31, 2026. Correct it on the Recurring tab if that is wrong.</t>
   </si>
   <si>
+    <t xml:space="preserve">Central Maine Power: the $43.87 payment plan covers usage through August, so the $163.50 regular bill does not start until Sep 10, 2026. OPEN QUESTION: the $43.87 plan is still set to repeat every month from Aug 25. If the plan ends once the $163.50 billing resumes, set its Active to No or give it an end, or the sheet will charge you both from September onward.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Patrick Rombalski is 'Twice a Month' with Weekend Rule = Move Before, which is why the August payment lands on Fri Aug 14 rather than Sat Aug 15, matching your app.</t>
   </si>
   <si>
@@ -330,7 +333,7 @@
     <t xml:space="preserve">Microsoft</t>
   </si>
   <si>
-    <t xml:space="preserve">Central Maine Power: Property</t>
+    <t xml:space="preserve">Central Maine Power: Payment Plan</t>
   </si>
   <si>
     <t xml:space="preserve">Maine Revenue Services (2)</t>
@@ -1427,7 +1430,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:C44"/>
+  <dimension ref="B2:C45"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -1717,6 +1720,14 @@
       </c>
       <c r="C44" s="14" t="s">
         <v>61</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B45" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="C45" s="14" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -1752,44 +1763,44 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J4" s="15" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1797,10 +1808,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D5" s="18" t="n">
         <v>90</v>
@@ -1812,13 +1823,13 @@
         <v>46246</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J5" s="6"/>
     </row>
@@ -1827,10 +1838,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D6" s="23" t="n">
         <v>790</v>
@@ -1842,13 +1853,13 @@
         <v>46248</v>
       </c>
       <c r="G6" s="22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H6" s="22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I6" s="21" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J6" s="21"/>
     </row>
@@ -1857,10 +1868,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D7" s="18" t="n">
         <v>21.1</v>
@@ -1872,13 +1883,13 @@
         <v>46269</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J7" s="6"/>
     </row>
@@ -1887,10 +1898,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D8" s="23" t="n">
         <v>20</v>
@@ -1902,13 +1913,13 @@
         <v>46270</v>
       </c>
       <c r="G8" s="22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H8" s="22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I8" s="21" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J8" s="21"/>
     </row>
@@ -1917,10 +1928,10 @@
         <v>5</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D9" s="18" t="n">
         <v>10</v>
@@ -1932,13 +1943,13 @@
         <v>46270</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J9" s="6"/>
     </row>
@@ -1947,10 +1958,10 @@
         <v>6</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D10" s="23" t="n">
         <v>4.99</v>
@@ -1962,13 +1973,13 @@
         <v>46272</v>
       </c>
       <c r="G10" s="22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H10" s="22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I10" s="21" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J10" s="21"/>
     </row>
@@ -1977,10 +1988,10 @@
         <v>7</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D11" s="18" t="n">
         <v>500</v>
@@ -1992,13 +2003,13 @@
         <v>46272</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J11" s="6"/>
     </row>
@@ -2007,10 +2018,10 @@
         <v>8</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D12" s="23" t="n">
         <v>163.5</v>
@@ -2019,16 +2030,16 @@
         <v>46</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>46244</v>
+        <v>46275</v>
       </c>
       <c r="G12" s="22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H12" s="22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I12" s="21" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J12" s="21"/>
     </row>
@@ -2037,10 +2048,10 @@
         <v>9</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D13" s="18" t="n">
         <v>2.99</v>
@@ -2052,13 +2063,13 @@
         <v>46247</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H13" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J13" s="6"/>
     </row>
@@ -2067,10 +2078,10 @@
         <v>10</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D14" s="23" t="n">
         <v>350</v>
@@ -2082,13 +2093,13 @@
         <v>46248</v>
       </c>
       <c r="G14" s="22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H14" s="22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I14" s="21" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J14" s="21"/>
     </row>
@@ -2097,10 +2108,10 @@
         <v>11</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D15" s="18" t="n">
         <v>171.1</v>
@@ -2112,13 +2123,13 @@
         <v>46250</v>
       </c>
       <c r="G15" s="17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H15" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J15" s="6"/>
     </row>
@@ -2127,10 +2138,10 @@
         <v>12</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D16" s="23" t="n">
         <v>45</v>
@@ -2142,13 +2153,13 @@
         <v>46250</v>
       </c>
       <c r="G16" s="22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H16" s="22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I16" s="21" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J16" s="21"/>
     </row>
@@ -2157,10 +2168,10 @@
         <v>13</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D17" s="18" t="n">
         <v>16.99</v>
@@ -2172,13 +2183,13 @@
         <v>46252</v>
       </c>
       <c r="G17" s="17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H17" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J17" s="6"/>
     </row>
@@ -2187,10 +2198,10 @@
         <v>14</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D18" s="23" t="n">
         <v>13.7</v>
@@ -2202,13 +2213,13 @@
         <v>46259</v>
       </c>
       <c r="G18" s="22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H18" s="22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I18" s="21" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J18" s="21"/>
     </row>
@@ -2217,10 +2228,10 @@
         <v>15</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D19" s="18" t="n">
         <v>43.87</v>
@@ -2232,13 +2243,13 @@
         <v>46259</v>
       </c>
       <c r="G19" s="17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H19" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J19" s="6"/>
     </row>
@@ -2247,10 +2258,10 @@
         <v>16</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D20" s="23" t="n">
         <v>150</v>
@@ -2262,13 +2273,13 @@
         <v>46264</v>
       </c>
       <c r="G20" s="22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H20" s="22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I20" s="21" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J20" s="21"/>
     </row>
@@ -2277,10 +2288,10 @@
         <v>17</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D21" s="18" t="n">
         <v>143.37</v>
@@ -2292,13 +2303,13 @@
         <v>46265</v>
       </c>
       <c r="G21" s="17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H21" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J21" s="6"/>
     </row>
@@ -2486,17 +2497,17 @@
     </row>
     <row r="36" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="14" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="25" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -2563,17 +2574,17 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E5" s="26" t="n">
         <v>71.17</v>
@@ -2581,7 +2592,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E6" s="27" t="n">
         <v>46241</v>
@@ -2593,7 +2604,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E7" s="26" t="n">
         <v>200</v>
@@ -2601,7 +2612,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E8" s="30" t="n">
         <f aca="true">TODAY()</f>
@@ -2610,12 +2621,12 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="25" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="25" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2628,7 +2639,7 @@
       <c r="E13" s="32"/>
       <c r="F13" s="32"/>
       <c r="G13" s="33" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H13" s="32"/>
       <c r="I13" s="34" t="n">
@@ -2643,19 +2654,19 @@
     </row>
     <row r="14" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="35" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C14" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D14" s="35" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F14" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G14" s="36" t="s">
         <v>18</v>
@@ -2664,41 +2675,41 @@
         <v>20</v>
       </c>
       <c r="I14" s="35" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J14" s="35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="11" t="str">
         <f aca="false">IFERROR(INDEX(Schedule!$C$4:$C$483,MATCH(1001,Schedule!$K$4:$K$483,0)),"")</f>
-        <v>Central Maine Power Co.</v>
+        <v>Bruno's Restaurant (paycheck)</v>
       </c>
       <c r="C15" s="38" t="n">
         <f aca="false">IF($B15="","",INDEX(Schedule!$G$4:$G$483,MATCH(1001,Schedule!$K$4:$K$483,0)))</f>
-        <v>46244</v>
+        <v>46246</v>
       </c>
       <c r="D15" s="39" t="str">
         <f aca="false">IF($B15="","",INDEX(Schedule!$D$4:$D$483,MATCH(1001,Schedule!$K$4:$K$483,0)))</f>
-        <v>Expense</v>
+        <v>Income</v>
       </c>
       <c r="E15" s="40" t="n">
         <f aca="false">IF($B15="","",INDEX(Schedule!$E$4:$E$483,MATCH(1001,Schedule!$K$4:$K$483,0)))</f>
-        <v>163.5</v>
+        <v>90</v>
       </c>
       <c r="F15" s="18"/>
-      <c r="G15" s="41" t="str">
+      <c r="G15" s="41" t="n">
         <f aca="false">IF($B15="","",IF($D15="Income",IF($F15&lt;&gt;"",$F15,$E15),""))</f>
-        <v/>
-      </c>
-      <c r="H15" s="42" t="n">
+        <v>90</v>
+      </c>
+      <c r="H15" s="42" t="str">
         <f aca="false">IF($B15="","",IF($D15="Income","",IF($F15&lt;&gt;"",$F15,$E15)))</f>
-        <v>163.5</v>
+        <v/>
       </c>
       <c r="I15" s="43" t="n">
         <f aca="false">IF($B15="","",$I$13+SUM($G$15:$G15)-SUM($H$15:$H15))</f>
-        <v>-92.33</v>
+        <v>161.17</v>
       </c>
       <c r="J15" s="44" t="str">
         <f aca="true">IF($B15="","",IF($F15&lt;&gt;"","PAID",IF($C15&lt;TODAY(),"PAST DUE",IF($C15&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -2708,32 +2719,32 @@
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="11" t="str">
         <f aca="false">IFERROR(INDEX(Schedule!$C$4:$C$483,MATCH(1002,Schedule!$K$4:$K$483,0)),"")</f>
-        <v>Bruno's Restaurant (paycheck)</v>
+        <v>Apple: iCloud</v>
       </c>
       <c r="C16" s="38" t="n">
         <f aca="false">IF($B16="","",INDEX(Schedule!$G$4:$G$483,MATCH(1002,Schedule!$K$4:$K$483,0)))</f>
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="D16" s="39" t="str">
         <f aca="false">IF($B16="","",INDEX(Schedule!$D$4:$D$483,MATCH(1002,Schedule!$K$4:$K$483,0)))</f>
-        <v>Income</v>
+        <v>Expense</v>
       </c>
       <c r="E16" s="40" t="n">
         <f aca="false">IF($B16="","",INDEX(Schedule!$E$4:$E$483,MATCH(1002,Schedule!$K$4:$K$483,0)))</f>
-        <v>90</v>
+        <v>2.99</v>
       </c>
       <c r="F16" s="18"/>
-      <c r="G16" s="41" t="n">
+      <c r="G16" s="41" t="str">
         <f aca="false">IF($B16="","",IF($D16="Income",IF($F16&lt;&gt;"",$F16,$E16),""))</f>
-        <v>90</v>
-      </c>
-      <c r="H16" s="42" t="str">
+        <v/>
+      </c>
+      <c r="H16" s="42" t="n">
         <f aca="false">IF($B16="","",IF($D16="Income","",IF($F16&lt;&gt;"",$F16,$E16)))</f>
-        <v/>
+        <v>2.99</v>
       </c>
       <c r="I16" s="43" t="n">
         <f aca="false">IF($B16="","",$I$13+SUM($G$15:$G16)-SUM($H$15:$H16))</f>
-        <v>-2.32999999999998</v>
+        <v>158.18</v>
       </c>
       <c r="J16" s="44" t="str">
         <f aca="true">IF($B16="","",IF($F16&lt;&gt;"","PAID",IF($C16&lt;TODAY(),"PAST DUE",IF($C16&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -2743,36 +2754,36 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="11" t="str">
         <f aca="false">IFERROR(INDEX(Schedule!$C$4:$C$483,MATCH(1003,Schedule!$K$4:$K$483,0)),"")</f>
-        <v>Apple: iCloud</v>
-      </c>
-      <c r="C17" s="38" t="n">
+        <v/>
+      </c>
+      <c r="C17" s="38" t="str">
         <f aca="false">IF($B17="","",INDEX(Schedule!$G$4:$G$483,MATCH(1003,Schedule!$K$4:$K$483,0)))</f>
-        <v>46247</v>
+        <v/>
       </c>
       <c r="D17" s="39" t="str">
         <f aca="false">IF($B17="","",INDEX(Schedule!$D$4:$D$483,MATCH(1003,Schedule!$K$4:$K$483,0)))</f>
-        <v>Expense</v>
-      </c>
-      <c r="E17" s="40" t="n">
+        <v/>
+      </c>
+      <c r="E17" s="40" t="str">
         <f aca="false">IF($B17="","",INDEX(Schedule!$E$4:$E$483,MATCH(1003,Schedule!$K$4:$K$483,0)))</f>
-        <v>2.99</v>
+        <v/>
       </c>
       <c r="F17" s="18"/>
       <c r="G17" s="41" t="str">
         <f aca="false">IF($B17="","",IF($D17="Income",IF($F17&lt;&gt;"",$F17,$E17),""))</f>
         <v/>
       </c>
-      <c r="H17" s="42" t="n">
+      <c r="H17" s="42" t="str">
         <f aca="false">IF($B17="","",IF($D17="Income","",IF($F17&lt;&gt;"",$F17,$E17)))</f>
-        <v>2.99</v>
-      </c>
-      <c r="I17" s="43" t="n">
+        <v/>
+      </c>
+      <c r="I17" s="43" t="str">
         <f aca="false">IF($B17="","",$I$13+SUM($G$15:$G17)-SUM($H$15:$H17))</f>
-        <v>-5.31999999999999</v>
+        <v/>
       </c>
       <c r="J17" s="44" t="str">
         <f aca="true">IF($B17="","",IF($F17&lt;&gt;"","PAID",IF($C17&lt;TODAY(),"PAST DUE",IF($C17&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
-        <v>DUE</v>
+        <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3022,7 +3033,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="45" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C25" s="46"/>
       <c r="D25" s="46"/>
@@ -3155,7 +3166,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="47" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C32" s="48"/>
       <c r="D32" s="48"/>
@@ -3167,19 +3178,19 @@
       </c>
       <c r="H32" s="49" t="n">
         <f aca="false">SUM($H$15:$H$31)</f>
-        <v>166.49</v>
+        <v>2.99</v>
       </c>
       <c r="I32" s="50" t="n">
         <f aca="false">$I$13+$G$32-$H$32</f>
-        <v>-5.31999999999999</v>
+        <v>158.18</v>
       </c>
       <c r="J32" s="51" t="str">
         <f aca="false">IF($I$32&lt;0,"SHORTFALL",IF($I$32&lt;$E$7,"TIGHT","OK"))</f>
-        <v>SHORTFALL</v>
+        <v>TIGHT</v>
       </c>
       <c r="K32" s="25" t="str">
         <f aca="false">"In "&amp;TEXT($G$32,"$#,##0.00")&amp;"   less out "&amp;TEXT($H$32,"$#,##0.00")&amp;"   =  net "&amp;TEXT($G$32-$H$32,"$#,##0.00;-$#,##0.00")</f>
-        <v>In $90.00   less out $166.49   =  net -$76.49</v>
+        <v>In $90.00   less out $2.99   =  net $87.01</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3192,12 +3203,12 @@
       <c r="E34" s="32"/>
       <c r="F34" s="32"/>
       <c r="G34" s="33" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H34" s="32"/>
       <c r="I34" s="34" t="n">
         <f aca="false">$I$32</f>
-        <v>-5.31999999999999</v>
+        <v>158.18</v>
       </c>
       <c r="J34" s="32"/>
       <c r="K34" s="28" t="str">
@@ -3207,19 +3218,19 @@
     </row>
     <row r="35" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="35" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C35" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D35" s="35" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E35" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F35" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G35" s="36" t="s">
         <v>18</v>
@@ -3228,10 +3239,10 @@
         <v>20</v>
       </c>
       <c r="I35" s="35" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J35" s="35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3262,7 +3273,7 @@
       </c>
       <c r="I36" s="43" t="n">
         <f aca="false">IF($B36="","",$I$34+SUM($G$36:$G36)-SUM($H$36:$H36))</f>
-        <v>784.68</v>
+        <v>948.18</v>
       </c>
       <c r="J36" s="44" t="str">
         <f aca="true">IF($B36="","",IF($F36&lt;&gt;"","PAID",IF($C36&lt;TODAY(),"PAST DUE",IF($C36&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -3297,7 +3308,7 @@
       </c>
       <c r="I37" s="43" t="n">
         <f aca="false">IF($B37="","",$I$34+SUM($G$36:$G37)-SUM($H$36:$H37))</f>
-        <v>434.68</v>
+        <v>598.18</v>
       </c>
       <c r="J37" s="44" t="str">
         <f aca="true">IF($B37="","",IF($F37&lt;&gt;"","PAID",IF($C37&lt;TODAY(),"PAST DUE",IF($C37&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -3332,7 +3343,7 @@
       </c>
       <c r="I38" s="43" t="n">
         <f aca="false">IF($B38="","",$I$34+SUM($G$36:$G38)-SUM($H$36:$H38))</f>
-        <v>263.58</v>
+        <v>427.08</v>
       </c>
       <c r="J38" s="44" t="str">
         <f aca="true">IF($B38="","",IF($F38&lt;&gt;"","PAID",IF($C38&lt;TODAY(),"PAST DUE",IF($C38&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -3367,7 +3378,7 @@
       </c>
       <c r="I39" s="43" t="n">
         <f aca="false">IF($B39="","",$I$34+SUM($G$36:$G39)-SUM($H$36:$H39))</f>
-        <v>218.58</v>
+        <v>382.08</v>
       </c>
       <c r="J39" s="44" t="str">
         <f aca="true">IF($B39="","",IF($F39&lt;&gt;"","PAID",IF($C39&lt;TODAY(),"PAST DUE",IF($C39&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -3402,7 +3413,7 @@
       </c>
       <c r="I40" s="43" t="n">
         <f aca="false">IF($B40="","",$I$34+SUM($G$36:$G40)-SUM($H$36:$H40))</f>
-        <v>201.59</v>
+        <v>365.09</v>
       </c>
       <c r="J40" s="44" t="str">
         <f aca="true">IF($B40="","",IF($F40&lt;&gt;"","PAID",IF($C40&lt;TODAY(),"PAST DUE",IF($C40&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -3437,7 +3448,7 @@
       </c>
       <c r="I41" s="43" t="n">
         <f aca="false">IF($B41="","",$I$34+SUM($G$36:$G41)-SUM($H$36:$H41))</f>
-        <v>291.59</v>
+        <v>455.09</v>
       </c>
       <c r="J41" s="44" t="str">
         <f aca="true">IF($B41="","",IF($F41&lt;&gt;"","PAID",IF($C41&lt;TODAY(),"PAST DUE",IF($C41&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -3586,7 +3597,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="45" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C46" s="46"/>
       <c r="D46" s="46"/>
@@ -3719,7 +3730,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="47" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C53" s="48"/>
       <c r="D53" s="48"/>
@@ -3735,7 +3746,7 @@
       </c>
       <c r="I53" s="50" t="n">
         <f aca="false">$I$34+$G$53-$H$53</f>
-        <v>291.59</v>
+        <v>455.09</v>
       </c>
       <c r="J53" s="51" t="str">
         <f aca="false">IF($I$53&lt;0,"SHORTFALL",IF($I$53&lt;$E$7,"TIGHT","OK"))</f>
@@ -3756,12 +3767,12 @@
       <c r="E55" s="32"/>
       <c r="F55" s="32"/>
       <c r="G55" s="33" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H55" s="32"/>
       <c r="I55" s="34" t="n">
         <f aca="false">$I$53</f>
-        <v>291.59</v>
+        <v>455.09</v>
       </c>
       <c r="J55" s="32"/>
       <c r="K55" s="28" t="str">
@@ -3771,19 +3782,19 @@
     </row>
     <row r="56" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B56" s="35" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C56" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D56" s="35" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E56" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F56" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G56" s="36" t="s">
         <v>18</v>
@@ -3792,10 +3803,10 @@
         <v>20</v>
       </c>
       <c r="I56" s="35" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J56" s="35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3826,7 +3837,7 @@
       </c>
       <c r="I57" s="43" t="n">
         <f aca="false">IF($B57="","",$I$55+SUM($G$57:$G57)-SUM($H$57:$H57))</f>
-        <v>1081.59</v>
+        <v>1245.09</v>
       </c>
       <c r="J57" s="44" t="str">
         <f aca="true">IF($B57="","",IF($F57&lt;&gt;"","PAID",IF($C57&lt;TODAY(),"PAST DUE",IF($C57&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -3861,7 +3872,7 @@
       </c>
       <c r="I58" s="43" t="n">
         <f aca="false">IF($B58="","",$I$55+SUM($G$57:$G58)-SUM($H$57:$H58))</f>
-        <v>1067.89</v>
+        <v>1231.39</v>
       </c>
       <c r="J58" s="44" t="str">
         <f aca="true">IF($B58="","",IF($F58&lt;&gt;"","PAID",IF($C58&lt;TODAY(),"PAST DUE",IF($C58&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -3871,7 +3882,7 @@
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="11" t="str">
         <f aca="false">IFERROR(INDEX(Schedule!$C$4:$C$483,MATCH(3003,Schedule!$K$4:$K$483,0)),"")</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="C59" s="38" t="n">
         <f aca="false">IF($B59="","",INDEX(Schedule!$G$4:$G$483,MATCH(3003,Schedule!$K$4:$K$483,0)))</f>
@@ -3896,7 +3907,7 @@
       </c>
       <c r="I59" s="43" t="n">
         <f aca="false">IF($B59="","",$I$55+SUM($G$57:$G59)-SUM($H$57:$H59))</f>
-        <v>1024.02</v>
+        <v>1187.52</v>
       </c>
       <c r="J59" s="44" t="str">
         <f aca="true">IF($B59="","",IF($F59&lt;&gt;"","PAID",IF($C59&lt;TODAY(),"PAST DUE",IF($C59&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -3931,7 +3942,7 @@
       </c>
       <c r="I60" s="43" t="n">
         <f aca="false">IF($B60="","",$I$55+SUM($G$57:$G60)-SUM($H$57:$H60))</f>
-        <v>1114.02</v>
+        <v>1277.52</v>
       </c>
       <c r="J60" s="44" t="str">
         <f aca="true">IF($B60="","",IF($F60&lt;&gt;"","PAID",IF($C60&lt;TODAY(),"PAST DUE",IF($C60&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -4150,7 +4161,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="45" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C67" s="46"/>
       <c r="D67" s="46"/>
@@ -4283,7 +4294,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="47" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C74" s="48"/>
       <c r="D74" s="48"/>
@@ -4299,7 +4310,7 @@
       </c>
       <c r="I74" s="50" t="n">
         <f aca="false">$I$55+$G$74-$H$74</f>
-        <v>1114.02</v>
+        <v>1277.52</v>
       </c>
       <c r="J74" s="51" t="str">
         <f aca="false">IF($I$74&lt;0,"SHORTFALL",IF($I$74&lt;$E$7,"TIGHT","OK"))</f>
@@ -4320,12 +4331,12 @@
       <c r="E76" s="32"/>
       <c r="F76" s="32"/>
       <c r="G76" s="33" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H76" s="32"/>
       <c r="I76" s="34" t="n">
         <f aca="false">$I$74</f>
-        <v>1114.02</v>
+        <v>1277.52</v>
       </c>
       <c r="J76" s="32"/>
       <c r="K76" s="28" t="str">
@@ -4335,19 +4346,19 @@
     </row>
     <row r="77" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B77" s="35" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C77" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D77" s="35" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E77" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F77" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G77" s="36" t="s">
         <v>18</v>
@@ -4356,10 +4367,10 @@
         <v>20</v>
       </c>
       <c r="I77" s="35" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J77" s="35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4390,7 +4401,7 @@
       </c>
       <c r="I78" s="43" t="n">
         <f aca="false">IF($B78="","",$I$76+SUM($G$78:$G78)-SUM($H$78:$H78))</f>
-        <v>1904.02</v>
+        <v>2067.52</v>
       </c>
       <c r="J78" s="44" t="str">
         <f aca="true">IF($B78="","",IF($F78&lt;&gt;"","PAID",IF($C78&lt;TODAY(),"PAST DUE",IF($C78&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -4425,7 +4436,7 @@
       </c>
       <c r="I79" s="43" t="n">
         <f aca="false">IF($B79="","",$I$76+SUM($G$78:$G79)-SUM($H$78:$H79))</f>
-        <v>1754.02</v>
+        <v>1917.52</v>
       </c>
       <c r="J79" s="44" t="str">
         <f aca="true">IF($B79="","",IF($F79&lt;&gt;"","PAID",IF($C79&lt;TODAY(),"PAST DUE",IF($C79&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -4460,7 +4471,7 @@
       </c>
       <c r="I80" s="43" t="n">
         <f aca="false">IF($B80="","",$I$76+SUM($G$78:$G80)-SUM($H$78:$H80))</f>
-        <v>1404.02</v>
+        <v>1567.52</v>
       </c>
       <c r="J80" s="44" t="str">
         <f aca="true">IF($B80="","",IF($F80&lt;&gt;"","PAID",IF($C80&lt;TODAY(),"PAST DUE",IF($C80&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -4495,7 +4506,7 @@
       </c>
       <c r="I81" s="43" t="n">
         <f aca="false">IF($B81="","",$I$76+SUM($G$78:$G81)-SUM($H$78:$H81))</f>
-        <v>1260.65</v>
+        <v>1424.15</v>
       </c>
       <c r="J81" s="44" t="str">
         <f aca="true">IF($B81="","",IF($F81&lt;&gt;"","PAID",IF($C81&lt;TODAY(),"PAST DUE",IF($C81&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -4530,7 +4541,7 @@
       </c>
       <c r="I82" s="43" t="n">
         <f aca="false">IF($B82="","",$I$76+SUM($G$78:$G82)-SUM($H$78:$H82))</f>
-        <v>1350.65</v>
+        <v>1514.15</v>
       </c>
       <c r="J82" s="44" t="str">
         <f aca="true">IF($B82="","",IF($F82&lt;&gt;"","PAID",IF($C82&lt;TODAY(),"PAST DUE",IF($C82&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -4714,7 +4725,7 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="45" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C88" s="46"/>
       <c r="D88" s="46"/>
@@ -4847,7 +4858,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B95" s="47" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C95" s="48"/>
       <c r="D95" s="48"/>
@@ -4863,7 +4874,7 @@
       </c>
       <c r="I95" s="50" t="n">
         <f aca="false">$I$76+$G$95-$H$95</f>
-        <v>1350.65</v>
+        <v>1514.15</v>
       </c>
       <c r="J95" s="51" t="str">
         <f aca="false">IF($I$95&lt;0,"SHORTFALL",IF($I$95&lt;$E$7,"TIGHT","OK"))</f>
@@ -4884,12 +4895,12 @@
       <c r="E97" s="32"/>
       <c r="F97" s="32"/>
       <c r="G97" s="33" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H97" s="32"/>
       <c r="I97" s="34" t="n">
         <f aca="false">$I$95</f>
-        <v>1350.65</v>
+        <v>1514.15</v>
       </c>
       <c r="J97" s="32"/>
       <c r="K97" s="28" t="str">
@@ -4899,19 +4910,19 @@
     </row>
     <row r="98" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B98" s="35" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C98" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D98" s="35" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E98" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F98" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G98" s="36" t="s">
         <v>18</v>
@@ -4920,10 +4931,10 @@
         <v>20</v>
       </c>
       <c r="I98" s="35" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J98" s="35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4954,7 +4965,7 @@
       </c>
       <c r="I99" s="43" t="n">
         <f aca="false">IF($B99="","",$I$97+SUM($G$99:$G99)-SUM($H$99:$H99))</f>
-        <v>2140.65</v>
+        <v>2304.15</v>
       </c>
       <c r="J99" s="44" t="str">
         <f aca="true">IF($B99="","",IF($F99&lt;&gt;"","PAID",IF($C99&lt;TODAY(),"PAST DUE",IF($C99&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -4989,7 +5000,7 @@
       </c>
       <c r="I100" s="43" t="n">
         <f aca="false">IF($B100="","",$I$97+SUM($G$99:$G100)-SUM($H$99:$H100))</f>
-        <v>2119.55</v>
+        <v>2283.05</v>
       </c>
       <c r="J100" s="44" t="str">
         <f aca="true">IF($B100="","",IF($F100&lt;&gt;"","PAID",IF($C100&lt;TODAY(),"PAST DUE",IF($C100&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5024,7 +5035,7 @@
       </c>
       <c r="I101" s="43" t="n">
         <f aca="false">IF($B101="","",$I$97+SUM($G$99:$G101)-SUM($H$99:$H101))</f>
-        <v>2099.55</v>
+        <v>2263.05</v>
       </c>
       <c r="J101" s="44" t="str">
         <f aca="true">IF($B101="","",IF($F101&lt;&gt;"","PAID",IF($C101&lt;TODAY(),"PAST DUE",IF($C101&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5059,7 +5070,7 @@
       </c>
       <c r="I102" s="43" t="n">
         <f aca="false">IF($B102="","",$I$97+SUM($G$99:$G102)-SUM($H$99:$H102))</f>
-        <v>2089.55</v>
+        <v>2253.05</v>
       </c>
       <c r="J102" s="44" t="str">
         <f aca="true">IF($B102="","",IF($F102&lt;&gt;"","PAID",IF($C102&lt;TODAY(),"PAST DUE",IF($C102&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5094,7 +5105,7 @@
       </c>
       <c r="I103" s="43" t="n">
         <f aca="false">IF($B103="","",$I$97+SUM($G$99:$G103)-SUM($H$99:$H103))</f>
-        <v>2084.56</v>
+        <v>2248.06</v>
       </c>
       <c r="J103" s="44" t="str">
         <f aca="true">IF($B103="","",IF($F103&lt;&gt;"","PAID",IF($C103&lt;TODAY(),"PAST DUE",IF($C103&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5129,7 +5140,7 @@
       </c>
       <c r="I104" s="43" t="n">
         <f aca="false">IF($B104="","",$I$97+SUM($G$99:$G104)-SUM($H$99:$H104))</f>
-        <v>1584.56</v>
+        <v>1748.06</v>
       </c>
       <c r="J104" s="44" t="str">
         <f aca="true">IF($B104="","",IF($F104&lt;&gt;"","PAID",IF($C104&lt;TODAY(),"PAST DUE",IF($C104&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5164,7 +5175,7 @@
       </c>
       <c r="I105" s="43" t="n">
         <f aca="false">IF($B105="","",$I$97+SUM($G$99:$G105)-SUM($H$99:$H105))</f>
-        <v>1674.56</v>
+        <v>1838.06</v>
       </c>
       <c r="J105" s="44" t="str">
         <f aca="true">IF($B105="","",IF($F105&lt;&gt;"","PAID",IF($C105&lt;TODAY(),"PAST DUE",IF($C105&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5199,7 +5210,7 @@
       </c>
       <c r="I106" s="43" t="n">
         <f aca="false">IF($B106="","",$I$97+SUM($G$99:$G106)-SUM($H$99:$H106))</f>
-        <v>1511.06</v>
+        <v>1674.56</v>
       </c>
       <c r="J106" s="44" t="str">
         <f aca="true">IF($B106="","",IF($F106&lt;&gt;"","PAID",IF($C106&lt;TODAY(),"PAST DUE",IF($C106&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5278,7 +5289,7 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B109" s="45" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C109" s="46"/>
       <c r="D109" s="46"/>
@@ -5411,7 +5422,7 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B116" s="47" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C116" s="48"/>
       <c r="D116" s="48"/>
@@ -5427,7 +5438,7 @@
       </c>
       <c r="I116" s="50" t="n">
         <f aca="false">$I$97+$G$116-$H$116</f>
-        <v>1511.06</v>
+        <v>1674.56</v>
       </c>
       <c r="J116" s="51" t="str">
         <f aca="false">IF($I$116&lt;0,"SHORTFALL",IF($I$116&lt;$E$7,"TIGHT","OK"))</f>
@@ -5448,12 +5459,12 @@
       <c r="E118" s="32"/>
       <c r="F118" s="32"/>
       <c r="G118" s="33" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H118" s="32"/>
       <c r="I118" s="34" t="n">
         <f aca="false">$I$116</f>
-        <v>1511.06</v>
+        <v>1674.56</v>
       </c>
       <c r="J118" s="32"/>
       <c r="K118" s="28" t="str">
@@ -5463,19 +5474,19 @@
     </row>
     <row r="119" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B119" s="35" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C119" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D119" s="35" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E119" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F119" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G119" s="36" t="s">
         <v>18</v>
@@ -5484,10 +5495,10 @@
         <v>20</v>
       </c>
       <c r="I119" s="35" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J119" s="35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5518,7 +5529,7 @@
       </c>
       <c r="I120" s="43" t="n">
         <f aca="false">IF($B120="","",$I$118+SUM($G$120:$G120)-SUM($H$120:$H120))</f>
-        <v>2301.06</v>
+        <v>2464.56</v>
       </c>
       <c r="J120" s="44" t="str">
         <f aca="true">IF($B120="","",IF($F120&lt;&gt;"","PAID",IF($C120&lt;TODAY(),"PAST DUE",IF($C120&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5553,7 +5564,7 @@
       </c>
       <c r="I121" s="43" t="n">
         <f aca="false">IF($B121="","",$I$118+SUM($G$120:$G121)-SUM($H$120:$H121))</f>
-        <v>2298.07</v>
+        <v>2461.57</v>
       </c>
       <c r="J121" s="44" t="str">
         <f aca="true">IF($B121="","",IF($F121&lt;&gt;"","PAID",IF($C121&lt;TODAY(),"PAST DUE",IF($C121&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5588,7 +5599,7 @@
       </c>
       <c r="I122" s="43" t="n">
         <f aca="false">IF($B122="","",$I$118+SUM($G$120:$G122)-SUM($H$120:$H122))</f>
-        <v>1948.07</v>
+        <v>2111.57</v>
       </c>
       <c r="J122" s="44" t="str">
         <f aca="true">IF($B122="","",IF($F122&lt;&gt;"","PAID",IF($C122&lt;TODAY(),"PAST DUE",IF($C122&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5623,7 +5634,7 @@
       </c>
       <c r="I123" s="43" t="n">
         <f aca="false">IF($B123="","",$I$118+SUM($G$120:$G123)-SUM($H$120:$H123))</f>
-        <v>2038.07</v>
+        <v>2201.57</v>
       </c>
       <c r="J123" s="44" t="str">
         <f aca="true">IF($B123="","",IF($F123&lt;&gt;"","PAID",IF($C123&lt;TODAY(),"PAST DUE",IF($C123&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5658,7 +5669,7 @@
       </c>
       <c r="I124" s="43" t="n">
         <f aca="false">IF($B124="","",$I$118+SUM($G$120:$G124)-SUM($H$120:$H124))</f>
-        <v>1866.97</v>
+        <v>2030.47</v>
       </c>
       <c r="J124" s="44" t="str">
         <f aca="true">IF($B124="","",IF($F124&lt;&gt;"","PAID",IF($C124&lt;TODAY(),"PAST DUE",IF($C124&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5693,7 +5704,7 @@
       </c>
       <c r="I125" s="43" t="n">
         <f aca="false">IF($B125="","",$I$118+SUM($G$120:$G125)-SUM($H$120:$H125))</f>
-        <v>1821.97</v>
+        <v>1985.47</v>
       </c>
       <c r="J125" s="44" t="str">
         <f aca="true">IF($B125="","",IF($F125&lt;&gt;"","PAID",IF($C125&lt;TODAY(),"PAST DUE",IF($C125&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -5842,7 +5853,7 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B130" s="45" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C130" s="46"/>
       <c r="D130" s="46"/>
@@ -5975,7 +5986,7 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B137" s="47" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C137" s="48"/>
       <c r="D137" s="48"/>
@@ -5991,7 +6002,7 @@
       </c>
       <c r="I137" s="50" t="n">
         <f aca="false">$I$118+$G$137-$H$137</f>
-        <v>1821.97</v>
+        <v>1985.47</v>
       </c>
       <c r="J137" s="51" t="str">
         <f aca="false">IF($I$137&lt;0,"SHORTFALL",IF($I$137&lt;$E$7,"TIGHT","OK"))</f>
@@ -6012,12 +6023,12 @@
       <c r="E139" s="32"/>
       <c r="F139" s="32"/>
       <c r="G139" s="33" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H139" s="32"/>
       <c r="I139" s="34" t="n">
         <f aca="false">$I$137</f>
-        <v>1821.97</v>
+        <v>1985.47</v>
       </c>
       <c r="J139" s="32"/>
       <c r="K139" s="28" t="str">
@@ -6027,19 +6038,19 @@
     </row>
     <row r="140" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B140" s="35" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C140" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D140" s="35" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E140" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F140" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G140" s="36" t="s">
         <v>18</v>
@@ -6048,10 +6059,10 @@
         <v>20</v>
       </c>
       <c r="I140" s="35" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J140" s="35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6082,7 +6093,7 @@
       </c>
       <c r="I141" s="43" t="n">
         <f aca="false">IF($B141="","",$I$139+SUM($G$141:$G141)-SUM($H$141:$H141))</f>
-        <v>2611.97</v>
+        <v>2775.47</v>
       </c>
       <c r="J141" s="44" t="str">
         <f aca="true">IF($B141="","",IF($F141&lt;&gt;"","PAID",IF($C141&lt;TODAY(),"PAST DUE",IF($C141&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6117,7 +6128,7 @@
       </c>
       <c r="I142" s="43" t="n">
         <f aca="false">IF($B142="","",$I$139+SUM($G$141:$G142)-SUM($H$141:$H142))</f>
-        <v>2594.98</v>
+        <v>2758.48</v>
       </c>
       <c r="J142" s="44" t="str">
         <f aca="true">IF($B142="","",IF($F142&lt;&gt;"","PAID",IF($C142&lt;TODAY(),"PAST DUE",IF($C142&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6152,7 +6163,7 @@
       </c>
       <c r="I143" s="43" t="n">
         <f aca="false">IF($B143="","",$I$139+SUM($G$141:$G143)-SUM($H$141:$H143))</f>
-        <v>2684.98</v>
+        <v>2848.48</v>
       </c>
       <c r="J143" s="44" t="str">
         <f aca="true">IF($B143="","",IF($F143&lt;&gt;"","PAID",IF($C143&lt;TODAY(),"PAST DUE",IF($C143&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6406,7 +6417,7 @@
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B151" s="45" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C151" s="46"/>
       <c r="D151" s="46"/>
@@ -6539,7 +6550,7 @@
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B158" s="47" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C158" s="48"/>
       <c r="D158" s="48"/>
@@ -6555,7 +6566,7 @@
       </c>
       <c r="I158" s="50" t="n">
         <f aca="false">$I$139+$G$158-$H$158</f>
-        <v>2684.98</v>
+        <v>2848.48</v>
       </c>
       <c r="J158" s="51" t="str">
         <f aca="false">IF($I$158&lt;0,"SHORTFALL",IF($I$158&lt;$E$7,"TIGHT","OK"))</f>
@@ -6576,12 +6587,12 @@
       <c r="E160" s="32"/>
       <c r="F160" s="32"/>
       <c r="G160" s="33" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H160" s="32"/>
       <c r="I160" s="34" t="n">
         <f aca="false">$I$158</f>
-        <v>2684.98</v>
+        <v>2848.48</v>
       </c>
       <c r="J160" s="32"/>
       <c r="K160" s="28" t="str">
@@ -6591,19 +6602,19 @@
     </row>
     <row r="161" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B161" s="35" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C161" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D161" s="35" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E161" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F161" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G161" s="36" t="s">
         <v>18</v>
@@ -6612,10 +6623,10 @@
         <v>20</v>
       </c>
       <c r="I161" s="35" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J161" s="35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6646,7 +6657,7 @@
       </c>
       <c r="I162" s="43" t="n">
         <f aca="false">IF($B162="","",$I$160+SUM($G$162:$G162)-SUM($H$162:$H162))</f>
-        <v>3474.98</v>
+        <v>3638.48</v>
       </c>
       <c r="J162" s="44" t="str">
         <f aca="true">IF($B162="","",IF($F162&lt;&gt;"","PAID",IF($C162&lt;TODAY(),"PAST DUE",IF($C162&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6681,7 +6692,7 @@
       </c>
       <c r="I163" s="43" t="n">
         <f aca="false">IF($B163="","",$I$160+SUM($G$162:$G163)-SUM($H$162:$H163))</f>
-        <v>3461.28</v>
+        <v>3624.78</v>
       </c>
       <c r="J163" s="44" t="str">
         <f aca="true">IF($B163="","",IF($F163&lt;&gt;"","PAID",IF($C163&lt;TODAY(),"PAST DUE",IF($C163&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6691,7 +6702,7 @@
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B164" s="11" t="str">
         <f aca="false">IFERROR(INDEX(Schedule!$C$4:$C$483,MATCH(8003,Schedule!$K$4:$K$483,0)),"")</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="C164" s="38" t="n">
         <f aca="false">IF($B164="","",INDEX(Schedule!$G$4:$G$483,MATCH(8003,Schedule!$K$4:$K$483,0)))</f>
@@ -6716,7 +6727,7 @@
       </c>
       <c r="I164" s="43" t="n">
         <f aca="false">IF($B164="","",$I$160+SUM($G$162:$G164)-SUM($H$162:$H164))</f>
-        <v>3417.41</v>
+        <v>3580.91</v>
       </c>
       <c r="J164" s="44" t="str">
         <f aca="true">IF($B164="","",IF($F164&lt;&gt;"","PAID",IF($C164&lt;TODAY(),"PAST DUE",IF($C164&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6751,7 +6762,7 @@
       </c>
       <c r="I165" s="43" t="n">
         <f aca="false">IF($B165="","",$I$160+SUM($G$162:$G165)-SUM($H$162:$H165))</f>
-        <v>3507.41</v>
+        <v>3670.91</v>
       </c>
       <c r="J165" s="44" t="str">
         <f aca="true">IF($B165="","",IF($F165&lt;&gt;"","PAID",IF($C165&lt;TODAY(),"PAST DUE",IF($C165&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6786,7 +6797,7 @@
       </c>
       <c r="I166" s="43" t="n">
         <f aca="false">IF($B166="","",$I$160+SUM($G$162:$G166)-SUM($H$162:$H166))</f>
-        <v>3157.41</v>
+        <v>3320.91</v>
       </c>
       <c r="J166" s="44" t="str">
         <f aca="true">IF($B166="","",IF($F166&lt;&gt;"","PAID",IF($C166&lt;TODAY(),"PAST DUE",IF($C166&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6821,7 +6832,7 @@
       </c>
       <c r="I167" s="43" t="n">
         <f aca="false">IF($B167="","",$I$160+SUM($G$162:$G167)-SUM($H$162:$H167))</f>
-        <v>3007.41</v>
+        <v>3170.91</v>
       </c>
       <c r="J167" s="44" t="str">
         <f aca="true">IF($B167="","",IF($F167&lt;&gt;"","PAID",IF($C167&lt;TODAY(),"PAST DUE",IF($C167&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6856,7 +6867,7 @@
       </c>
       <c r="I168" s="43" t="n">
         <f aca="false">IF($B168="","",$I$160+SUM($G$162:$G168)-SUM($H$162:$H168))</f>
-        <v>2864.04</v>
+        <v>3027.54</v>
       </c>
       <c r="J168" s="44" t="str">
         <f aca="true">IF($B168="","",IF($F168&lt;&gt;"","PAID",IF($C168&lt;TODAY(),"PAST DUE",IF($C168&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -6970,7 +6981,7 @@
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B172" s="45" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C172" s="46"/>
       <c r="D172" s="46"/>
@@ -7103,7 +7114,7 @@
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B179" s="47" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C179" s="48"/>
       <c r="D179" s="48"/>
@@ -7119,7 +7130,7 @@
       </c>
       <c r="I179" s="50" t="n">
         <f aca="false">$I$160+$G$179-$H$179</f>
-        <v>2864.04</v>
+        <v>3027.54</v>
       </c>
       <c r="J179" s="51" t="str">
         <f aca="false">IF($I$179&lt;0,"SHORTFALL",IF($I$179&lt;$E$7,"TIGHT","OK"))</f>
@@ -7140,12 +7151,12 @@
       <c r="E181" s="32"/>
       <c r="F181" s="32"/>
       <c r="G181" s="33" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H181" s="32"/>
       <c r="I181" s="34" t="n">
         <f aca="false">$I$179</f>
-        <v>2864.04</v>
+        <v>3027.54</v>
       </c>
       <c r="J181" s="32"/>
       <c r="K181" s="28" t="str">
@@ -7155,19 +7166,19 @@
     </row>
     <row r="182" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B182" s="35" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C182" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D182" s="35" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E182" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F182" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G182" s="36" t="s">
         <v>18</v>
@@ -7176,10 +7187,10 @@
         <v>20</v>
       </c>
       <c r="I182" s="35" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J182" s="35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7210,7 +7221,7 @@
       </c>
       <c r="I183" s="43" t="n">
         <f aca="false">IF($B183="","",$I$181+SUM($G$183:$G183)-SUM($H$183:$H183))</f>
-        <v>3654.04</v>
+        <v>3817.54</v>
       </c>
       <c r="J183" s="44" t="str">
         <f aca="true">IF($B183="","",IF($F183&lt;&gt;"","PAID",IF($C183&lt;TODAY(),"PAST DUE",IF($C183&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7245,7 +7256,7 @@
       </c>
       <c r="I184" s="43" t="n">
         <f aca="false">IF($B184="","",$I$181+SUM($G$183:$G184)-SUM($H$183:$H184))</f>
-        <v>3632.94</v>
+        <v>3796.44</v>
       </c>
       <c r="J184" s="44" t="str">
         <f aca="true">IF($B184="","",IF($F184&lt;&gt;"","PAID",IF($C184&lt;TODAY(),"PAST DUE",IF($C184&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7280,7 +7291,7 @@
       </c>
       <c r="I185" s="43" t="n">
         <f aca="false">IF($B185="","",$I$181+SUM($G$183:$G185)-SUM($H$183:$H185))</f>
-        <v>3612.94</v>
+        <v>3776.44</v>
       </c>
       <c r="J185" s="44" t="str">
         <f aca="true">IF($B185="","",IF($F185&lt;&gt;"","PAID",IF($C185&lt;TODAY(),"PAST DUE",IF($C185&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7315,7 +7326,7 @@
       </c>
       <c r="I186" s="43" t="n">
         <f aca="false">IF($B186="","",$I$181+SUM($G$183:$G186)-SUM($H$183:$H186))</f>
-        <v>3602.94</v>
+        <v>3766.44</v>
       </c>
       <c r="J186" s="44" t="str">
         <f aca="true">IF($B186="","",IF($F186&lt;&gt;"","PAID",IF($C186&lt;TODAY(),"PAST DUE",IF($C186&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7350,7 +7361,7 @@
       </c>
       <c r="I187" s="43" t="n">
         <f aca="false">IF($B187="","",$I$181+SUM($G$183:$G187)-SUM($H$183:$H187))</f>
-        <v>3692.94</v>
+        <v>3856.44</v>
       </c>
       <c r="J187" s="44" t="str">
         <f aca="true">IF($B187="","",IF($F187&lt;&gt;"","PAID",IF($C187&lt;TODAY(),"PAST DUE",IF($C187&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7385,7 +7396,7 @@
       </c>
       <c r="I188" s="43" t="n">
         <f aca="false">IF($B188="","",$I$181+SUM($G$183:$G188)-SUM($H$183:$H188))</f>
-        <v>3687.95</v>
+        <v>3851.45</v>
       </c>
       <c r="J188" s="44" t="str">
         <f aca="true">IF($B188="","",IF($F188&lt;&gt;"","PAID",IF($C188&lt;TODAY(),"PAST DUE",IF($C188&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7420,7 +7431,7 @@
       </c>
       <c r="I189" s="43" t="n">
         <f aca="false">IF($B189="","",$I$181+SUM($G$183:$G189)-SUM($H$183:$H189))</f>
-        <v>3187.95</v>
+        <v>3351.45</v>
       </c>
       <c r="J189" s="44" t="str">
         <f aca="true">IF($B189="","",IF($F189&lt;&gt;"","PAID",IF($C189&lt;TODAY(),"PAST DUE",IF($C189&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7534,7 +7545,7 @@
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B193" s="45" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C193" s="46"/>
       <c r="D193" s="46"/>
@@ -7667,7 +7678,7 @@
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B200" s="47" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C200" s="48"/>
       <c r="D200" s="48"/>
@@ -7683,7 +7694,7 @@
       </c>
       <c r="I200" s="50" t="n">
         <f aca="false">$I$181+$G$200-$H$200</f>
-        <v>3187.95</v>
+        <v>3351.45</v>
       </c>
       <c r="J200" s="51" t="str">
         <f aca="false">IF($I$200&lt;0,"SHORTFALL",IF($I$200&lt;$E$7,"TIGHT","OK"))</f>
@@ -7704,12 +7715,12 @@
       <c r="E202" s="32"/>
       <c r="F202" s="32"/>
       <c r="G202" s="33" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H202" s="32"/>
       <c r="I202" s="34" t="n">
         <f aca="false">$I$200</f>
-        <v>3187.95</v>
+        <v>3351.45</v>
       </c>
       <c r="J202" s="32"/>
       <c r="K202" s="28" t="str">
@@ -7719,19 +7730,19 @@
     </row>
     <row r="203" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B203" s="35" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C203" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D203" s="35" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E203" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F203" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G203" s="36" t="s">
         <v>18</v>
@@ -7740,10 +7751,10 @@
         <v>20</v>
       </c>
       <c r="I203" s="35" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J203" s="35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7774,7 +7785,7 @@
       </c>
       <c r="I204" s="43" t="n">
         <f aca="false">IF($B204="","",$I$202+SUM($G$204:$G204)-SUM($H$204:$H204))</f>
-        <v>3977.95</v>
+        <v>4141.45</v>
       </c>
       <c r="J204" s="44" t="str">
         <f aca="true">IF($B204="","",IF($F204&lt;&gt;"","PAID",IF($C204&lt;TODAY(),"PAST DUE",IF($C204&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7809,7 +7820,7 @@
       </c>
       <c r="I205" s="43" t="n">
         <f aca="false">IF($B205="","",$I$202+SUM($G$204:$G205)-SUM($H$204:$H205))</f>
-        <v>3814.45</v>
+        <v>3977.95</v>
       </c>
       <c r="J205" s="44" t="str">
         <f aca="true">IF($B205="","",IF($F205&lt;&gt;"","PAID",IF($C205&lt;TODAY(),"PAST DUE",IF($C205&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7844,7 +7855,7 @@
       </c>
       <c r="I206" s="43" t="n">
         <f aca="false">IF($B206="","",$I$202+SUM($G$204:$G206)-SUM($H$204:$H206))</f>
-        <v>3811.46</v>
+        <v>3974.96</v>
       </c>
       <c r="J206" s="44" t="str">
         <f aca="true">IF($B206="","",IF($F206&lt;&gt;"","PAID",IF($C206&lt;TODAY(),"PAST DUE",IF($C206&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7879,7 +7890,7 @@
       </c>
       <c r="I207" s="43" t="n">
         <f aca="false">IF($B207="","",$I$202+SUM($G$204:$G207)-SUM($H$204:$H207))</f>
-        <v>3901.46</v>
+        <v>4064.96</v>
       </c>
       <c r="J207" s="44" t="str">
         <f aca="true">IF($B207="","",IF($F207&lt;&gt;"","PAID",IF($C207&lt;TODAY(),"PAST DUE",IF($C207&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -7914,7 +7925,7 @@
       </c>
       <c r="I208" s="43" t="n">
         <f aca="false">IF($B208="","",$I$202+SUM($G$204:$G208)-SUM($H$204:$H208))</f>
-        <v>3551.46</v>
+        <v>3714.96</v>
       </c>
       <c r="J208" s="44" t="str">
         <f aca="true">IF($B208="","",IF($F208&lt;&gt;"","PAID",IF($C208&lt;TODAY(),"PAST DUE",IF($C208&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -8098,7 +8109,7 @@
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B214" s="45" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C214" s="46"/>
       <c r="D214" s="46"/>
@@ -8231,7 +8242,7 @@
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B221" s="47" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C221" s="48"/>
       <c r="D221" s="48"/>
@@ -8247,7 +8258,7 @@
       </c>
       <c r="I221" s="50" t="n">
         <f aca="false">$I$202+$G$221-$H$221</f>
-        <v>3551.46</v>
+        <v>3714.96</v>
       </c>
       <c r="J221" s="51" t="str">
         <f aca="false">IF($I$221&lt;0,"SHORTFALL",IF($I$221&lt;$E$7,"TIGHT","OK"))</f>
@@ -8268,12 +8279,12 @@
       <c r="E223" s="32"/>
       <c r="F223" s="32"/>
       <c r="G223" s="33" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H223" s="32"/>
       <c r="I223" s="34" t="n">
         <f aca="false">$I$221</f>
-        <v>3551.46</v>
+        <v>3714.96</v>
       </c>
       <c r="J223" s="32"/>
       <c r="K223" s="28" t="str">
@@ -8283,19 +8294,19 @@
     </row>
     <row r="224" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B224" s="35" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C224" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D224" s="35" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E224" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F224" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G224" s="36" t="s">
         <v>18</v>
@@ -8304,10 +8315,10 @@
         <v>20</v>
       </c>
       <c r="I224" s="35" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J224" s="35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8338,7 +8349,7 @@
       </c>
       <c r="I225" s="43" t="n">
         <f aca="false">IF($B225="","",$I$223+SUM($G$225:$G225)-SUM($H$225:$H225))</f>
-        <v>4341.46</v>
+        <v>4504.96</v>
       </c>
       <c r="J225" s="44" t="str">
         <f aca="true">IF($B225="","",IF($F225&lt;&gt;"","PAID",IF($C225&lt;TODAY(),"PAST DUE",IF($C225&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -8373,7 +8384,7 @@
       </c>
       <c r="I226" s="43" t="n">
         <f aca="false">IF($B226="","",$I$223+SUM($G$225:$G226)-SUM($H$225:$H226))</f>
-        <v>4170.36</v>
+        <v>4333.86</v>
       </c>
       <c r="J226" s="44" t="str">
         <f aca="true">IF($B226="","",IF($F226&lt;&gt;"","PAID",IF($C226&lt;TODAY(),"PAST DUE",IF($C226&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -8408,7 +8419,7 @@
       </c>
       <c r="I227" s="43" t="n">
         <f aca="false">IF($B227="","",$I$223+SUM($G$225:$G227)-SUM($H$225:$H227))</f>
-        <v>4125.36</v>
+        <v>4288.86</v>
       </c>
       <c r="J227" s="44" t="str">
         <f aca="true">IF($B227="","",IF($F227&lt;&gt;"","PAID",IF($C227&lt;TODAY(),"PAST DUE",IF($C227&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -8443,7 +8454,7 @@
       </c>
       <c r="I228" s="43" t="n">
         <f aca="false">IF($B228="","",$I$223+SUM($G$225:$G228)-SUM($H$225:$H228))</f>
-        <v>4108.37</v>
+        <v>4271.87</v>
       </c>
       <c r="J228" s="44" t="str">
         <f aca="true">IF($B228="","",IF($F228&lt;&gt;"","PAID",IF($C228&lt;TODAY(),"PAST DUE",IF($C228&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -8478,7 +8489,7 @@
       </c>
       <c r="I229" s="43" t="n">
         <f aca="false">IF($B229="","",$I$223+SUM($G$225:$G229)-SUM($H$225:$H229))</f>
-        <v>4198.37</v>
+        <v>4361.87</v>
       </c>
       <c r="J229" s="44" t="str">
         <f aca="true">IF($B229="","",IF($F229&lt;&gt;"","PAID",IF($C229&lt;TODAY(),"PAST DUE",IF($C229&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -8662,7 +8673,7 @@
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B235" s="45" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C235" s="46"/>
       <c r="D235" s="46"/>
@@ -8795,7 +8806,7 @@
     </row>
     <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B242" s="47" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C242" s="48"/>
       <c r="D242" s="48"/>
@@ -8811,7 +8822,7 @@
       </c>
       <c r="I242" s="50" t="n">
         <f aca="false">$I$223+$G$242-$H$242</f>
-        <v>4198.37</v>
+        <v>4361.87</v>
       </c>
       <c r="J242" s="51" t="str">
         <f aca="false">IF($I$242&lt;0,"SHORTFALL",IF($I$242&lt;$E$7,"TIGHT","OK"))</f>
@@ -8832,12 +8843,12 @@
       <c r="E244" s="32"/>
       <c r="F244" s="32"/>
       <c r="G244" s="33" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H244" s="32"/>
       <c r="I244" s="34" t="n">
         <f aca="false">$I$242</f>
-        <v>4198.37</v>
+        <v>4361.87</v>
       </c>
       <c r="J244" s="32"/>
       <c r="K244" s="28" t="str">
@@ -8847,19 +8858,19 @@
     </row>
     <row r="245" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B245" s="35" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C245" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D245" s="35" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E245" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F245" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G245" s="36" t="s">
         <v>18</v>
@@ -8868,10 +8879,10 @@
         <v>20</v>
       </c>
       <c r="I245" s="35" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J245" s="35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8902,7 +8913,7 @@
       </c>
       <c r="I246" s="43" t="n">
         <f aca="false">IF($B246="","",$I$244+SUM($G$246:$G246)-SUM($H$246:$H246))</f>
-        <v>4988.37</v>
+        <v>5151.87</v>
       </c>
       <c r="J246" s="44" t="str">
         <f aca="true">IF($B246="","",IF($F246&lt;&gt;"","PAID",IF($C246&lt;TODAY(),"PAST DUE",IF($C246&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -8937,7 +8948,7 @@
       </c>
       <c r="I247" s="43" t="n">
         <f aca="false">IF($B247="","",$I$244+SUM($G$246:$G247)-SUM($H$246:$H247))</f>
-        <v>4974.67</v>
+        <v>5138.17</v>
       </c>
       <c r="J247" s="44" t="str">
         <f aca="true">IF($B247="","",IF($F247&lt;&gt;"","PAID",IF($C247&lt;TODAY(),"PAST DUE",IF($C247&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -8947,7 +8958,7 @@
     <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B248" s="11" t="str">
         <f aca="false">IFERROR(INDEX(Schedule!$C$4:$C$483,MATCH(12003,Schedule!$K$4:$K$483,0)),"")</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="C248" s="38" t="n">
         <f aca="false">IF($B248="","",INDEX(Schedule!$G$4:$G$483,MATCH(12003,Schedule!$K$4:$K$483,0)))</f>
@@ -8972,7 +8983,7 @@
       </c>
       <c r="I248" s="43" t="n">
         <f aca="false">IF($B248="","",$I$244+SUM($G$246:$G248)-SUM($H$246:$H248))</f>
-        <v>4930.8</v>
+        <v>5094.3</v>
       </c>
       <c r="J248" s="44" t="str">
         <f aca="true">IF($B248="","",IF($F248&lt;&gt;"","PAID",IF($C248&lt;TODAY(),"PAST DUE",IF($C248&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9007,7 +9018,7 @@
       </c>
       <c r="I249" s="43" t="n">
         <f aca="false">IF($B249="","",$I$244+SUM($G$246:$G249)-SUM($H$246:$H249))</f>
-        <v>5020.8</v>
+        <v>5184.3</v>
       </c>
       <c r="J249" s="44" t="str">
         <f aca="true">IF($B249="","",IF($F249&lt;&gt;"","PAID",IF($C249&lt;TODAY(),"PAST DUE",IF($C249&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9226,7 +9237,7 @@
     </row>
     <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B256" s="45" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C256" s="46"/>
       <c r="D256" s="46"/>
@@ -9359,7 +9370,7 @@
     </row>
     <row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B263" s="47" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C263" s="48"/>
       <c r="D263" s="48"/>
@@ -9375,7 +9386,7 @@
       </c>
       <c r="I263" s="50" t="n">
         <f aca="false">$I$244+$G$263-$H$263</f>
-        <v>5020.8</v>
+        <v>5184.3</v>
       </c>
       <c r="J263" s="51" t="str">
         <f aca="false">IF($I$263&lt;0,"SHORTFALL",IF($I$263&lt;$E$7,"TIGHT","OK"))</f>
@@ -9396,12 +9407,12 @@
       <c r="E265" s="32"/>
       <c r="F265" s="32"/>
       <c r="G265" s="33" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H265" s="32"/>
       <c r="I265" s="34" t="n">
         <f aca="false">$I$263</f>
-        <v>5020.8</v>
+        <v>5184.3</v>
       </c>
       <c r="J265" s="32"/>
       <c r="K265" s="28" t="str">
@@ -9411,19 +9422,19 @@
     </row>
     <row r="266" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B266" s="35" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C266" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D266" s="35" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E266" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F266" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G266" s="36" t="s">
         <v>18</v>
@@ -9432,10 +9443,10 @@
         <v>20</v>
       </c>
       <c r="I266" s="35" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J266" s="35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="267" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9466,7 +9477,7 @@
       </c>
       <c r="I267" s="43" t="n">
         <f aca="false">IF($B267="","",$I$265+SUM($G$267:$G267)-SUM($H$267:$H267))</f>
-        <v>5810.8</v>
+        <v>5974.3</v>
       </c>
       <c r="J267" s="44" t="str">
         <f aca="true">IF($B267="","",IF($F267&lt;&gt;"","PAID",IF($C267&lt;TODAY(),"PAST DUE",IF($C267&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9501,7 +9512,7 @@
       </c>
       <c r="I268" s="43" t="n">
         <f aca="false">IF($B268="","",$I$265+SUM($G$267:$G268)-SUM($H$267:$H268))</f>
-        <v>5460.8</v>
+        <v>5624.3</v>
       </c>
       <c r="J268" s="44" t="str">
         <f aca="true">IF($B268="","",IF($F268&lt;&gt;"","PAID",IF($C268&lt;TODAY(),"PAST DUE",IF($C268&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9536,7 +9547,7 @@
       </c>
       <c r="I269" s="43" t="n">
         <f aca="false">IF($B269="","",$I$265+SUM($G$267:$G269)-SUM($H$267:$H269))</f>
-        <v>5310.8</v>
+        <v>5474.3</v>
       </c>
       <c r="J269" s="44" t="str">
         <f aca="true">IF($B269="","",IF($F269&lt;&gt;"","PAID",IF($C269&lt;TODAY(),"PAST DUE",IF($C269&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9571,7 +9582,7 @@
       </c>
       <c r="I270" s="43" t="n">
         <f aca="false">IF($B270="","",$I$265+SUM($G$267:$G270)-SUM($H$267:$H270))</f>
-        <v>5167.43</v>
+        <v>5330.93</v>
       </c>
       <c r="J270" s="44" t="str">
         <f aca="true">IF($B270="","",IF($F270&lt;&gt;"","PAID",IF($C270&lt;TODAY(),"PAST DUE",IF($C270&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9606,7 +9617,7 @@
       </c>
       <c r="I271" s="43" t="n">
         <f aca="false">IF($B271="","",$I$265+SUM($G$267:$G271)-SUM($H$267:$H271))</f>
-        <v>5257.43</v>
+        <v>5420.93</v>
       </c>
       <c r="J271" s="44" t="str">
         <f aca="true">IF($B271="","",IF($F271&lt;&gt;"","PAID",IF($C271&lt;TODAY(),"PAST DUE",IF($C271&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9641,7 +9652,7 @@
       </c>
       <c r="I272" s="43" t="n">
         <f aca="false">IF($B272="","",$I$265+SUM($G$267:$G272)-SUM($H$267:$H272))</f>
-        <v>5236.33</v>
+        <v>5399.83</v>
       </c>
       <c r="J272" s="44" t="str">
         <f aca="true">IF($B272="","",IF($F272&lt;&gt;"","PAID",IF($C272&lt;TODAY(),"PAST DUE",IF($C272&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9676,7 +9687,7 @@
       </c>
       <c r="I273" s="43" t="n">
         <f aca="false">IF($B273="","",$I$265+SUM($G$267:$G273)-SUM($H$267:$H273))</f>
-        <v>5216.33</v>
+        <v>5379.83</v>
       </c>
       <c r="J273" s="44" t="str">
         <f aca="true">IF($B273="","",IF($F273&lt;&gt;"","PAID",IF($C273&lt;TODAY(),"PAST DUE",IF($C273&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9711,7 +9722,7 @@
       </c>
       <c r="I274" s="43" t="n">
         <f aca="false">IF($B274="","",$I$265+SUM($G$267:$G274)-SUM($H$267:$H274))</f>
-        <v>5206.33</v>
+        <v>5369.83</v>
       </c>
       <c r="J274" s="44" t="str">
         <f aca="true">IF($B274="","",IF($F274&lt;&gt;"","PAID",IF($C274&lt;TODAY(),"PAST DUE",IF($C274&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
@@ -9790,7 +9801,7 @@
     </row>
     <row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B277" s="45" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C277" s="46"/>
       <c r="D277" s="46"/>
@@ -9923,7 +9934,7 @@
     </row>
     <row r="284" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B284" s="47" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C284" s="48"/>
       <c r="D284" s="48"/>
@@ -9939,7 +9950,7 @@
       </c>
       <c r="I284" s="50" t="n">
         <f aca="false">$I$265+$G$284-$H$284</f>
-        <v>5206.33</v>
+        <v>5369.83</v>
       </c>
       <c r="J284" s="51" t="str">
         <f aca="false">IF($I$284&lt;0,"SHORTFALL",IF($I$284&lt;$E$7,"TIGHT","OK"))</f>
@@ -10004,28 +10015,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="52" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C4" s="52"/>
       <c r="D4" s="52"/>
       <c r="E4" s="53" t="n">
         <f aca="false">MIN($I$13:$I$25)</f>
-        <v>-5.31999999999999</v>
+        <v>158.18</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="52" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C5" s="52"/>
       <c r="D5" s="52"/>
@@ -10040,13 +10051,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="52" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C6" s="52"/>
       <c r="D6" s="52"/>
       <c r="E6" s="54" t="str">
         <f aca="false">IF(MIN($K$13:$K$25)=999,"None — you stay above zero all 13 weeks","Week "&amp;MIN($K$13:$K$25)&amp;"  ("&amp;TEXT(INDEX($C$13:$C$25,MATCH(MIN($K$13:$K$25),$B$13:$B$25,0)),"mmm d, yyyy")&amp;")")</f>
-        <v>Week 1  (Aug 7, 2026)</v>
+        <v>None — you stay above zero all 13 weeks</v>
       </c>
       <c r="F6" s="54"/>
       <c r="G6" s="54"/>
@@ -10055,7 +10066,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="52" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C7" s="52"/>
       <c r="D7" s="52"/>
@@ -10066,67 +10077,67 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="52" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C8" s="52"/>
       <c r="D8" s="52"/>
       <c r="E8" s="55" t="n">
         <f aca="false">SUM($F$13:$F$25)+SUM($G$13:$G$25)</f>
-        <v>5514.84</v>
+        <v>5351.34</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="52" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C9" s="52"/>
       <c r="D9" s="52"/>
       <c r="E9" s="53" t="n">
         <f aca="false">SUM($H$13:$H$25)</f>
-        <v>5135.16</v>
+        <v>5298.66</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="52" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C10" s="52"/>
       <c r="D10" s="52"/>
       <c r="E10" s="53" t="n">
         <f aca="false">$I$25</f>
-        <v>5206.33</v>
+        <v>5369.83</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="15" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I12" s="15" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J12" s="15" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K12" s="15" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10147,7 +10158,7 @@
       </c>
       <c r="F13" s="58" t="n">
         <f aca="false">SUM('Cash Flow'!$H$15:$H$24)</f>
-        <v>166.49</v>
+        <v>2.99</v>
       </c>
       <c r="G13" s="58" t="n">
         <f aca="false">SUM('Cash Flow'!$H$26:$H$31)</f>
@@ -10155,19 +10166,19 @@
       </c>
       <c r="H13" s="59" t="n">
         <f aca="false">$E13-$F13-$G13</f>
-        <v>-76.49</v>
+        <v>87.01</v>
       </c>
       <c r="I13" s="59" t="n">
         <f aca="false">'Cash Flow'!$I$32</f>
-        <v>-5.31999999999999</v>
+        <v>158.18</v>
       </c>
       <c r="J13" s="60" t="str">
         <f aca="false">IF($I13&lt;0,"SHORTFALL",IF($I13&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
-        <v>SHORTFALL</v>
+        <v>TIGHT</v>
       </c>
       <c r="K13" s="29" t="n">
         <f aca="false">IF($I13&lt;0,$B13,999)</f>
-        <v>1</v>
+        <v>999</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10180,7 +10191,7 @@
       </c>
       <c r="D14" s="62" t="n">
         <f aca="false">'Cash Flow'!$I$34</f>
-        <v>-5.31999999999999</v>
+        <v>158.18</v>
       </c>
       <c r="E14" s="63" t="n">
         <f aca="false">SUM('Cash Flow'!$G$36:$G$52)</f>
@@ -10200,7 +10211,7 @@
       </c>
       <c r="I14" s="64" t="n">
         <f aca="false">'Cash Flow'!$I$53</f>
-        <v>291.59</v>
+        <v>455.09</v>
       </c>
       <c r="J14" s="65" t="str">
         <f aca="false">IF($I14&lt;0,"SHORTFALL",IF($I14&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10221,7 +10232,7 @@
       </c>
       <c r="D15" s="57" t="n">
         <f aca="false">'Cash Flow'!$I$55</f>
-        <v>291.59</v>
+        <v>455.09</v>
       </c>
       <c r="E15" s="58" t="n">
         <f aca="false">SUM('Cash Flow'!$G$57:$G$73)</f>
@@ -10241,7 +10252,7 @@
       </c>
       <c r="I15" s="59" t="n">
         <f aca="false">'Cash Flow'!$I$74</f>
-        <v>1114.02</v>
+        <v>1277.52</v>
       </c>
       <c r="J15" s="60" t="str">
         <f aca="false">IF($I15&lt;0,"SHORTFALL",IF($I15&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10262,7 +10273,7 @@
       </c>
       <c r="D16" s="62" t="n">
         <f aca="false">'Cash Flow'!$I$76</f>
-        <v>1114.02</v>
+        <v>1277.52</v>
       </c>
       <c r="E16" s="63" t="n">
         <f aca="false">SUM('Cash Flow'!$G$78:$G$94)</f>
@@ -10282,7 +10293,7 @@
       </c>
       <c r="I16" s="64" t="n">
         <f aca="false">'Cash Flow'!$I$95</f>
-        <v>1350.65</v>
+        <v>1514.15</v>
       </c>
       <c r="J16" s="65" t="str">
         <f aca="false">IF($I16&lt;0,"SHORTFALL",IF($I16&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10303,7 +10314,7 @@
       </c>
       <c r="D17" s="57" t="n">
         <f aca="false">'Cash Flow'!$I$97</f>
-        <v>1350.65</v>
+        <v>1514.15</v>
       </c>
       <c r="E17" s="58" t="n">
         <f aca="false">SUM('Cash Flow'!$G$99:$G$115)</f>
@@ -10323,7 +10334,7 @@
       </c>
       <c r="I17" s="59" t="n">
         <f aca="false">'Cash Flow'!$I$116</f>
-        <v>1511.06</v>
+        <v>1674.56</v>
       </c>
       <c r="J17" s="60" t="str">
         <f aca="false">IF($I17&lt;0,"SHORTFALL",IF($I17&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10344,7 +10355,7 @@
       </c>
       <c r="D18" s="62" t="n">
         <f aca="false">'Cash Flow'!$I$118</f>
-        <v>1511.06</v>
+        <v>1674.56</v>
       </c>
       <c r="E18" s="63" t="n">
         <f aca="false">SUM('Cash Flow'!$G$120:$G$136)</f>
@@ -10364,7 +10375,7 @@
       </c>
       <c r="I18" s="64" t="n">
         <f aca="false">'Cash Flow'!$I$137</f>
-        <v>1821.97</v>
+        <v>1985.47</v>
       </c>
       <c r="J18" s="65" t="str">
         <f aca="false">IF($I18&lt;0,"SHORTFALL",IF($I18&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10385,7 +10396,7 @@
       </c>
       <c r="D19" s="57" t="n">
         <f aca="false">'Cash Flow'!$I$139</f>
-        <v>1821.97</v>
+        <v>1985.47</v>
       </c>
       <c r="E19" s="58" t="n">
         <f aca="false">SUM('Cash Flow'!$G$141:$G$157)</f>
@@ -10405,7 +10416,7 @@
       </c>
       <c r="I19" s="59" t="n">
         <f aca="false">'Cash Flow'!$I$158</f>
-        <v>2684.98</v>
+        <v>2848.48</v>
       </c>
       <c r="J19" s="60" t="str">
         <f aca="false">IF($I19&lt;0,"SHORTFALL",IF($I19&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10426,7 +10437,7 @@
       </c>
       <c r="D20" s="62" t="n">
         <f aca="false">'Cash Flow'!$I$160</f>
-        <v>2684.98</v>
+        <v>2848.48</v>
       </c>
       <c r="E20" s="63" t="n">
         <f aca="false">SUM('Cash Flow'!$G$162:$G$178)</f>
@@ -10446,7 +10457,7 @@
       </c>
       <c r="I20" s="64" t="n">
         <f aca="false">'Cash Flow'!$I$179</f>
-        <v>2864.04</v>
+        <v>3027.54</v>
       </c>
       <c r="J20" s="65" t="str">
         <f aca="false">IF($I20&lt;0,"SHORTFALL",IF($I20&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10467,7 +10478,7 @@
       </c>
       <c r="D21" s="57" t="n">
         <f aca="false">'Cash Flow'!$I$181</f>
-        <v>2864.04</v>
+        <v>3027.54</v>
       </c>
       <c r="E21" s="58" t="n">
         <f aca="false">SUM('Cash Flow'!$G$183:$G$199)</f>
@@ -10487,7 +10498,7 @@
       </c>
       <c r="I21" s="59" t="n">
         <f aca="false">'Cash Flow'!$I$200</f>
-        <v>3187.95</v>
+        <v>3351.45</v>
       </c>
       <c r="J21" s="60" t="str">
         <f aca="false">IF($I21&lt;0,"SHORTFALL",IF($I21&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10508,7 +10519,7 @@
       </c>
       <c r="D22" s="62" t="n">
         <f aca="false">'Cash Flow'!$I$202</f>
-        <v>3187.95</v>
+        <v>3351.45</v>
       </c>
       <c r="E22" s="63" t="n">
         <f aca="false">SUM('Cash Flow'!$G$204:$G$220)</f>
@@ -10528,7 +10539,7 @@
       </c>
       <c r="I22" s="64" t="n">
         <f aca="false">'Cash Flow'!$I$221</f>
-        <v>3551.46</v>
+        <v>3714.96</v>
       </c>
       <c r="J22" s="65" t="str">
         <f aca="false">IF($I22&lt;0,"SHORTFALL",IF($I22&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10549,7 +10560,7 @@
       </c>
       <c r="D23" s="57" t="n">
         <f aca="false">'Cash Flow'!$I$223</f>
-        <v>3551.46</v>
+        <v>3714.96</v>
       </c>
       <c r="E23" s="58" t="n">
         <f aca="false">SUM('Cash Flow'!$G$225:$G$241)</f>
@@ -10569,7 +10580,7 @@
       </c>
       <c r="I23" s="59" t="n">
         <f aca="false">'Cash Flow'!$I$242</f>
-        <v>4198.37</v>
+        <v>4361.87</v>
       </c>
       <c r="J23" s="60" t="str">
         <f aca="false">IF($I23&lt;0,"SHORTFALL",IF($I23&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10590,7 +10601,7 @@
       </c>
       <c r="D24" s="62" t="n">
         <f aca="false">'Cash Flow'!$I$244</f>
-        <v>4198.37</v>
+        <v>4361.87</v>
       </c>
       <c r="E24" s="63" t="n">
         <f aca="false">SUM('Cash Flow'!$G$246:$G$262)</f>
@@ -10610,7 +10621,7 @@
       </c>
       <c r="I24" s="64" t="n">
         <f aca="false">'Cash Flow'!$I$263</f>
-        <v>5020.8</v>
+        <v>5184.3</v>
       </c>
       <c r="J24" s="65" t="str">
         <f aca="false">IF($I24&lt;0,"SHORTFALL",IF($I24&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10631,7 +10642,7 @@
       </c>
       <c r="D25" s="57" t="n">
         <f aca="false">'Cash Flow'!$I$265</f>
-        <v>5020.8</v>
+        <v>5184.3</v>
       </c>
       <c r="E25" s="58" t="n">
         <f aca="false">SUM('Cash Flow'!$G$267:$G$283)</f>
@@ -10651,7 +10662,7 @@
       </c>
       <c r="I25" s="59" t="n">
         <f aca="false">'Cash Flow'!$I$284</f>
-        <v>5206.33</v>
+        <v>5369.83</v>
       </c>
       <c r="J25" s="60" t="str">
         <f aca="false">IF($I25&lt;0,"SHORTFALL",IF($I25&lt;'Cash Flow'!$E$7,"TIGHT","OK"))</f>
@@ -10664,10 +10675,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="51" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C26" s="66" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D26" s="67" t="n">
         <f aca="false">$D$13</f>
@@ -10679,7 +10690,7 @@
       </c>
       <c r="F26" s="49" t="n">
         <f aca="false">SUM($F$13:$F$25)</f>
-        <v>5514.84</v>
+        <v>5351.34</v>
       </c>
       <c r="G26" s="49" t="n">
         <f aca="false">SUM($G$13:$G$25)</f>
@@ -10687,17 +10698,17 @@
       </c>
       <c r="H26" s="67" t="n">
         <f aca="false">SUM($H$13:$H$25)</f>
-        <v>5135.16</v>
+        <v>5298.66</v>
       </c>
       <c r="I26" s="67" t="n">
         <f aca="false">$I$25</f>
-        <v>5206.33</v>
+        <v>5369.83</v>
       </c>
       <c r="J26" s="48"/>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="68" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C28" s="68"/>
       <c r="D28" s="68"/>
@@ -10767,47 +10778,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="69" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="70" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B3" s="70" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C3" s="70" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D3" s="70" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E3" s="70" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F3" s="70" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G3" s="70" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H3" s="70" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I3" s="70" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J3" s="70" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K3" s="70" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10851,7 +10862,7 @@
       </c>
       <c r="K4" s="72" t="n">
         <f aca="false">IF($H4=1,$I4*1000+COUNTIFS($I$4:$I$483,$I4,$J$4:$J$483,"&lt;"&amp;$J4)+1,"")</f>
-        <v>1002</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15759,11 +15770,11 @@
       </c>
       <c r="F116" s="74" t="n">
         <f aca="false">IF($C116="","",IF(Recurring!$E$12="Weekly",Recurring!$F$12+7*0,IF(Recurring!$E$12="Every 2 Weeks",Recurring!$F$12+14*0,IF(Recurring!$E$12="Monthly",EDATE(Recurring!$F$12,0),IF(Recurring!$E$12="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+0),2)=1,EOMONTH(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+0)/2)),DATE(YEAR(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+0)/2))),MONTH(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+0)/2))),15)),IF(Recurring!$E$12="One Time",IF(1=1,Recurring!$F$12,""),""))))))</f>
-        <v>46244</v>
+        <v>46275</v>
       </c>
       <c r="G116" s="74" t="n">
         <f aca="false">IF($F116="","",IF(Recurring!$G$12="Move Before",IF(WEEKDAY($F116,2)=6,$F116-1,IF(WEEKDAY($F116,2)=7,$F116-2,$F116)),IF(Recurring!$G$12="Move After",IF(WEEKDAY($F116,2)=6,$F116+2,IF(WEEKDAY($F116,2)=7,$F116+1,$F116)),$F116)))</f>
-        <v>46244</v>
+        <v>46275</v>
       </c>
       <c r="H116" s="75" t="n">
         <f aca="false">IF($G116="",0,IF(AND($G116&gt;='Cash Flow'!$E$6,$G116&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15771,15 +15782,15 @@
       </c>
       <c r="I116" s="75" t="n">
         <f aca="false">IF($H116=1,INT(($G116-'Cash Flow'!$E$6)/7)+1,"")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J116" s="72" t="n">
         <f aca="false">IF($H116=1,$G116*10000+ROW(),"")</f>
-        <v>462440116</v>
+        <v>462750116</v>
       </c>
       <c r="K116" s="72" t="n">
         <f aca="false">IF($H116=1,$I116*1000+COUNTIFS($I$4:$I$483,$I116,$J$4:$J$483,"&lt;"&amp;$J116)+1,"")</f>
-        <v>1001</v>
+        <v>5008</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15803,11 +15814,11 @@
       </c>
       <c r="F117" s="74" t="n">
         <f aca="false">IF($C117="","",IF(Recurring!$E$12="Weekly",Recurring!$F$12+7*1,IF(Recurring!$E$12="Every 2 Weeks",Recurring!$F$12+14*1,IF(Recurring!$E$12="Monthly",EDATE(Recurring!$F$12,1),IF(Recurring!$E$12="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+1),2)=1,EOMONTH(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+1)/2)),DATE(YEAR(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+1)/2))),MONTH(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+1)/2))),15)),IF(Recurring!$E$12="One Time",IF(2=1,Recurring!$F$12,""),""))))))</f>
-        <v>46275</v>
+        <v>46305</v>
       </c>
       <c r="G117" s="74" t="n">
         <f aca="false">IF($F117="","",IF(Recurring!$G$12="Move Before",IF(WEEKDAY($F117,2)=6,$F117-1,IF(WEEKDAY($F117,2)=7,$F117-2,$F117)),IF(Recurring!$G$12="Move After",IF(WEEKDAY($F117,2)=6,$F117+2,IF(WEEKDAY($F117,2)=7,$F117+1,$F117)),$F117)))</f>
-        <v>46275</v>
+        <v>46305</v>
       </c>
       <c r="H117" s="75" t="n">
         <f aca="false">IF($G117="",0,IF(AND($G117&gt;='Cash Flow'!$E$6,$G117&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15815,15 +15826,15 @@
       </c>
       <c r="I117" s="75" t="n">
         <f aca="false">IF($H117=1,INT(($G117-'Cash Flow'!$E$6)/7)+1,"")</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J117" s="72" t="n">
         <f aca="false">IF($H117=1,$G117*10000+ROW(),"")</f>
-        <v>462750117</v>
+        <v>463050117</v>
       </c>
       <c r="K117" s="72" t="n">
         <f aca="false">IF($H117=1,$I117*1000+COUNTIFS($I$4:$I$483,$I117,$J$4:$J$483,"&lt;"&amp;$J117)+1,"")</f>
-        <v>5008</v>
+        <v>10002</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15847,27 +15858,27 @@
       </c>
       <c r="F118" s="74" t="n">
         <f aca="false">IF($C118="","",IF(Recurring!$E$12="Weekly",Recurring!$F$12+7*2,IF(Recurring!$E$12="Every 2 Weeks",Recurring!$F$12+14*2,IF(Recurring!$E$12="Monthly",EDATE(Recurring!$F$12,2),IF(Recurring!$E$12="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+2),2)=1,EOMONTH(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+2)/2)),DATE(YEAR(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+2)/2))),MONTH(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+2)/2))),15)),IF(Recurring!$E$12="One Time",IF(3=1,Recurring!$F$12,""),""))))))</f>
-        <v>46305</v>
+        <v>46336</v>
       </c>
       <c r="G118" s="74" t="n">
         <f aca="false">IF($F118="","",IF(Recurring!$G$12="Move Before",IF(WEEKDAY($F118,2)=6,$F118-1,IF(WEEKDAY($F118,2)=7,$F118-2,$F118)),IF(Recurring!$G$12="Move After",IF(WEEKDAY($F118,2)=6,$F118+2,IF(WEEKDAY($F118,2)=7,$F118+1,$F118)),$F118)))</f>
-        <v>46305</v>
+        <v>46336</v>
       </c>
       <c r="H118" s="75" t="n">
         <f aca="false">IF($G118="",0,IF(AND($G118&gt;='Cash Flow'!$E$6,$G118&lt;'Cash Flow'!$E$6+91),1,0))</f>
-        <v>1</v>
-      </c>
-      <c r="I118" s="75" t="n">
+        <v>0</v>
+      </c>
+      <c r="I118" s="75" t="str">
         <f aca="false">IF($H118=1,INT(($G118-'Cash Flow'!$E$6)/7)+1,"")</f>
-        <v>10</v>
-      </c>
-      <c r="J118" s="72" t="n">
+        <v/>
+      </c>
+      <c r="J118" s="72" t="str">
         <f aca="false">IF($H118=1,$G118*10000+ROW(),"")</f>
-        <v>463050118</v>
-      </c>
-      <c r="K118" s="72" t="n">
+        <v/>
+      </c>
+      <c r="K118" s="72" t="str">
         <f aca="false">IF($H118=1,$I118*1000+COUNTIFS($I$4:$I$483,$I118,$J$4:$J$483,"&lt;"&amp;$J118)+1,"")</f>
-        <v>10002</v>
+        <v/>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15891,11 +15902,11 @@
       </c>
       <c r="F119" s="74" t="n">
         <f aca="false">IF($C119="","",IF(Recurring!$E$12="Weekly",Recurring!$F$12+7*3,IF(Recurring!$E$12="Every 2 Weeks",Recurring!$F$12+14*3,IF(Recurring!$E$12="Monthly",EDATE(Recurring!$F$12,3),IF(Recurring!$E$12="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+3),2)=1,EOMONTH(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+3)/2)),DATE(YEAR(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+3)/2))),MONTH(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+3)/2))),15)),IF(Recurring!$E$12="One Time",IF(4=1,Recurring!$F$12,""),""))))))</f>
-        <v>46336</v>
+        <v>46366</v>
       </c>
       <c r="G119" s="74" t="n">
         <f aca="false">IF($F119="","",IF(Recurring!$G$12="Move Before",IF(WEEKDAY($F119,2)=6,$F119-1,IF(WEEKDAY($F119,2)=7,$F119-2,$F119)),IF(Recurring!$G$12="Move After",IF(WEEKDAY($F119,2)=6,$F119+2,IF(WEEKDAY($F119,2)=7,$F119+1,$F119)),$F119)))</f>
-        <v>46336</v>
+        <v>46366</v>
       </c>
       <c r="H119" s="75" t="n">
         <f aca="false">IF($G119="",0,IF(AND($G119&gt;='Cash Flow'!$E$6,$G119&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15935,11 +15946,11 @@
       </c>
       <c r="F120" s="74" t="n">
         <f aca="false">IF($C120="","",IF(Recurring!$E$12="Weekly",Recurring!$F$12+7*4,IF(Recurring!$E$12="Every 2 Weeks",Recurring!$F$12+14*4,IF(Recurring!$E$12="Monthly",EDATE(Recurring!$F$12,4),IF(Recurring!$E$12="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+4),2)=1,EOMONTH(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+4)/2)),DATE(YEAR(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+4)/2))),MONTH(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+4)/2))),15)),IF(Recurring!$E$12="One Time",IF(5=1,Recurring!$F$12,""),""))))))</f>
-        <v>46366</v>
+        <v>46397</v>
       </c>
       <c r="G120" s="74" t="n">
         <f aca="false">IF($F120="","",IF(Recurring!$G$12="Move Before",IF(WEEKDAY($F120,2)=6,$F120-1,IF(WEEKDAY($F120,2)=7,$F120-2,$F120)),IF(Recurring!$G$12="Move After",IF(WEEKDAY($F120,2)=6,$F120+2,IF(WEEKDAY($F120,2)=7,$F120+1,$F120)),$F120)))</f>
-        <v>46366</v>
+        <v>46397</v>
       </c>
       <c r="H120" s="75" t="n">
         <f aca="false">IF($G120="",0,IF(AND($G120&gt;='Cash Flow'!$E$6,$G120&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -15979,11 +15990,11 @@
       </c>
       <c r="F121" s="74" t="n">
         <f aca="false">IF($C121="","",IF(Recurring!$E$12="Weekly",Recurring!$F$12+7*5,IF(Recurring!$E$12="Every 2 Weeks",Recurring!$F$12+14*5,IF(Recurring!$E$12="Monthly",EDATE(Recurring!$F$12,5),IF(Recurring!$E$12="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+5),2)=1,EOMONTH(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+5)/2)),DATE(YEAR(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+5)/2))),MONTH(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+5)/2))),15)),IF(Recurring!$E$12="One Time",IF(6=1,Recurring!$F$12,""),""))))))</f>
-        <v>46397</v>
+        <v>46428</v>
       </c>
       <c r="G121" s="74" t="n">
         <f aca="false">IF($F121="","",IF(Recurring!$G$12="Move Before",IF(WEEKDAY($F121,2)=6,$F121-1,IF(WEEKDAY($F121,2)=7,$F121-2,$F121)),IF(Recurring!$G$12="Move After",IF(WEEKDAY($F121,2)=6,$F121+2,IF(WEEKDAY($F121,2)=7,$F121+1,$F121)),$F121)))</f>
-        <v>46397</v>
+        <v>46428</v>
       </c>
       <c r="H121" s="75" t="n">
         <f aca="false">IF($G121="",0,IF(AND($G121&gt;='Cash Flow'!$E$6,$G121&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -16023,11 +16034,11 @@
       </c>
       <c r="F122" s="74" t="n">
         <f aca="false">IF($C122="","",IF(Recurring!$E$12="Weekly",Recurring!$F$12+7*6,IF(Recurring!$E$12="Every 2 Weeks",Recurring!$F$12+14*6,IF(Recurring!$E$12="Monthly",EDATE(Recurring!$F$12,6),IF(Recurring!$E$12="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+6),2)=1,EOMONTH(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+6)/2)),DATE(YEAR(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+6)/2))),MONTH(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+6)/2))),15)),IF(Recurring!$E$12="One Time",IF(7=1,Recurring!$F$12,""),""))))))</f>
-        <v>46428</v>
+        <v>46456</v>
       </c>
       <c r="G122" s="74" t="n">
         <f aca="false">IF($F122="","",IF(Recurring!$G$12="Move Before",IF(WEEKDAY($F122,2)=6,$F122-1,IF(WEEKDAY($F122,2)=7,$F122-2,$F122)),IF(Recurring!$G$12="Move After",IF(WEEKDAY($F122,2)=6,$F122+2,IF(WEEKDAY($F122,2)=7,$F122+1,$F122)),$F122)))</f>
-        <v>46428</v>
+        <v>46456</v>
       </c>
       <c r="H122" s="75" t="n">
         <f aca="false">IF($G122="",0,IF(AND($G122&gt;='Cash Flow'!$E$6,$G122&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -16067,11 +16078,11 @@
       </c>
       <c r="F123" s="74" t="n">
         <f aca="false">IF($C123="","",IF(Recurring!$E$12="Weekly",Recurring!$F$12+7*7,IF(Recurring!$E$12="Every 2 Weeks",Recurring!$F$12+14*7,IF(Recurring!$E$12="Monthly",EDATE(Recurring!$F$12,7),IF(Recurring!$E$12="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+7),2)=1,EOMONTH(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+7)/2)),DATE(YEAR(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+7)/2))),MONTH(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+7)/2))),15)),IF(Recurring!$E$12="One Time",IF(8=1,Recurring!$F$12,""),""))))))</f>
-        <v>46456</v>
+        <v>46487</v>
       </c>
       <c r="G123" s="74" t="n">
         <f aca="false">IF($F123="","",IF(Recurring!$G$12="Move Before",IF(WEEKDAY($F123,2)=6,$F123-1,IF(WEEKDAY($F123,2)=7,$F123-2,$F123)),IF(Recurring!$G$12="Move After",IF(WEEKDAY($F123,2)=6,$F123+2,IF(WEEKDAY($F123,2)=7,$F123+1,$F123)),$F123)))</f>
-        <v>46456</v>
+        <v>46487</v>
       </c>
       <c r="H123" s="75" t="n">
         <f aca="false">IF($G123="",0,IF(AND($G123&gt;='Cash Flow'!$E$6,$G123&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -16111,11 +16122,11 @@
       </c>
       <c r="F124" s="74" t="n">
         <f aca="false">IF($C124="","",IF(Recurring!$E$12="Weekly",Recurring!$F$12+7*8,IF(Recurring!$E$12="Every 2 Weeks",Recurring!$F$12+14*8,IF(Recurring!$E$12="Monthly",EDATE(Recurring!$F$12,8),IF(Recurring!$E$12="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+8),2)=1,EOMONTH(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+8)/2)),DATE(YEAR(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+8)/2))),MONTH(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+8)/2))),15)),IF(Recurring!$E$12="One Time",IF(9=1,Recurring!$F$12,""),""))))))</f>
-        <v>46487</v>
+        <v>46517</v>
       </c>
       <c r="G124" s="74" t="n">
         <f aca="false">IF($F124="","",IF(Recurring!$G$12="Move Before",IF(WEEKDAY($F124,2)=6,$F124-1,IF(WEEKDAY($F124,2)=7,$F124-2,$F124)),IF(Recurring!$G$12="Move After",IF(WEEKDAY($F124,2)=6,$F124+2,IF(WEEKDAY($F124,2)=7,$F124+1,$F124)),$F124)))</f>
-        <v>46487</v>
+        <v>46517</v>
       </c>
       <c r="H124" s="75" t="n">
         <f aca="false">IF($G124="",0,IF(AND($G124&gt;='Cash Flow'!$E$6,$G124&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -16155,11 +16166,11 @@
       </c>
       <c r="F125" s="74" t="n">
         <f aca="false">IF($C125="","",IF(Recurring!$E$12="Weekly",Recurring!$F$12+7*9,IF(Recurring!$E$12="Every 2 Weeks",Recurring!$F$12+14*9,IF(Recurring!$E$12="Monthly",EDATE(Recurring!$F$12,9),IF(Recurring!$E$12="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+9),2)=1,EOMONTH(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+9)/2)),DATE(YEAR(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+9)/2))),MONTH(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+9)/2))),15)),IF(Recurring!$E$12="One Time",IF(10=1,Recurring!$F$12,""),""))))))</f>
-        <v>46517</v>
+        <v>46548</v>
       </c>
       <c r="G125" s="74" t="n">
         <f aca="false">IF($F125="","",IF(Recurring!$G$12="Move Before",IF(WEEKDAY($F125,2)=6,$F125-1,IF(WEEKDAY($F125,2)=7,$F125-2,$F125)),IF(Recurring!$G$12="Move After",IF(WEEKDAY($F125,2)=6,$F125+2,IF(WEEKDAY($F125,2)=7,$F125+1,$F125)),$F125)))</f>
-        <v>46517</v>
+        <v>46548</v>
       </c>
       <c r="H125" s="75" t="n">
         <f aca="false">IF($G125="",0,IF(AND($G125&gt;='Cash Flow'!$E$6,$G125&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -16199,11 +16210,11 @@
       </c>
       <c r="F126" s="74" t="n">
         <f aca="false">IF($C126="","",IF(Recurring!$E$12="Weekly",Recurring!$F$12+7*10,IF(Recurring!$E$12="Every 2 Weeks",Recurring!$F$12+14*10,IF(Recurring!$E$12="Monthly",EDATE(Recurring!$F$12,10),IF(Recurring!$E$12="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+10),2)=1,EOMONTH(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+10)/2)),DATE(YEAR(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+10)/2))),MONTH(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+10)/2))),15)),IF(Recurring!$E$12="One Time",IF(11=1,Recurring!$F$12,""),""))))))</f>
-        <v>46548</v>
+        <v>46578</v>
       </c>
       <c r="G126" s="74" t="n">
         <f aca="false">IF($F126="","",IF(Recurring!$G$12="Move Before",IF(WEEKDAY($F126,2)=6,$F126-1,IF(WEEKDAY($F126,2)=7,$F126-2,$F126)),IF(Recurring!$G$12="Move After",IF(WEEKDAY($F126,2)=6,$F126+2,IF(WEEKDAY($F126,2)=7,$F126+1,$F126)),$F126)))</f>
-        <v>46548</v>
+        <v>46578</v>
       </c>
       <c r="H126" s="75" t="n">
         <f aca="false">IF($G126="",0,IF(AND($G126&gt;='Cash Flow'!$E$6,$G126&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -16243,11 +16254,11 @@
       </c>
       <c r="F127" s="74" t="n">
         <f aca="false">IF($C127="","",IF(Recurring!$E$12="Weekly",Recurring!$F$12+7*11,IF(Recurring!$E$12="Every 2 Weeks",Recurring!$F$12+14*11,IF(Recurring!$E$12="Monthly",EDATE(Recurring!$F$12,11),IF(Recurring!$E$12="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+11),2)=1,EOMONTH(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+11)/2)),DATE(YEAR(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+11)/2))),MONTH(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+11)/2))),15)),IF(Recurring!$E$12="One Time",IF(12=1,Recurring!$F$12,""),""))))))</f>
-        <v>46578</v>
+        <v>46609</v>
       </c>
       <c r="G127" s="74" t="n">
         <f aca="false">IF($F127="","",IF(Recurring!$G$12="Move Before",IF(WEEKDAY($F127,2)=6,$F127-1,IF(WEEKDAY($F127,2)=7,$F127-2,$F127)),IF(Recurring!$G$12="Move After",IF(WEEKDAY($F127,2)=6,$F127+2,IF(WEEKDAY($F127,2)=7,$F127+1,$F127)),$F127)))</f>
-        <v>46578</v>
+        <v>46609</v>
       </c>
       <c r="H127" s="75" t="n">
         <f aca="false">IF($G127="",0,IF(AND($G127&gt;='Cash Flow'!$E$6,$G127&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -16287,11 +16298,11 @@
       </c>
       <c r="F128" s="74" t="n">
         <f aca="false">IF($C128="","",IF(Recurring!$E$12="Weekly",Recurring!$F$12+7*12,IF(Recurring!$E$12="Every 2 Weeks",Recurring!$F$12+14*12,IF(Recurring!$E$12="Monthly",EDATE(Recurring!$F$12,12),IF(Recurring!$E$12="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+12),2)=1,EOMONTH(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+12)/2)),DATE(YEAR(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+12)/2))),MONTH(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+12)/2))),15)),IF(Recurring!$E$12="One Time",IF(13=1,Recurring!$F$12,""),""))))))</f>
-        <v>46609</v>
+        <v>46640</v>
       </c>
       <c r="G128" s="74" t="n">
         <f aca="false">IF($F128="","",IF(Recurring!$G$12="Move Before",IF(WEEKDAY($F128,2)=6,$F128-1,IF(WEEKDAY($F128,2)=7,$F128-2,$F128)),IF(Recurring!$G$12="Move After",IF(WEEKDAY($F128,2)=6,$F128+2,IF(WEEKDAY($F128,2)=7,$F128+1,$F128)),$F128)))</f>
-        <v>46609</v>
+        <v>46640</v>
       </c>
       <c r="H128" s="75" t="n">
         <f aca="false">IF($G128="",0,IF(AND($G128&gt;='Cash Flow'!$E$6,$G128&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -16331,11 +16342,11 @@
       </c>
       <c r="F129" s="74" t="n">
         <f aca="false">IF($C129="","",IF(Recurring!$E$12="Weekly",Recurring!$F$12+7*13,IF(Recurring!$E$12="Every 2 Weeks",Recurring!$F$12+14*13,IF(Recurring!$E$12="Monthly",EDATE(Recurring!$F$12,13),IF(Recurring!$E$12="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+13),2)=1,EOMONTH(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+13)/2)),DATE(YEAR(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+13)/2))),MONTH(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+13)/2))),15)),IF(Recurring!$E$12="One Time",IF(14=1,Recurring!$F$12,""),""))))))</f>
-        <v>46640</v>
+        <v>46670</v>
       </c>
       <c r="G129" s="74" t="n">
         <f aca="false">IF($F129="","",IF(Recurring!$G$12="Move Before",IF(WEEKDAY($F129,2)=6,$F129-1,IF(WEEKDAY($F129,2)=7,$F129-2,$F129)),IF(Recurring!$G$12="Move After",IF(WEEKDAY($F129,2)=6,$F129+2,IF(WEEKDAY($F129,2)=7,$F129+1,$F129)),$F129)))</f>
-        <v>46640</v>
+        <v>46670</v>
       </c>
       <c r="H129" s="75" t="n">
         <f aca="false">IF($G129="",0,IF(AND($G129&gt;='Cash Flow'!$E$6,$G129&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -16375,11 +16386,11 @@
       </c>
       <c r="F130" s="74" t="n">
         <f aca="false">IF($C130="","",IF(Recurring!$E$12="Weekly",Recurring!$F$12+7*14,IF(Recurring!$E$12="Every 2 Weeks",Recurring!$F$12+14*14,IF(Recurring!$E$12="Monthly",EDATE(Recurring!$F$12,14),IF(Recurring!$E$12="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+14),2)=1,EOMONTH(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+14)/2)),DATE(YEAR(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+14)/2))),MONTH(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+14)/2))),15)),IF(Recurring!$E$12="One Time",IF(15=1,Recurring!$F$12,""),""))))))</f>
-        <v>46670</v>
+        <v>46701</v>
       </c>
       <c r="G130" s="74" t="n">
         <f aca="false">IF($F130="","",IF(Recurring!$G$12="Move Before",IF(WEEKDAY($F130,2)=6,$F130-1,IF(WEEKDAY($F130,2)=7,$F130-2,$F130)),IF(Recurring!$G$12="Move After",IF(WEEKDAY($F130,2)=6,$F130+2,IF(WEEKDAY($F130,2)=7,$F130+1,$F130)),$F130)))</f>
-        <v>46670</v>
+        <v>46701</v>
       </c>
       <c r="H130" s="75" t="n">
         <f aca="false">IF($G130="",0,IF(AND($G130&gt;='Cash Flow'!$E$6,$G130&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -16419,11 +16430,11 @@
       </c>
       <c r="F131" s="74" t="n">
         <f aca="false">IF($C131="","",IF(Recurring!$E$12="Weekly",Recurring!$F$12+7*15,IF(Recurring!$E$12="Every 2 Weeks",Recurring!$F$12+14*15,IF(Recurring!$E$12="Monthly",EDATE(Recurring!$F$12,15),IF(Recurring!$E$12="Twice a Month",IF(MOD((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+15),2)=1,EOMONTH(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+15)/2)),DATE(YEAR(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+15)/2))),MONTH(EDATE(Recurring!$F$12,INT((IF(DAY(Recurring!$F$12)&lt;=20,0,1)+15)/2))),15)),IF(Recurring!$E$12="One Time",IF(16=1,Recurring!$F$12,""),""))))))</f>
-        <v>46701</v>
+        <v>46731</v>
       </c>
       <c r="G131" s="74" t="n">
         <f aca="false">IF($F131="","",IF(Recurring!$G$12="Move Before",IF(WEEKDAY($F131,2)=6,$F131-1,IF(WEEKDAY($F131,2)=7,$F131-2,$F131)),IF(Recurring!$G$12="Move After",IF(WEEKDAY($F131,2)=6,$F131+2,IF(WEEKDAY($F131,2)=7,$F131+1,$F131)),$F131)))</f>
-        <v>46701</v>
+        <v>46731</v>
       </c>
       <c r="H131" s="75" t="n">
         <f aca="false">IF($G131="",0,IF(AND($G131&gt;='Cash Flow'!$E$6,$G131&lt;'Cash Flow'!$E$6+91),1,0))</f>
@@ -16483,7 +16494,7 @@
       </c>
       <c r="K132" s="72" t="n">
         <f aca="false">IF($H132=1,$I132*1000+COUNTIFS($I$4:$I$483,$I132,$J$4:$J$483,"&lt;"&amp;$J132)+1,"")</f>
-        <v>1003</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20675,7 +20686,7 @@
       </c>
       <c r="C228" s="72" t="str">
         <f aca="false">IF(OR(Recurring!$B$19="",Recurring!$H$19&lt;&gt;"Yes",Recurring!$D$19=""),"",Recurring!$B$19)</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="D228" s="72" t="str">
         <f aca="false">IF($C228="","",Recurring!$C$19)</f>
@@ -20719,7 +20730,7 @@
       </c>
       <c r="C229" s="72" t="str">
         <f aca="false">IF(OR(Recurring!$B$19="",Recurring!$H$19&lt;&gt;"Yes",Recurring!$D$19=""),"",Recurring!$B$19)</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="D229" s="72" t="str">
         <f aca="false">IF($C229="","",Recurring!$C$19)</f>
@@ -20763,7 +20774,7 @@
       </c>
       <c r="C230" s="72" t="str">
         <f aca="false">IF(OR(Recurring!$B$19="",Recurring!$H$19&lt;&gt;"Yes",Recurring!$D$19=""),"",Recurring!$B$19)</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="D230" s="72" t="str">
         <f aca="false">IF($C230="","",Recurring!$C$19)</f>
@@ -20807,7 +20818,7 @@
       </c>
       <c r="C231" s="72" t="str">
         <f aca="false">IF(OR(Recurring!$B$19="",Recurring!$H$19&lt;&gt;"Yes",Recurring!$D$19=""),"",Recurring!$B$19)</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="D231" s="72" t="str">
         <f aca="false">IF($C231="","",Recurring!$C$19)</f>
@@ -20851,7 +20862,7 @@
       </c>
       <c r="C232" s="72" t="str">
         <f aca="false">IF(OR(Recurring!$B$19="",Recurring!$H$19&lt;&gt;"Yes",Recurring!$D$19=""),"",Recurring!$B$19)</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="D232" s="72" t="str">
         <f aca="false">IF($C232="","",Recurring!$C$19)</f>
@@ -20895,7 +20906,7 @@
       </c>
       <c r="C233" s="72" t="str">
         <f aca="false">IF(OR(Recurring!$B$19="",Recurring!$H$19&lt;&gt;"Yes",Recurring!$D$19=""),"",Recurring!$B$19)</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="D233" s="72" t="str">
         <f aca="false">IF($C233="","",Recurring!$C$19)</f>
@@ -20939,7 +20950,7 @@
       </c>
       <c r="C234" s="72" t="str">
         <f aca="false">IF(OR(Recurring!$B$19="",Recurring!$H$19&lt;&gt;"Yes",Recurring!$D$19=""),"",Recurring!$B$19)</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="D234" s="72" t="str">
         <f aca="false">IF($C234="","",Recurring!$C$19)</f>
@@ -20983,7 +20994,7 @@
       </c>
       <c r="C235" s="72" t="str">
         <f aca="false">IF(OR(Recurring!$B$19="",Recurring!$H$19&lt;&gt;"Yes",Recurring!$D$19=""),"",Recurring!$B$19)</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="D235" s="72" t="str">
         <f aca="false">IF($C235="","",Recurring!$C$19)</f>
@@ -21027,7 +21038,7 @@
       </c>
       <c r="C236" s="72" t="str">
         <f aca="false">IF(OR(Recurring!$B$19="",Recurring!$H$19&lt;&gt;"Yes",Recurring!$D$19=""),"",Recurring!$B$19)</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="D236" s="72" t="str">
         <f aca="false">IF($C236="","",Recurring!$C$19)</f>
@@ -21071,7 +21082,7 @@
       </c>
       <c r="C237" s="72" t="str">
         <f aca="false">IF(OR(Recurring!$B$19="",Recurring!$H$19&lt;&gt;"Yes",Recurring!$D$19=""),"",Recurring!$B$19)</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="D237" s="72" t="str">
         <f aca="false">IF($C237="","",Recurring!$C$19)</f>
@@ -21115,7 +21126,7 @@
       </c>
       <c r="C238" s="72" t="str">
         <f aca="false">IF(OR(Recurring!$B$19="",Recurring!$H$19&lt;&gt;"Yes",Recurring!$D$19=""),"",Recurring!$B$19)</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="D238" s="72" t="str">
         <f aca="false">IF($C238="","",Recurring!$C$19)</f>
@@ -21159,7 +21170,7 @@
       </c>
       <c r="C239" s="72" t="str">
         <f aca="false">IF(OR(Recurring!$B$19="",Recurring!$H$19&lt;&gt;"Yes",Recurring!$D$19=""),"",Recurring!$B$19)</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="D239" s="72" t="str">
         <f aca="false">IF($C239="","",Recurring!$C$19)</f>
@@ -21203,7 +21214,7 @@
       </c>
       <c r="C240" s="72" t="str">
         <f aca="false">IF(OR(Recurring!$B$19="",Recurring!$H$19&lt;&gt;"Yes",Recurring!$D$19=""),"",Recurring!$B$19)</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="D240" s="72" t="str">
         <f aca="false">IF($C240="","",Recurring!$C$19)</f>
@@ -21247,7 +21258,7 @@
       </c>
       <c r="C241" s="72" t="str">
         <f aca="false">IF(OR(Recurring!$B$19="",Recurring!$H$19&lt;&gt;"Yes",Recurring!$D$19=""),"",Recurring!$B$19)</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="D241" s="72" t="str">
         <f aca="false">IF($C241="","",Recurring!$C$19)</f>
@@ -21291,7 +21302,7 @@
       </c>
       <c r="C242" s="72" t="str">
         <f aca="false">IF(OR(Recurring!$B$19="",Recurring!$H$19&lt;&gt;"Yes",Recurring!$D$19=""),"",Recurring!$B$19)</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="D242" s="72" t="str">
         <f aca="false">IF($C242="","",Recurring!$C$19)</f>
@@ -21335,7 +21346,7 @@
       </c>
       <c r="C243" s="72" t="str">
         <f aca="false">IF(OR(Recurring!$B$19="",Recurring!$H$19&lt;&gt;"Yes",Recurring!$D$19=""),"",Recurring!$B$19)</f>
-        <v>Central Maine Power: Property</v>
+        <v>Central Maine Power: Payment Plan</v>
       </c>
       <c r="D243" s="72" t="str">
         <f aca="false">IF($C243="","",Recurring!$C$19)</f>

</xml_diff>

<commit_message>
Make one-week amount changes discoverable
Overriding a single week's figure already worked through the Amount Paid
column, but nothing about a column called "Amount Paid" suggests it accepts a
bigger paycheck you are expecting. Renamed to "Amount Paid / Received" so it
reads as the right cell for income as well as bills.

A figure entered against a future date now reads ADJUSTED rather than PAID: a
revised expectation is not money that has moved, and the sheet should not
claim otherwise.

Documented on the Instructions tab with the concrete case - extra shifts at
Bruno's, $150 instead of $90 - and verified: MONEY IN, the running balance and
the Summary all follow the entered figure, the row stays linked to the
Recurring tab, and every other week keeps the usual $90.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0171RmRt5NEruH3aRWtNMF8Q
</commit_message>
<xml_diff>
--- a/Weekly_Cash_Flow_Survival.xlsx
+++ b/Weekly_Cash_Flow_Survival.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">'Cash Flow'!$A$1:$K$284</definedName>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Instructions!$A$1:$C$46</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Instructions!$A$1:$C$48</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">Recurring!$A$1:$J$38</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">Recurring!$4:$4</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Summary!$A$1:$J$28</definedName>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="171">
   <si>
     <t xml:space="preserve">WEEKLY CASH FLOW SURVIVAL WORKSHEET</t>
   </si>
@@ -138,10 +138,22 @@
     <t xml:space="preserve">Type a description, date, Income or Expense, and an amount into any blank row in a week block. Nothing needs to exist on the Recurring tab first.</t>
   </si>
   <si>
+    <t xml:space="preserve">One week's amount is different</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is what the 'Amount Paid / Received' column is for, and it needs no formula touched at all. Working extra shifts and expecting $150 from Bruno's instead of $90? Type 150 into that row's Amount Paid / Received cell. MONEY IN, the running balance and the Summary all follow it, that row stays linked to the Recurring tab, and every other week keeps the usual $90. It works the same for a bill that comes in higher or lower than scheduled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADJUSTED vs PAID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A figure typed against a date still in the future reads ADJUSTED — you have revised what you expect, not recorded money that moved. Once the date arrives it reads PAID.</t>
+  </si>
+  <si>
     <t xml:space="preserve">To pay part of a bill</t>
   </si>
   <si>
-    <t xml:space="preserve">Leave the scheduled row alone and put what you actually paid in Amount Paid. That column is yours already and always wins over the scheduled figure.</t>
+    <t xml:space="preserve">Same column. Put what you actually paid in Amount Paid / Received; it always wins over the scheduled figure.</t>
   </si>
   <si>
     <t xml:space="preserve">To get the formula back</t>
@@ -393,7 +405,7 @@
     <t xml:space="preserve">Scheduled Amount</t>
   </si>
   <si>
-    <t xml:space="preserve">Amount Paid</t>
+    <t xml:space="preserve">Amount Paid / Received</t>
   </si>
   <si>
     <t xml:space="preserve">Running Balance</t>
@@ -1462,7 +1474,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:C46"/>
+  <dimension ref="B2:C48"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -1640,24 +1652,24 @@
         <v>40</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="3" t="s">
+    <row r="28" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B28" s="12" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="12" t="s">
+      <c r="C28" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="5" t="s">
+    </row>
+    <row r="29" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="12" t="s">
         <v>43</v>
       </c>
+      <c r="C29" s="5" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C31" s="5" t="s">
+      <c r="B31" s="3" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1685,89 +1697,105 @@
         <v>51</v>
       </c>
     </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="C37" s="14" t="s">
+      <c r="B36" s="12" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="38" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="C38" s="14" t="s">
+      <c r="C36" s="5" t="s">
         <v>55</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="3" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="13" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="13" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="13" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="13" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="13" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="13" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="13" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="13" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>63</v>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B47" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C47" s="14" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B48" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C48" s="14" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1803,44 +1831,44 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="J4" s="15" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1848,28 +1876,28 @@
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D5" s="18" t="n">
         <v>90</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="F5" s="19" t="n">
         <v>46246</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="J5" s="6"/>
     </row>
@@ -1878,28 +1906,28 @@
         <v>2</v>
       </c>
       <c r="B6" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="C6" s="22" t="s">
         <v>81</v>
-      </c>
-      <c r="C6" s="22" t="s">
-        <v>77</v>
       </c>
       <c r="D6" s="23" t="n">
         <v>790</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="F6" s="24" t="n">
         <v>46248</v>
       </c>
       <c r="G6" s="22" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H6" s="22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I6" s="21" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="J6" s="21"/>
     </row>
@@ -1908,28 +1936,28 @@
         <v>3</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D7" s="18" t="n">
         <v>21.1</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F7" s="19" t="n">
         <v>46238</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="J7" s="6"/>
     </row>
@@ -1938,28 +1966,28 @@
         <v>4</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D8" s="23" t="n">
         <v>20</v>
       </c>
       <c r="E8" s="22" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F8" s="24" t="n">
         <v>46239</v>
       </c>
       <c r="G8" s="22" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H8" s="22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I8" s="21" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="J8" s="21"/>
     </row>
@@ -1968,28 +1996,28 @@
         <v>5</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D9" s="18" t="n">
         <v>10</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F9" s="19" t="n">
         <v>46239</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="J9" s="6"/>
     </row>
@@ -1998,28 +2026,28 @@
         <v>6</v>
       </c>
       <c r="B10" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10" s="22" t="s">
         <v>87</v>
-      </c>
-      <c r="C10" s="22" t="s">
-        <v>83</v>
       </c>
       <c r="D10" s="23" t="n">
         <v>4.99</v>
       </c>
       <c r="E10" s="22" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F10" s="24" t="n">
         <v>46272</v>
       </c>
       <c r="G10" s="22" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H10" s="22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I10" s="21" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="J10" s="21"/>
     </row>
@@ -2028,28 +2056,28 @@
         <v>7</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D11" s="18" t="n">
         <v>500</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F11" s="19" t="n">
         <v>46272</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="J11" s="6"/>
     </row>
@@ -2058,28 +2086,28 @@
         <v>8</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D12" s="23" t="n">
         <v>163.5</v>
       </c>
       <c r="E12" s="22" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F12" s="24" t="n">
         <v>46275</v>
       </c>
       <c r="G12" s="22" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H12" s="22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I12" s="21" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="J12" s="21"/>
     </row>
@@ -2088,28 +2116,28 @@
         <v>9</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D13" s="18" t="n">
         <v>2.99</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F13" s="19" t="n">
         <v>46247</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H13" s="17" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="J13" s="6"/>
     </row>
@@ -2118,28 +2146,28 @@
         <v>10</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D14" s="23" t="n">
         <v>350</v>
       </c>
       <c r="E14" s="22" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F14" s="24" t="n">
         <v>46248</v>
       </c>
       <c r="G14" s="22" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="H14" s="22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I14" s="21" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="J14" s="21"/>
     </row>
@@ -2148,28 +2176,28 @@
         <v>11</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D15" s="18" t="n">
         <v>171.1</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F15" s="19" t="n">
         <v>46250</v>
       </c>
       <c r="G15" s="17" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H15" s="17" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="J15" s="6"/>
     </row>
@@ -2178,28 +2206,28 @@
         <v>12</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D16" s="23" t="n">
         <v>45</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F16" s="24" t="n">
         <v>46250</v>
       </c>
       <c r="G16" s="22" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H16" s="22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I16" s="21" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="J16" s="21"/>
     </row>
@@ -2208,28 +2236,28 @@
         <v>13</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D17" s="18" t="n">
         <v>16.99</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F17" s="19" t="n">
         <v>46252</v>
       </c>
       <c r="G17" s="17" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H17" s="17" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="J17" s="6"/>
     </row>
@@ -2238,28 +2266,28 @@
         <v>14</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D18" s="23" t="n">
         <v>13.7</v>
       </c>
       <c r="E18" s="22" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F18" s="24" t="n">
         <v>46259</v>
       </c>
       <c r="G18" s="22" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H18" s="22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I18" s="21" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="J18" s="21"/>
     </row>
@@ -2268,28 +2296,28 @@
         <v>15</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D19" s="18" t="n">
         <v>43.87</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F19" s="19" t="n">
         <v>46259</v>
       </c>
       <c r="G19" s="17" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H19" s="17" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="J19" s="6"/>
     </row>
@@ -2298,28 +2326,28 @@
         <v>16</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D20" s="23" t="n">
         <v>150</v>
       </c>
       <c r="E20" s="22" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F20" s="24" t="n">
         <v>46264</v>
       </c>
       <c r="G20" s="22" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H20" s="22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I20" s="21" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="J20" s="21"/>
     </row>
@@ -2328,28 +2356,28 @@
         <v>17</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D21" s="18" t="n">
         <v>143.37</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F21" s="19" t="n">
         <v>46265</v>
       </c>
       <c r="G21" s="17" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H21" s="17" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="J21" s="6"/>
     </row>
@@ -2537,17 +2565,17 @@
     </row>
     <row r="36" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="14" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="14" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="25" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -2614,17 +2642,17 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="12" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E5" s="26" t="n">
         <v>71.17</v>
@@ -2632,7 +2660,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="12" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="E6" s="27" t="n">
         <v>46241</v>
@@ -2644,7 +2672,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="12" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E7" s="26" t="n">
         <v>200</v>
@@ -2652,7 +2680,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="29" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="E8" s="30" t="n">
         <f aca="true">TODAY()</f>
@@ -2661,12 +2689,12 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="25" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="25" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2679,7 +2707,7 @@
       <c r="E13" s="32"/>
       <c r="F13" s="32"/>
       <c r="G13" s="33" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="H13" s="32"/>
       <c r="I13" s="34" t="n">
@@ -2694,19 +2722,19 @@
     </row>
     <row r="14" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="35" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C14" s="35" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D14" s="35" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F14" s="35" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G14" s="36" t="s">
         <v>18</v>
@@ -2715,10 +2743,10 @@
         <v>20</v>
       </c>
       <c r="I14" s="35" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="J14" s="35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2752,7 +2780,7 @@
         <v>50.07</v>
       </c>
       <c r="J15" s="46" t="str">
-        <f aca="true">IF($B15="","",IF($F15&lt;&gt;"","PAID",IF($C15&lt;TODAY(),"PAST DUE",IF($C15&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B15="","",IF($F15&lt;&gt;"",IF($C15&gt;TODAY(),"ADJUSTED","PAID"),IF($C15&lt;TODAY(),"PAST DUE",IF($C15&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>PAST DUE</v>
       </c>
     </row>
@@ -2787,7 +2815,7 @@
         <v>30.07</v>
       </c>
       <c r="J16" s="46" t="str">
-        <f aca="true">IF($B16="","",IF($F16&lt;&gt;"","PAID",IF($C16&lt;TODAY(),"PAST DUE",IF($C16&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B16="","",IF($F16&lt;&gt;"",IF($C16&gt;TODAY(),"ADJUSTED","PAID"),IF($C16&lt;TODAY(),"PAST DUE",IF($C16&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>PAST DUE</v>
       </c>
     </row>
@@ -2822,7 +2850,7 @@
         <v>20.07</v>
       </c>
       <c r="J17" s="46" t="str">
-        <f aca="true">IF($B17="","",IF($F17&lt;&gt;"","PAID",IF($C17&lt;TODAY(),"PAST DUE",IF($C17&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B17="","",IF($F17&lt;&gt;"",IF($C17&gt;TODAY(),"ADJUSTED","PAID"),IF($C17&lt;TODAY(),"PAST DUE",IF($C17&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>PAST DUE</v>
       </c>
     </row>
@@ -2857,7 +2885,7 @@
         <v>110.07</v>
       </c>
       <c r="J18" s="46" t="str">
-        <f aca="true">IF($B18="","",IF($F18&lt;&gt;"","PAID",IF($C18&lt;TODAY(),"PAST DUE",IF($C18&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B18="","",IF($F18&lt;&gt;"",IF($C18&gt;TODAY(),"ADJUSTED","PAID"),IF($C18&lt;TODAY(),"PAST DUE",IF($C18&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>DUE</v>
       </c>
     </row>
@@ -2892,7 +2920,7 @@
         <v>107.08</v>
       </c>
       <c r="J19" s="46" t="str">
-        <f aca="true">IF($B19="","",IF($F19&lt;&gt;"","PAID",IF($C19&lt;TODAY(),"PAST DUE",IF($C19&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B19="","",IF($F19&lt;&gt;"",IF($C19&gt;TODAY(),"ADJUSTED","PAID"),IF($C19&lt;TODAY(),"PAST DUE",IF($C19&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>DUE</v>
       </c>
     </row>
@@ -2927,7 +2955,7 @@
         <v/>
       </c>
       <c r="J20" s="46" t="str">
-        <f aca="true">IF($B20="","",IF($F20&lt;&gt;"","PAID",IF($C20&lt;TODAY(),"PAST DUE",IF($C20&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B20="","",IF($F20&lt;&gt;"",IF($C20&gt;TODAY(),"ADJUSTED","PAID"),IF($C20&lt;TODAY(),"PAST DUE",IF($C20&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -2962,7 +2990,7 @@
         <v/>
       </c>
       <c r="J21" s="46" t="str">
-        <f aca="true">IF($B21="","",IF($F21&lt;&gt;"","PAID",IF($C21&lt;TODAY(),"PAST DUE",IF($C21&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B21="","",IF($F21&lt;&gt;"",IF($C21&gt;TODAY(),"ADJUSTED","PAID"),IF($C21&lt;TODAY(),"PAST DUE",IF($C21&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -2997,7 +3025,7 @@
         <v/>
       </c>
       <c r="J22" s="46" t="str">
-        <f aca="true">IF($B22="","",IF($F22&lt;&gt;"","PAID",IF($C22&lt;TODAY(),"PAST DUE",IF($C22&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B22="","",IF($F22&lt;&gt;"",IF($C22&gt;TODAY(),"ADJUSTED","PAID"),IF($C22&lt;TODAY(),"PAST DUE",IF($C22&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -3032,7 +3060,7 @@
         <v/>
       </c>
       <c r="J23" s="46" t="str">
-        <f aca="true">IF($B23="","",IF($F23&lt;&gt;"","PAID",IF($C23&lt;TODAY(),"PAST DUE",IF($C23&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B23="","",IF($F23&lt;&gt;"",IF($C23&gt;TODAY(),"ADJUSTED","PAID"),IF($C23&lt;TODAY(),"PAST DUE",IF($C23&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -3067,13 +3095,13 @@
         <v/>
       </c>
       <c r="J24" s="46" t="str">
-        <f aca="true">IF($B24="","",IF($F24&lt;&gt;"","PAID",IF($C24&lt;TODAY(),"PAST DUE",IF($C24&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B24="","",IF($F24&lt;&gt;"",IF($C24&gt;TODAY(),"ADJUSTED","PAID"),IF($C24&lt;TODAY(),"PAST DUE",IF($C24&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="47" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C25" s="48"/>
       <c r="D25" s="48"/>
@@ -3206,7 +3234,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="52" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C32" s="53"/>
       <c r="D32" s="53"/>
@@ -3243,7 +3271,7 @@
       <c r="E34" s="32"/>
       <c r="F34" s="32"/>
       <c r="G34" s="33" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="H34" s="32"/>
       <c r="I34" s="34" t="n">
@@ -3258,19 +3286,19 @@
     </row>
     <row r="35" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="35" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C35" s="35" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D35" s="35" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E35" s="35" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F35" s="35" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G35" s="36" t="s">
         <v>18</v>
@@ -3279,10 +3307,10 @@
         <v>20</v>
       </c>
       <c r="I35" s="35" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="J35" s="35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3316,7 +3344,7 @@
         <v>897.08</v>
       </c>
       <c r="J36" s="46" t="str">
-        <f aca="true">IF($B36="","",IF($F36&lt;&gt;"","PAID",IF($C36&lt;TODAY(),"PAST DUE",IF($C36&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B36="","",IF($F36&lt;&gt;"",IF($C36&gt;TODAY(),"ADJUSTED","PAID"),IF($C36&lt;TODAY(),"PAST DUE",IF($C36&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>DUE</v>
       </c>
     </row>
@@ -3351,7 +3379,7 @@
         <v>547.08</v>
       </c>
       <c r="J37" s="46" t="str">
-        <f aca="true">IF($B37="","",IF($F37&lt;&gt;"","PAID",IF($C37&lt;TODAY(),"PAST DUE",IF($C37&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B37="","",IF($F37&lt;&gt;"",IF($C37&gt;TODAY(),"ADJUSTED","PAID"),IF($C37&lt;TODAY(),"PAST DUE",IF($C37&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>DUE</v>
       </c>
     </row>
@@ -3386,7 +3414,7 @@
         <v>375.98</v>
       </c>
       <c r="J38" s="46" t="str">
-        <f aca="true">IF($B38="","",IF($F38&lt;&gt;"","PAID",IF($C38&lt;TODAY(),"PAST DUE",IF($C38&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B38="","",IF($F38&lt;&gt;"",IF($C38&gt;TODAY(),"ADJUSTED","PAID"),IF($C38&lt;TODAY(),"PAST DUE",IF($C38&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -3421,7 +3449,7 @@
         <v>330.98</v>
       </c>
       <c r="J39" s="46" t="str">
-        <f aca="true">IF($B39="","",IF($F39&lt;&gt;"","PAID",IF($C39&lt;TODAY(),"PAST DUE",IF($C39&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B39="","",IF($F39&lt;&gt;"",IF($C39&gt;TODAY(),"ADJUSTED","PAID"),IF($C39&lt;TODAY(),"PAST DUE",IF($C39&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -3456,7 +3484,7 @@
         <v>313.99</v>
       </c>
       <c r="J40" s="46" t="str">
-        <f aca="true">IF($B40="","",IF($F40&lt;&gt;"","PAID",IF($C40&lt;TODAY(),"PAST DUE",IF($C40&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B40="","",IF($F40&lt;&gt;"",IF($C40&gt;TODAY(),"ADJUSTED","PAID"),IF($C40&lt;TODAY(),"PAST DUE",IF($C40&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -3491,7 +3519,7 @@
         <v>403.99</v>
       </c>
       <c r="J41" s="46" t="str">
-        <f aca="true">IF($B41="","",IF($F41&lt;&gt;"","PAID",IF($C41&lt;TODAY(),"PAST DUE",IF($C41&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B41="","",IF($F41&lt;&gt;"",IF($C41&gt;TODAY(),"ADJUSTED","PAID"),IF($C41&lt;TODAY(),"PAST DUE",IF($C41&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -3526,7 +3554,7 @@
         <v/>
       </c>
       <c r="J42" s="46" t="str">
-        <f aca="true">IF($B42="","",IF($F42&lt;&gt;"","PAID",IF($C42&lt;TODAY(),"PAST DUE",IF($C42&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B42="","",IF($F42&lt;&gt;"",IF($C42&gt;TODAY(),"ADJUSTED","PAID"),IF($C42&lt;TODAY(),"PAST DUE",IF($C42&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -3561,7 +3589,7 @@
         <v/>
       </c>
       <c r="J43" s="46" t="str">
-        <f aca="true">IF($B43="","",IF($F43&lt;&gt;"","PAID",IF($C43&lt;TODAY(),"PAST DUE",IF($C43&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B43="","",IF($F43&lt;&gt;"",IF($C43&gt;TODAY(),"ADJUSTED","PAID"),IF($C43&lt;TODAY(),"PAST DUE",IF($C43&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -3596,7 +3624,7 @@
         <v/>
       </c>
       <c r="J44" s="46" t="str">
-        <f aca="true">IF($B44="","",IF($F44&lt;&gt;"","PAID",IF($C44&lt;TODAY(),"PAST DUE",IF($C44&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B44="","",IF($F44&lt;&gt;"",IF($C44&gt;TODAY(),"ADJUSTED","PAID"),IF($C44&lt;TODAY(),"PAST DUE",IF($C44&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -3631,13 +3659,13 @@
         <v/>
       </c>
       <c r="J45" s="46" t="str">
-        <f aca="true">IF($B45="","",IF($F45&lt;&gt;"","PAID",IF($C45&lt;TODAY(),"PAST DUE",IF($C45&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B45="","",IF($F45&lt;&gt;"",IF($C45&gt;TODAY(),"ADJUSTED","PAID"),IF($C45&lt;TODAY(),"PAST DUE",IF($C45&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="47" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C46" s="48"/>
       <c r="D46" s="48"/>
@@ -3770,7 +3798,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="52" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C53" s="53"/>
       <c r="D53" s="53"/>
@@ -3807,7 +3835,7 @@
       <c r="E55" s="32"/>
       <c r="F55" s="32"/>
       <c r="G55" s="33" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="H55" s="32"/>
       <c r="I55" s="34" t="n">
@@ -3822,19 +3850,19 @@
     </row>
     <row r="56" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B56" s="35" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C56" s="35" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D56" s="35" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E56" s="35" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F56" s="35" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G56" s="36" t="s">
         <v>18</v>
@@ -3843,10 +3871,10 @@
         <v>20</v>
       </c>
       <c r="I56" s="35" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="J56" s="35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3880,7 +3908,7 @@
         <v>1193.99</v>
       </c>
       <c r="J57" s="46" t="str">
-        <f aca="true">IF($B57="","",IF($F57&lt;&gt;"","PAID",IF($C57&lt;TODAY(),"PAST DUE",IF($C57&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B57="","",IF($F57&lt;&gt;"",IF($C57&gt;TODAY(),"ADJUSTED","PAID"),IF($C57&lt;TODAY(),"PAST DUE",IF($C57&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -3915,7 +3943,7 @@
         <v>1180.29</v>
       </c>
       <c r="J58" s="46" t="str">
-        <f aca="true">IF($B58="","",IF($F58&lt;&gt;"","PAID",IF($C58&lt;TODAY(),"PAST DUE",IF($C58&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B58="","",IF($F58&lt;&gt;"",IF($C58&gt;TODAY(),"ADJUSTED","PAID"),IF($C58&lt;TODAY(),"PAST DUE",IF($C58&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -3950,7 +3978,7 @@
         <v>1136.42</v>
       </c>
       <c r="J59" s="46" t="str">
-        <f aca="true">IF($B59="","",IF($F59&lt;&gt;"","PAID",IF($C59&lt;TODAY(),"PAST DUE",IF($C59&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B59="","",IF($F59&lt;&gt;"",IF($C59&gt;TODAY(),"ADJUSTED","PAID"),IF($C59&lt;TODAY(),"PAST DUE",IF($C59&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -3985,7 +4013,7 @@
         <v>1226.42</v>
       </c>
       <c r="J60" s="46" t="str">
-        <f aca="true">IF($B60="","",IF($F60&lt;&gt;"","PAID",IF($C60&lt;TODAY(),"PAST DUE",IF($C60&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B60="","",IF($F60&lt;&gt;"",IF($C60&gt;TODAY(),"ADJUSTED","PAID"),IF($C60&lt;TODAY(),"PAST DUE",IF($C60&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -4020,7 +4048,7 @@
         <v/>
       </c>
       <c r="J61" s="46" t="str">
-        <f aca="true">IF($B61="","",IF($F61&lt;&gt;"","PAID",IF($C61&lt;TODAY(),"PAST DUE",IF($C61&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B61="","",IF($F61&lt;&gt;"",IF($C61&gt;TODAY(),"ADJUSTED","PAID"),IF($C61&lt;TODAY(),"PAST DUE",IF($C61&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -4055,7 +4083,7 @@
         <v/>
       </c>
       <c r="J62" s="46" t="str">
-        <f aca="true">IF($B62="","",IF($F62&lt;&gt;"","PAID",IF($C62&lt;TODAY(),"PAST DUE",IF($C62&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B62="","",IF($F62&lt;&gt;"",IF($C62&gt;TODAY(),"ADJUSTED","PAID"),IF($C62&lt;TODAY(),"PAST DUE",IF($C62&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -4090,7 +4118,7 @@
         <v/>
       </c>
       <c r="J63" s="46" t="str">
-        <f aca="true">IF($B63="","",IF($F63&lt;&gt;"","PAID",IF($C63&lt;TODAY(),"PAST DUE",IF($C63&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B63="","",IF($F63&lt;&gt;"",IF($C63&gt;TODAY(),"ADJUSTED","PAID"),IF($C63&lt;TODAY(),"PAST DUE",IF($C63&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -4125,7 +4153,7 @@
         <v/>
       </c>
       <c r="J64" s="46" t="str">
-        <f aca="true">IF($B64="","",IF($F64&lt;&gt;"","PAID",IF($C64&lt;TODAY(),"PAST DUE",IF($C64&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B64="","",IF($F64&lt;&gt;"",IF($C64&gt;TODAY(),"ADJUSTED","PAID"),IF($C64&lt;TODAY(),"PAST DUE",IF($C64&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -4160,7 +4188,7 @@
         <v/>
       </c>
       <c r="J65" s="46" t="str">
-        <f aca="true">IF($B65="","",IF($F65&lt;&gt;"","PAID",IF($C65&lt;TODAY(),"PAST DUE",IF($C65&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B65="","",IF($F65&lt;&gt;"",IF($C65&gt;TODAY(),"ADJUSTED","PAID"),IF($C65&lt;TODAY(),"PAST DUE",IF($C65&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -4195,13 +4223,13 @@
         <v/>
       </c>
       <c r="J66" s="46" t="str">
-        <f aca="true">IF($B66="","",IF($F66&lt;&gt;"","PAID",IF($C66&lt;TODAY(),"PAST DUE",IF($C66&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B66="","",IF($F66&lt;&gt;"",IF($C66&gt;TODAY(),"ADJUSTED","PAID"),IF($C66&lt;TODAY(),"PAST DUE",IF($C66&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="47" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C67" s="48"/>
       <c r="D67" s="48"/>
@@ -4334,7 +4362,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="52" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C74" s="53"/>
       <c r="D74" s="53"/>
@@ -4371,7 +4399,7 @@
       <c r="E76" s="32"/>
       <c r="F76" s="32"/>
       <c r="G76" s="33" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="H76" s="32"/>
       <c r="I76" s="34" t="n">
@@ -4386,19 +4414,19 @@
     </row>
     <row r="77" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B77" s="35" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C77" s="35" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D77" s="35" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E77" s="35" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F77" s="35" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G77" s="36" t="s">
         <v>18</v>
@@ -4407,10 +4435,10 @@
         <v>20</v>
       </c>
       <c r="I77" s="35" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="J77" s="35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4444,7 +4472,7 @@
         <v>2016.42</v>
       </c>
       <c r="J78" s="46" t="str">
-        <f aca="true">IF($B78="","",IF($F78&lt;&gt;"","PAID",IF($C78&lt;TODAY(),"PAST DUE",IF($C78&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B78="","",IF($F78&lt;&gt;"",IF($C78&gt;TODAY(),"ADJUSTED","PAID"),IF($C78&lt;TODAY(),"PAST DUE",IF($C78&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -4479,7 +4507,7 @@
         <v>1866.42</v>
       </c>
       <c r="J79" s="46" t="str">
-        <f aca="true">IF($B79="","",IF($F79&lt;&gt;"","PAID",IF($C79&lt;TODAY(),"PAST DUE",IF($C79&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B79="","",IF($F79&lt;&gt;"",IF($C79&gt;TODAY(),"ADJUSTED","PAID"),IF($C79&lt;TODAY(),"PAST DUE",IF($C79&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -4514,7 +4542,7 @@
         <v>1516.42</v>
       </c>
       <c r="J80" s="46" t="str">
-        <f aca="true">IF($B80="","",IF($F80&lt;&gt;"","PAID",IF($C80&lt;TODAY(),"PAST DUE",IF($C80&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B80="","",IF($F80&lt;&gt;"",IF($C80&gt;TODAY(),"ADJUSTED","PAID"),IF($C80&lt;TODAY(),"PAST DUE",IF($C80&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -4549,7 +4577,7 @@
         <v>1373.05</v>
       </c>
       <c r="J81" s="46" t="str">
-        <f aca="true">IF($B81="","",IF($F81&lt;&gt;"","PAID",IF($C81&lt;TODAY(),"PAST DUE",IF($C81&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B81="","",IF($F81&lt;&gt;"",IF($C81&gt;TODAY(),"ADJUSTED","PAID"),IF($C81&lt;TODAY(),"PAST DUE",IF($C81&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -4584,7 +4612,7 @@
         <v>1463.05</v>
       </c>
       <c r="J82" s="46" t="str">
-        <f aca="true">IF($B82="","",IF($F82&lt;&gt;"","PAID",IF($C82&lt;TODAY(),"PAST DUE",IF($C82&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B82="","",IF($F82&lt;&gt;"",IF($C82&gt;TODAY(),"ADJUSTED","PAID"),IF($C82&lt;TODAY(),"PAST DUE",IF($C82&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -4619,7 +4647,7 @@
         <v/>
       </c>
       <c r="J83" s="46" t="str">
-        <f aca="true">IF($B83="","",IF($F83&lt;&gt;"","PAID",IF($C83&lt;TODAY(),"PAST DUE",IF($C83&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B83="","",IF($F83&lt;&gt;"",IF($C83&gt;TODAY(),"ADJUSTED","PAID"),IF($C83&lt;TODAY(),"PAST DUE",IF($C83&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -4654,7 +4682,7 @@
         <v/>
       </c>
       <c r="J84" s="46" t="str">
-        <f aca="true">IF($B84="","",IF($F84&lt;&gt;"","PAID",IF($C84&lt;TODAY(),"PAST DUE",IF($C84&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B84="","",IF($F84&lt;&gt;"",IF($C84&gt;TODAY(),"ADJUSTED","PAID"),IF($C84&lt;TODAY(),"PAST DUE",IF($C84&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -4689,7 +4717,7 @@
         <v/>
       </c>
       <c r="J85" s="46" t="str">
-        <f aca="true">IF($B85="","",IF($F85&lt;&gt;"","PAID",IF($C85&lt;TODAY(),"PAST DUE",IF($C85&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B85="","",IF($F85&lt;&gt;"",IF($C85&gt;TODAY(),"ADJUSTED","PAID"),IF($C85&lt;TODAY(),"PAST DUE",IF($C85&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -4724,7 +4752,7 @@
         <v/>
       </c>
       <c r="J86" s="46" t="str">
-        <f aca="true">IF($B86="","",IF($F86&lt;&gt;"","PAID",IF($C86&lt;TODAY(),"PAST DUE",IF($C86&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B86="","",IF($F86&lt;&gt;"",IF($C86&gt;TODAY(),"ADJUSTED","PAID"),IF($C86&lt;TODAY(),"PAST DUE",IF($C86&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -4759,13 +4787,13 @@
         <v/>
       </c>
       <c r="J87" s="46" t="str">
-        <f aca="true">IF($B87="","",IF($F87&lt;&gt;"","PAID",IF($C87&lt;TODAY(),"PAST DUE",IF($C87&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B87="","",IF($F87&lt;&gt;"",IF($C87&gt;TODAY(),"ADJUSTED","PAID"),IF($C87&lt;TODAY(),"PAST DUE",IF($C87&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="47" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C88" s="48"/>
       <c r="D88" s="48"/>
@@ -4898,7 +4926,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B95" s="52" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C95" s="53"/>
       <c r="D95" s="53"/>
@@ -4935,7 +4963,7 @@
       <c r="E97" s="32"/>
       <c r="F97" s="32"/>
       <c r="G97" s="33" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="H97" s="32"/>
       <c r="I97" s="34" t="n">
@@ -4950,19 +4978,19 @@
     </row>
     <row r="98" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B98" s="35" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C98" s="35" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D98" s="35" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E98" s="35" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F98" s="35" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G98" s="36" t="s">
         <v>18</v>
@@ -4971,10 +4999,10 @@
         <v>20</v>
       </c>
       <c r="I98" s="35" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="J98" s="35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5008,7 +5036,7 @@
         <v>2253.05</v>
       </c>
       <c r="J99" s="46" t="str">
-        <f aca="true">IF($B99="","",IF($F99&lt;&gt;"","PAID",IF($C99&lt;TODAY(),"PAST DUE",IF($C99&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B99="","",IF($F99&lt;&gt;"",IF($C99&gt;TODAY(),"ADJUSTED","PAID"),IF($C99&lt;TODAY(),"PAST DUE",IF($C99&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -5043,7 +5071,7 @@
         <v>2231.95</v>
       </c>
       <c r="J100" s="46" t="str">
-        <f aca="true">IF($B100="","",IF($F100&lt;&gt;"","PAID",IF($C100&lt;TODAY(),"PAST DUE",IF($C100&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B100="","",IF($F100&lt;&gt;"",IF($C100&gt;TODAY(),"ADJUSTED","PAID"),IF($C100&lt;TODAY(),"PAST DUE",IF($C100&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -5078,7 +5106,7 @@
         <v>2211.95</v>
       </c>
       <c r="J101" s="46" t="str">
-        <f aca="true">IF($B101="","",IF($F101&lt;&gt;"","PAID",IF($C101&lt;TODAY(),"PAST DUE",IF($C101&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B101="","",IF($F101&lt;&gt;"",IF($C101&gt;TODAY(),"ADJUSTED","PAID"),IF($C101&lt;TODAY(),"PAST DUE",IF($C101&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -5113,7 +5141,7 @@
         <v>2201.95</v>
       </c>
       <c r="J102" s="46" t="str">
-        <f aca="true">IF($B102="","",IF($F102&lt;&gt;"","PAID",IF($C102&lt;TODAY(),"PAST DUE",IF($C102&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B102="","",IF($F102&lt;&gt;"",IF($C102&gt;TODAY(),"ADJUSTED","PAID"),IF($C102&lt;TODAY(),"PAST DUE",IF($C102&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -5148,7 +5176,7 @@
         <v>2196.96</v>
       </c>
       <c r="J103" s="46" t="str">
-        <f aca="true">IF($B103="","",IF($F103&lt;&gt;"","PAID",IF($C103&lt;TODAY(),"PAST DUE",IF($C103&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B103="","",IF($F103&lt;&gt;"",IF($C103&gt;TODAY(),"ADJUSTED","PAID"),IF($C103&lt;TODAY(),"PAST DUE",IF($C103&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -5183,7 +5211,7 @@
         <v>1696.96</v>
       </c>
       <c r="J104" s="46" t="str">
-        <f aca="true">IF($B104="","",IF($F104&lt;&gt;"","PAID",IF($C104&lt;TODAY(),"PAST DUE",IF($C104&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B104="","",IF($F104&lt;&gt;"",IF($C104&gt;TODAY(),"ADJUSTED","PAID"),IF($C104&lt;TODAY(),"PAST DUE",IF($C104&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -5218,7 +5246,7 @@
         <v>1786.96</v>
       </c>
       <c r="J105" s="46" t="str">
-        <f aca="true">IF($B105="","",IF($F105&lt;&gt;"","PAID",IF($C105&lt;TODAY(),"PAST DUE",IF($C105&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B105="","",IF($F105&lt;&gt;"",IF($C105&gt;TODAY(),"ADJUSTED","PAID"),IF($C105&lt;TODAY(),"PAST DUE",IF($C105&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -5253,7 +5281,7 @@
         <v>1623.46</v>
       </c>
       <c r="J106" s="46" t="str">
-        <f aca="true">IF($B106="","",IF($F106&lt;&gt;"","PAID",IF($C106&lt;TODAY(),"PAST DUE",IF($C106&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B106="","",IF($F106&lt;&gt;"",IF($C106&gt;TODAY(),"ADJUSTED","PAID"),IF($C106&lt;TODAY(),"PAST DUE",IF($C106&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -5288,7 +5316,7 @@
         <v/>
       </c>
       <c r="J107" s="46" t="str">
-        <f aca="true">IF($B107="","",IF($F107&lt;&gt;"","PAID",IF($C107&lt;TODAY(),"PAST DUE",IF($C107&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B107="","",IF($F107&lt;&gt;"",IF($C107&gt;TODAY(),"ADJUSTED","PAID"),IF($C107&lt;TODAY(),"PAST DUE",IF($C107&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -5323,13 +5351,13 @@
         <v/>
       </c>
       <c r="J108" s="46" t="str">
-        <f aca="true">IF($B108="","",IF($F108&lt;&gt;"","PAID",IF($C108&lt;TODAY(),"PAST DUE",IF($C108&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B108="","",IF($F108&lt;&gt;"",IF($C108&gt;TODAY(),"ADJUSTED","PAID"),IF($C108&lt;TODAY(),"PAST DUE",IF($C108&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B109" s="47" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C109" s="48"/>
       <c r="D109" s="48"/>
@@ -5462,7 +5490,7 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B116" s="52" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C116" s="53"/>
       <c r="D116" s="53"/>
@@ -5499,7 +5527,7 @@
       <c r="E118" s="32"/>
       <c r="F118" s="32"/>
       <c r="G118" s="33" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="H118" s="32"/>
       <c r="I118" s="34" t="n">
@@ -5514,19 +5542,19 @@
     </row>
     <row r="119" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B119" s="35" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C119" s="35" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D119" s="35" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E119" s="35" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F119" s="35" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G119" s="36" t="s">
         <v>18</v>
@@ -5535,10 +5563,10 @@
         <v>20</v>
       </c>
       <c r="I119" s="35" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="J119" s="35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5572,7 +5600,7 @@
         <v>2413.46</v>
       </c>
       <c r="J120" s="46" t="str">
-        <f aca="true">IF($B120="","",IF($F120&lt;&gt;"","PAID",IF($C120&lt;TODAY(),"PAST DUE",IF($C120&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B120="","",IF($F120&lt;&gt;"",IF($C120&gt;TODAY(),"ADJUSTED","PAID"),IF($C120&lt;TODAY(),"PAST DUE",IF($C120&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -5607,7 +5635,7 @@
         <v>2410.47</v>
       </c>
       <c r="J121" s="46" t="str">
-        <f aca="true">IF($B121="","",IF($F121&lt;&gt;"","PAID",IF($C121&lt;TODAY(),"PAST DUE",IF($C121&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B121="","",IF($F121&lt;&gt;"",IF($C121&gt;TODAY(),"ADJUSTED","PAID"),IF($C121&lt;TODAY(),"PAST DUE",IF($C121&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -5642,7 +5670,7 @@
         <v>2060.47</v>
       </c>
       <c r="J122" s="46" t="str">
-        <f aca="true">IF($B122="","",IF($F122&lt;&gt;"","PAID",IF($C122&lt;TODAY(),"PAST DUE",IF($C122&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B122="","",IF($F122&lt;&gt;"",IF($C122&gt;TODAY(),"ADJUSTED","PAID"),IF($C122&lt;TODAY(),"PAST DUE",IF($C122&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -5677,7 +5705,7 @@
         <v>2150.47</v>
       </c>
       <c r="J123" s="46" t="str">
-        <f aca="true">IF($B123="","",IF($F123&lt;&gt;"","PAID",IF($C123&lt;TODAY(),"PAST DUE",IF($C123&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B123="","",IF($F123&lt;&gt;"",IF($C123&gt;TODAY(),"ADJUSTED","PAID"),IF($C123&lt;TODAY(),"PAST DUE",IF($C123&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -5712,7 +5740,7 @@
         <v>1979.37</v>
       </c>
       <c r="J124" s="46" t="str">
-        <f aca="true">IF($B124="","",IF($F124&lt;&gt;"","PAID",IF($C124&lt;TODAY(),"PAST DUE",IF($C124&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B124="","",IF($F124&lt;&gt;"",IF($C124&gt;TODAY(),"ADJUSTED","PAID"),IF($C124&lt;TODAY(),"PAST DUE",IF($C124&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -5747,7 +5775,7 @@
         <v>1934.37</v>
       </c>
       <c r="J125" s="46" t="str">
-        <f aca="true">IF($B125="","",IF($F125&lt;&gt;"","PAID",IF($C125&lt;TODAY(),"PAST DUE",IF($C125&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B125="","",IF($F125&lt;&gt;"",IF($C125&gt;TODAY(),"ADJUSTED","PAID"),IF($C125&lt;TODAY(),"PAST DUE",IF($C125&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -5782,7 +5810,7 @@
         <v/>
       </c>
       <c r="J126" s="46" t="str">
-        <f aca="true">IF($B126="","",IF($F126&lt;&gt;"","PAID",IF($C126&lt;TODAY(),"PAST DUE",IF($C126&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B126="","",IF($F126&lt;&gt;"",IF($C126&gt;TODAY(),"ADJUSTED","PAID"),IF($C126&lt;TODAY(),"PAST DUE",IF($C126&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -5817,7 +5845,7 @@
         <v/>
       </c>
       <c r="J127" s="46" t="str">
-        <f aca="true">IF($B127="","",IF($F127&lt;&gt;"","PAID",IF($C127&lt;TODAY(),"PAST DUE",IF($C127&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B127="","",IF($F127&lt;&gt;"",IF($C127&gt;TODAY(),"ADJUSTED","PAID"),IF($C127&lt;TODAY(),"PAST DUE",IF($C127&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -5852,7 +5880,7 @@
         <v/>
       </c>
       <c r="J128" s="46" t="str">
-        <f aca="true">IF($B128="","",IF($F128&lt;&gt;"","PAID",IF($C128&lt;TODAY(),"PAST DUE",IF($C128&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B128="","",IF($F128&lt;&gt;"",IF($C128&gt;TODAY(),"ADJUSTED","PAID"),IF($C128&lt;TODAY(),"PAST DUE",IF($C128&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -5887,13 +5915,13 @@
         <v/>
       </c>
       <c r="J129" s="46" t="str">
-        <f aca="true">IF($B129="","",IF($F129&lt;&gt;"","PAID",IF($C129&lt;TODAY(),"PAST DUE",IF($C129&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B129="","",IF($F129&lt;&gt;"",IF($C129&gt;TODAY(),"ADJUSTED","PAID"),IF($C129&lt;TODAY(),"PAST DUE",IF($C129&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B130" s="47" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C130" s="48"/>
       <c r="D130" s="48"/>
@@ -6026,7 +6054,7 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B137" s="52" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C137" s="53"/>
       <c r="D137" s="53"/>
@@ -6063,7 +6091,7 @@
       <c r="E139" s="32"/>
       <c r="F139" s="32"/>
       <c r="G139" s="33" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="H139" s="32"/>
       <c r="I139" s="34" t="n">
@@ -6078,19 +6106,19 @@
     </row>
     <row r="140" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B140" s="35" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C140" s="35" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D140" s="35" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E140" s="35" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F140" s="35" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G140" s="36" t="s">
         <v>18</v>
@@ -6099,10 +6127,10 @@
         <v>20</v>
       </c>
       <c r="I140" s="35" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="J140" s="35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6136,7 +6164,7 @@
         <v>2724.37</v>
       </c>
       <c r="J141" s="46" t="str">
-        <f aca="true">IF($B141="","",IF($F141&lt;&gt;"","PAID",IF($C141&lt;TODAY(),"PAST DUE",IF($C141&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B141="","",IF($F141&lt;&gt;"",IF($C141&gt;TODAY(),"ADJUSTED","PAID"),IF($C141&lt;TODAY(),"PAST DUE",IF($C141&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -6171,7 +6199,7 @@
         <v>2707.38</v>
       </c>
       <c r="J142" s="46" t="str">
-        <f aca="true">IF($B142="","",IF($F142&lt;&gt;"","PAID",IF($C142&lt;TODAY(),"PAST DUE",IF($C142&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B142="","",IF($F142&lt;&gt;"",IF($C142&gt;TODAY(),"ADJUSTED","PAID"),IF($C142&lt;TODAY(),"PAST DUE",IF($C142&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -6206,7 +6234,7 @@
         <v>2797.38</v>
       </c>
       <c r="J143" s="46" t="str">
-        <f aca="true">IF($B143="","",IF($F143&lt;&gt;"","PAID",IF($C143&lt;TODAY(),"PAST DUE",IF($C143&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B143="","",IF($F143&lt;&gt;"",IF($C143&gt;TODAY(),"ADJUSTED","PAID"),IF($C143&lt;TODAY(),"PAST DUE",IF($C143&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -6241,7 +6269,7 @@
         <v/>
       </c>
       <c r="J144" s="46" t="str">
-        <f aca="true">IF($B144="","",IF($F144&lt;&gt;"","PAID",IF($C144&lt;TODAY(),"PAST DUE",IF($C144&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B144="","",IF($F144&lt;&gt;"",IF($C144&gt;TODAY(),"ADJUSTED","PAID"),IF($C144&lt;TODAY(),"PAST DUE",IF($C144&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -6276,7 +6304,7 @@
         <v/>
       </c>
       <c r="J145" s="46" t="str">
-        <f aca="true">IF($B145="","",IF($F145&lt;&gt;"","PAID",IF($C145&lt;TODAY(),"PAST DUE",IF($C145&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B145="","",IF($F145&lt;&gt;"",IF($C145&gt;TODAY(),"ADJUSTED","PAID"),IF($C145&lt;TODAY(),"PAST DUE",IF($C145&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -6311,7 +6339,7 @@
         <v/>
       </c>
       <c r="J146" s="46" t="str">
-        <f aca="true">IF($B146="","",IF($F146&lt;&gt;"","PAID",IF($C146&lt;TODAY(),"PAST DUE",IF($C146&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B146="","",IF($F146&lt;&gt;"",IF($C146&gt;TODAY(),"ADJUSTED","PAID"),IF($C146&lt;TODAY(),"PAST DUE",IF($C146&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -6346,7 +6374,7 @@
         <v/>
       </c>
       <c r="J147" s="46" t="str">
-        <f aca="true">IF($B147="","",IF($F147&lt;&gt;"","PAID",IF($C147&lt;TODAY(),"PAST DUE",IF($C147&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B147="","",IF($F147&lt;&gt;"",IF($C147&gt;TODAY(),"ADJUSTED","PAID"),IF($C147&lt;TODAY(),"PAST DUE",IF($C147&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -6381,7 +6409,7 @@
         <v/>
       </c>
       <c r="J148" s="46" t="str">
-        <f aca="true">IF($B148="","",IF($F148&lt;&gt;"","PAID",IF($C148&lt;TODAY(),"PAST DUE",IF($C148&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B148="","",IF($F148&lt;&gt;"",IF($C148&gt;TODAY(),"ADJUSTED","PAID"),IF($C148&lt;TODAY(),"PAST DUE",IF($C148&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -6416,7 +6444,7 @@
         <v/>
       </c>
       <c r="J149" s="46" t="str">
-        <f aca="true">IF($B149="","",IF($F149&lt;&gt;"","PAID",IF($C149&lt;TODAY(),"PAST DUE",IF($C149&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B149="","",IF($F149&lt;&gt;"",IF($C149&gt;TODAY(),"ADJUSTED","PAID"),IF($C149&lt;TODAY(),"PAST DUE",IF($C149&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -6451,13 +6479,13 @@
         <v/>
       </c>
       <c r="J150" s="46" t="str">
-        <f aca="true">IF($B150="","",IF($F150&lt;&gt;"","PAID",IF($C150&lt;TODAY(),"PAST DUE",IF($C150&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B150="","",IF($F150&lt;&gt;"",IF($C150&gt;TODAY(),"ADJUSTED","PAID"),IF($C150&lt;TODAY(),"PAST DUE",IF($C150&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B151" s="47" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C151" s="48"/>
       <c r="D151" s="48"/>
@@ -6590,7 +6618,7 @@
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B158" s="52" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C158" s="53"/>
       <c r="D158" s="53"/>
@@ -6627,7 +6655,7 @@
       <c r="E160" s="32"/>
       <c r="F160" s="32"/>
       <c r="G160" s="33" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="H160" s="32"/>
       <c r="I160" s="34" t="n">
@@ -6642,19 +6670,19 @@
     </row>
     <row r="161" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B161" s="35" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C161" s="35" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D161" s="35" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E161" s="35" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F161" s="35" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G161" s="36" t="s">
         <v>18</v>
@@ -6663,10 +6691,10 @@
         <v>20</v>
       </c>
       <c r="I161" s="35" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="J161" s="35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6700,7 +6728,7 @@
         <v>3587.38</v>
       </c>
       <c r="J162" s="46" t="str">
-        <f aca="true">IF($B162="","",IF($F162&lt;&gt;"","PAID",IF($C162&lt;TODAY(),"PAST DUE",IF($C162&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B162="","",IF($F162&lt;&gt;"",IF($C162&gt;TODAY(),"ADJUSTED","PAID"),IF($C162&lt;TODAY(),"PAST DUE",IF($C162&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -6735,7 +6763,7 @@
         <v>3573.68</v>
       </c>
       <c r="J163" s="46" t="str">
-        <f aca="true">IF($B163="","",IF($F163&lt;&gt;"","PAID",IF($C163&lt;TODAY(),"PAST DUE",IF($C163&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B163="","",IF($F163&lt;&gt;"",IF($C163&gt;TODAY(),"ADJUSTED","PAID"),IF($C163&lt;TODAY(),"PAST DUE",IF($C163&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -6770,7 +6798,7 @@
         <v>3529.81</v>
       </c>
       <c r="J164" s="46" t="str">
-        <f aca="true">IF($B164="","",IF($F164&lt;&gt;"","PAID",IF($C164&lt;TODAY(),"PAST DUE",IF($C164&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B164="","",IF($F164&lt;&gt;"",IF($C164&gt;TODAY(),"ADJUSTED","PAID"),IF($C164&lt;TODAY(),"PAST DUE",IF($C164&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -6805,7 +6833,7 @@
         <v>3619.81</v>
       </c>
       <c r="J165" s="46" t="str">
-        <f aca="true">IF($B165="","",IF($F165&lt;&gt;"","PAID",IF($C165&lt;TODAY(),"PAST DUE",IF($C165&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B165="","",IF($F165&lt;&gt;"",IF($C165&gt;TODAY(),"ADJUSTED","PAID"),IF($C165&lt;TODAY(),"PAST DUE",IF($C165&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -6840,7 +6868,7 @@
         <v>3269.81</v>
       </c>
       <c r="J166" s="46" t="str">
-        <f aca="true">IF($B166="","",IF($F166&lt;&gt;"","PAID",IF($C166&lt;TODAY(),"PAST DUE",IF($C166&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B166="","",IF($F166&lt;&gt;"",IF($C166&gt;TODAY(),"ADJUSTED","PAID"),IF($C166&lt;TODAY(),"PAST DUE",IF($C166&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -6875,7 +6903,7 @@
         <v>3119.81</v>
       </c>
       <c r="J167" s="46" t="str">
-        <f aca="true">IF($B167="","",IF($F167&lt;&gt;"","PAID",IF($C167&lt;TODAY(),"PAST DUE",IF($C167&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B167="","",IF($F167&lt;&gt;"",IF($C167&gt;TODAY(),"ADJUSTED","PAID"),IF($C167&lt;TODAY(),"PAST DUE",IF($C167&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -6910,7 +6938,7 @@
         <v>2976.44</v>
       </c>
       <c r="J168" s="46" t="str">
-        <f aca="true">IF($B168="","",IF($F168&lt;&gt;"","PAID",IF($C168&lt;TODAY(),"PAST DUE",IF($C168&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B168="","",IF($F168&lt;&gt;"",IF($C168&gt;TODAY(),"ADJUSTED","PAID"),IF($C168&lt;TODAY(),"PAST DUE",IF($C168&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -6945,7 +6973,7 @@
         <v/>
       </c>
       <c r="J169" s="46" t="str">
-        <f aca="true">IF($B169="","",IF($F169&lt;&gt;"","PAID",IF($C169&lt;TODAY(),"PAST DUE",IF($C169&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B169="","",IF($F169&lt;&gt;"",IF($C169&gt;TODAY(),"ADJUSTED","PAID"),IF($C169&lt;TODAY(),"PAST DUE",IF($C169&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -6980,7 +7008,7 @@
         <v/>
       </c>
       <c r="J170" s="46" t="str">
-        <f aca="true">IF($B170="","",IF($F170&lt;&gt;"","PAID",IF($C170&lt;TODAY(),"PAST DUE",IF($C170&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B170="","",IF($F170&lt;&gt;"",IF($C170&gt;TODAY(),"ADJUSTED","PAID"),IF($C170&lt;TODAY(),"PAST DUE",IF($C170&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -7015,13 +7043,13 @@
         <v/>
       </c>
       <c r="J171" s="46" t="str">
-        <f aca="true">IF($B171="","",IF($F171&lt;&gt;"","PAID",IF($C171&lt;TODAY(),"PAST DUE",IF($C171&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B171="","",IF($F171&lt;&gt;"",IF($C171&gt;TODAY(),"ADJUSTED","PAID"),IF($C171&lt;TODAY(),"PAST DUE",IF($C171&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B172" s="47" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C172" s="48"/>
       <c r="D172" s="48"/>
@@ -7154,7 +7182,7 @@
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B179" s="52" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C179" s="53"/>
       <c r="D179" s="53"/>
@@ -7191,7 +7219,7 @@
       <c r="E181" s="32"/>
       <c r="F181" s="32"/>
       <c r="G181" s="33" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="H181" s="32"/>
       <c r="I181" s="34" t="n">
@@ -7206,19 +7234,19 @@
     </row>
     <row r="182" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B182" s="35" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C182" s="35" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D182" s="35" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E182" s="35" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F182" s="35" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G182" s="36" t="s">
         <v>18</v>
@@ -7227,10 +7255,10 @@
         <v>20</v>
       </c>
       <c r="I182" s="35" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="J182" s="35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7264,7 +7292,7 @@
         <v>3766.44</v>
       </c>
       <c r="J183" s="46" t="str">
-        <f aca="true">IF($B183="","",IF($F183&lt;&gt;"","PAID",IF($C183&lt;TODAY(),"PAST DUE",IF($C183&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B183="","",IF($F183&lt;&gt;"",IF($C183&gt;TODAY(),"ADJUSTED","PAID"),IF($C183&lt;TODAY(),"PAST DUE",IF($C183&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -7299,7 +7327,7 @@
         <v>3745.34</v>
       </c>
       <c r="J184" s="46" t="str">
-        <f aca="true">IF($B184="","",IF($F184&lt;&gt;"","PAID",IF($C184&lt;TODAY(),"PAST DUE",IF($C184&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B184="","",IF($F184&lt;&gt;"",IF($C184&gt;TODAY(),"ADJUSTED","PAID"),IF($C184&lt;TODAY(),"PAST DUE",IF($C184&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -7334,7 +7362,7 @@
         <v>3725.34</v>
       </c>
       <c r="J185" s="46" t="str">
-        <f aca="true">IF($B185="","",IF($F185&lt;&gt;"","PAID",IF($C185&lt;TODAY(),"PAST DUE",IF($C185&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B185="","",IF($F185&lt;&gt;"",IF($C185&gt;TODAY(),"ADJUSTED","PAID"),IF($C185&lt;TODAY(),"PAST DUE",IF($C185&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -7369,7 +7397,7 @@
         <v>3715.34</v>
       </c>
       <c r="J186" s="46" t="str">
-        <f aca="true">IF($B186="","",IF($F186&lt;&gt;"","PAID",IF($C186&lt;TODAY(),"PAST DUE",IF($C186&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B186="","",IF($F186&lt;&gt;"",IF($C186&gt;TODAY(),"ADJUSTED","PAID"),IF($C186&lt;TODAY(),"PAST DUE",IF($C186&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -7404,7 +7432,7 @@
         <v>3805.34</v>
       </c>
       <c r="J187" s="46" t="str">
-        <f aca="true">IF($B187="","",IF($F187&lt;&gt;"","PAID",IF($C187&lt;TODAY(),"PAST DUE",IF($C187&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B187="","",IF($F187&lt;&gt;"",IF($C187&gt;TODAY(),"ADJUSTED","PAID"),IF($C187&lt;TODAY(),"PAST DUE",IF($C187&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -7439,7 +7467,7 @@
         <v>3800.35</v>
       </c>
       <c r="J188" s="46" t="str">
-        <f aca="true">IF($B188="","",IF($F188&lt;&gt;"","PAID",IF($C188&lt;TODAY(),"PAST DUE",IF($C188&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B188="","",IF($F188&lt;&gt;"",IF($C188&gt;TODAY(),"ADJUSTED","PAID"),IF($C188&lt;TODAY(),"PAST DUE",IF($C188&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -7474,7 +7502,7 @@
         <v>3300.35</v>
       </c>
       <c r="J189" s="46" t="str">
-        <f aca="true">IF($B189="","",IF($F189&lt;&gt;"","PAID",IF($C189&lt;TODAY(),"PAST DUE",IF($C189&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B189="","",IF($F189&lt;&gt;"",IF($C189&gt;TODAY(),"ADJUSTED","PAID"),IF($C189&lt;TODAY(),"PAST DUE",IF($C189&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -7509,7 +7537,7 @@
         <v/>
       </c>
       <c r="J190" s="46" t="str">
-        <f aca="true">IF($B190="","",IF($F190&lt;&gt;"","PAID",IF($C190&lt;TODAY(),"PAST DUE",IF($C190&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B190="","",IF($F190&lt;&gt;"",IF($C190&gt;TODAY(),"ADJUSTED","PAID"),IF($C190&lt;TODAY(),"PAST DUE",IF($C190&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -7544,7 +7572,7 @@
         <v/>
       </c>
       <c r="J191" s="46" t="str">
-        <f aca="true">IF($B191="","",IF($F191&lt;&gt;"","PAID",IF($C191&lt;TODAY(),"PAST DUE",IF($C191&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B191="","",IF($F191&lt;&gt;"",IF($C191&gt;TODAY(),"ADJUSTED","PAID"),IF($C191&lt;TODAY(),"PAST DUE",IF($C191&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -7579,13 +7607,13 @@
         <v/>
       </c>
       <c r="J192" s="46" t="str">
-        <f aca="true">IF($B192="","",IF($F192&lt;&gt;"","PAID",IF($C192&lt;TODAY(),"PAST DUE",IF($C192&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B192="","",IF($F192&lt;&gt;"",IF($C192&gt;TODAY(),"ADJUSTED","PAID"),IF($C192&lt;TODAY(),"PAST DUE",IF($C192&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B193" s="47" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C193" s="48"/>
       <c r="D193" s="48"/>
@@ -7718,7 +7746,7 @@
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B200" s="52" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C200" s="53"/>
       <c r="D200" s="53"/>
@@ -7755,7 +7783,7 @@
       <c r="E202" s="32"/>
       <c r="F202" s="32"/>
       <c r="G202" s="33" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="H202" s="32"/>
       <c r="I202" s="34" t="n">
@@ -7770,19 +7798,19 @@
     </row>
     <row r="203" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B203" s="35" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C203" s="35" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D203" s="35" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E203" s="35" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F203" s="35" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G203" s="36" t="s">
         <v>18</v>
@@ -7791,10 +7819,10 @@
         <v>20</v>
       </c>
       <c r="I203" s="35" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="J203" s="35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7828,7 +7856,7 @@
         <v>4090.35</v>
       </c>
       <c r="J204" s="46" t="str">
-        <f aca="true">IF($B204="","",IF($F204&lt;&gt;"","PAID",IF($C204&lt;TODAY(),"PAST DUE",IF($C204&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B204="","",IF($F204&lt;&gt;"",IF($C204&gt;TODAY(),"ADJUSTED","PAID"),IF($C204&lt;TODAY(),"PAST DUE",IF($C204&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -7863,7 +7891,7 @@
         <v>3926.85</v>
       </c>
       <c r="J205" s="46" t="str">
-        <f aca="true">IF($B205="","",IF($F205&lt;&gt;"","PAID",IF($C205&lt;TODAY(),"PAST DUE",IF($C205&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B205="","",IF($F205&lt;&gt;"",IF($C205&gt;TODAY(),"ADJUSTED","PAID"),IF($C205&lt;TODAY(),"PAST DUE",IF($C205&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -7898,7 +7926,7 @@
         <v>3923.86</v>
       </c>
       <c r="J206" s="46" t="str">
-        <f aca="true">IF($B206="","",IF($F206&lt;&gt;"","PAID",IF($C206&lt;TODAY(),"PAST DUE",IF($C206&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B206="","",IF($F206&lt;&gt;"",IF($C206&gt;TODAY(),"ADJUSTED","PAID"),IF($C206&lt;TODAY(),"PAST DUE",IF($C206&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -7933,7 +7961,7 @@
         <v>4013.86</v>
       </c>
       <c r="J207" s="46" t="str">
-        <f aca="true">IF($B207="","",IF($F207&lt;&gt;"","PAID",IF($C207&lt;TODAY(),"PAST DUE",IF($C207&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B207="","",IF($F207&lt;&gt;"",IF($C207&gt;TODAY(),"ADJUSTED","PAID"),IF($C207&lt;TODAY(),"PAST DUE",IF($C207&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -7968,7 +7996,7 @@
         <v>3663.86</v>
       </c>
       <c r="J208" s="46" t="str">
-        <f aca="true">IF($B208="","",IF($F208&lt;&gt;"","PAID",IF($C208&lt;TODAY(),"PAST DUE",IF($C208&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B208="","",IF($F208&lt;&gt;"",IF($C208&gt;TODAY(),"ADJUSTED","PAID"),IF($C208&lt;TODAY(),"PAST DUE",IF($C208&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -8003,7 +8031,7 @@
         <v/>
       </c>
       <c r="J209" s="46" t="str">
-        <f aca="true">IF($B209="","",IF($F209&lt;&gt;"","PAID",IF($C209&lt;TODAY(),"PAST DUE",IF($C209&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B209="","",IF($F209&lt;&gt;"",IF($C209&gt;TODAY(),"ADJUSTED","PAID"),IF($C209&lt;TODAY(),"PAST DUE",IF($C209&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -8038,7 +8066,7 @@
         <v/>
       </c>
       <c r="J210" s="46" t="str">
-        <f aca="true">IF($B210="","",IF($F210&lt;&gt;"","PAID",IF($C210&lt;TODAY(),"PAST DUE",IF($C210&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B210="","",IF($F210&lt;&gt;"",IF($C210&gt;TODAY(),"ADJUSTED","PAID"),IF($C210&lt;TODAY(),"PAST DUE",IF($C210&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -8073,7 +8101,7 @@
         <v/>
       </c>
       <c r="J211" s="46" t="str">
-        <f aca="true">IF($B211="","",IF($F211&lt;&gt;"","PAID",IF($C211&lt;TODAY(),"PAST DUE",IF($C211&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B211="","",IF($F211&lt;&gt;"",IF($C211&gt;TODAY(),"ADJUSTED","PAID"),IF($C211&lt;TODAY(),"PAST DUE",IF($C211&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -8108,7 +8136,7 @@
         <v/>
       </c>
       <c r="J212" s="46" t="str">
-        <f aca="true">IF($B212="","",IF($F212&lt;&gt;"","PAID",IF($C212&lt;TODAY(),"PAST DUE",IF($C212&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B212="","",IF($F212&lt;&gt;"",IF($C212&gt;TODAY(),"ADJUSTED","PAID"),IF($C212&lt;TODAY(),"PAST DUE",IF($C212&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -8143,13 +8171,13 @@
         <v/>
       </c>
       <c r="J213" s="46" t="str">
-        <f aca="true">IF($B213="","",IF($F213&lt;&gt;"","PAID",IF($C213&lt;TODAY(),"PAST DUE",IF($C213&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B213="","",IF($F213&lt;&gt;"",IF($C213&gt;TODAY(),"ADJUSTED","PAID"),IF($C213&lt;TODAY(),"PAST DUE",IF($C213&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B214" s="47" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C214" s="48"/>
       <c r="D214" s="48"/>
@@ -8282,7 +8310,7 @@
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B221" s="52" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C221" s="53"/>
       <c r="D221" s="53"/>
@@ -8319,7 +8347,7 @@
       <c r="E223" s="32"/>
       <c r="F223" s="32"/>
       <c r="G223" s="33" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="H223" s="32"/>
       <c r="I223" s="34" t="n">
@@ -8334,19 +8362,19 @@
     </row>
     <row r="224" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B224" s="35" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C224" s="35" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D224" s="35" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E224" s="35" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F224" s="35" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G224" s="36" t="s">
         <v>18</v>
@@ -8355,10 +8383,10 @@
         <v>20</v>
       </c>
       <c r="I224" s="35" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="J224" s="35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8392,7 +8420,7 @@
         <v>4453.86</v>
       </c>
       <c r="J225" s="46" t="str">
-        <f aca="true">IF($B225="","",IF($F225&lt;&gt;"","PAID",IF($C225&lt;TODAY(),"PAST DUE",IF($C225&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B225="","",IF($F225&lt;&gt;"",IF($C225&gt;TODAY(),"ADJUSTED","PAID"),IF($C225&lt;TODAY(),"PAST DUE",IF($C225&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -8427,7 +8455,7 @@
         <v>4282.76</v>
       </c>
       <c r="J226" s="46" t="str">
-        <f aca="true">IF($B226="","",IF($F226&lt;&gt;"","PAID",IF($C226&lt;TODAY(),"PAST DUE",IF($C226&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B226="","",IF($F226&lt;&gt;"",IF($C226&gt;TODAY(),"ADJUSTED","PAID"),IF($C226&lt;TODAY(),"PAST DUE",IF($C226&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -8462,7 +8490,7 @@
         <v>4237.76</v>
       </c>
       <c r="J227" s="46" t="str">
-        <f aca="true">IF($B227="","",IF($F227&lt;&gt;"","PAID",IF($C227&lt;TODAY(),"PAST DUE",IF($C227&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B227="","",IF($F227&lt;&gt;"",IF($C227&gt;TODAY(),"ADJUSTED","PAID"),IF($C227&lt;TODAY(),"PAST DUE",IF($C227&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -8497,7 +8525,7 @@
         <v>4220.77</v>
       </c>
       <c r="J228" s="46" t="str">
-        <f aca="true">IF($B228="","",IF($F228&lt;&gt;"","PAID",IF($C228&lt;TODAY(),"PAST DUE",IF($C228&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B228="","",IF($F228&lt;&gt;"",IF($C228&gt;TODAY(),"ADJUSTED","PAID"),IF($C228&lt;TODAY(),"PAST DUE",IF($C228&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -8532,7 +8560,7 @@
         <v>4310.77</v>
       </c>
       <c r="J229" s="46" t="str">
-        <f aca="true">IF($B229="","",IF($F229&lt;&gt;"","PAID",IF($C229&lt;TODAY(),"PAST DUE",IF($C229&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B229="","",IF($F229&lt;&gt;"",IF($C229&gt;TODAY(),"ADJUSTED","PAID"),IF($C229&lt;TODAY(),"PAST DUE",IF($C229&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -8567,7 +8595,7 @@
         <v/>
       </c>
       <c r="J230" s="46" t="str">
-        <f aca="true">IF($B230="","",IF($F230&lt;&gt;"","PAID",IF($C230&lt;TODAY(),"PAST DUE",IF($C230&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B230="","",IF($F230&lt;&gt;"",IF($C230&gt;TODAY(),"ADJUSTED","PAID"),IF($C230&lt;TODAY(),"PAST DUE",IF($C230&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -8602,7 +8630,7 @@
         <v/>
       </c>
       <c r="J231" s="46" t="str">
-        <f aca="true">IF($B231="","",IF($F231&lt;&gt;"","PAID",IF($C231&lt;TODAY(),"PAST DUE",IF($C231&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B231="","",IF($F231&lt;&gt;"",IF($C231&gt;TODAY(),"ADJUSTED","PAID"),IF($C231&lt;TODAY(),"PAST DUE",IF($C231&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -8637,7 +8665,7 @@
         <v/>
       </c>
       <c r="J232" s="46" t="str">
-        <f aca="true">IF($B232="","",IF($F232&lt;&gt;"","PAID",IF($C232&lt;TODAY(),"PAST DUE",IF($C232&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B232="","",IF($F232&lt;&gt;"",IF($C232&gt;TODAY(),"ADJUSTED","PAID"),IF($C232&lt;TODAY(),"PAST DUE",IF($C232&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -8672,7 +8700,7 @@
         <v/>
       </c>
       <c r="J233" s="46" t="str">
-        <f aca="true">IF($B233="","",IF($F233&lt;&gt;"","PAID",IF($C233&lt;TODAY(),"PAST DUE",IF($C233&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B233="","",IF($F233&lt;&gt;"",IF($C233&gt;TODAY(),"ADJUSTED","PAID"),IF($C233&lt;TODAY(),"PAST DUE",IF($C233&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -8707,13 +8735,13 @@
         <v/>
       </c>
       <c r="J234" s="46" t="str">
-        <f aca="true">IF($B234="","",IF($F234&lt;&gt;"","PAID",IF($C234&lt;TODAY(),"PAST DUE",IF($C234&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B234="","",IF($F234&lt;&gt;"",IF($C234&gt;TODAY(),"ADJUSTED","PAID"),IF($C234&lt;TODAY(),"PAST DUE",IF($C234&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B235" s="47" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C235" s="48"/>
       <c r="D235" s="48"/>
@@ -8846,7 +8874,7 @@
     </row>
     <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B242" s="52" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C242" s="53"/>
       <c r="D242" s="53"/>
@@ -8883,7 +8911,7 @@
       <c r="E244" s="32"/>
       <c r="F244" s="32"/>
       <c r="G244" s="33" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="H244" s="32"/>
       <c r="I244" s="34" t="n">
@@ -8898,19 +8926,19 @@
     </row>
     <row r="245" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B245" s="35" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C245" s="35" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D245" s="35" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E245" s="35" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F245" s="35" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G245" s="36" t="s">
         <v>18</v>
@@ -8919,10 +8947,10 @@
         <v>20</v>
       </c>
       <c r="I245" s="35" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="J245" s="35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8956,7 +8984,7 @@
         <v>5100.77</v>
       </c>
       <c r="J246" s="46" t="str">
-        <f aca="true">IF($B246="","",IF($F246&lt;&gt;"","PAID",IF($C246&lt;TODAY(),"PAST DUE",IF($C246&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B246="","",IF($F246&lt;&gt;"",IF($C246&gt;TODAY(),"ADJUSTED","PAID"),IF($C246&lt;TODAY(),"PAST DUE",IF($C246&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -8991,7 +9019,7 @@
         <v>5087.07</v>
       </c>
       <c r="J247" s="46" t="str">
-        <f aca="true">IF($B247="","",IF($F247&lt;&gt;"","PAID",IF($C247&lt;TODAY(),"PAST DUE",IF($C247&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B247="","",IF($F247&lt;&gt;"",IF($C247&gt;TODAY(),"ADJUSTED","PAID"),IF($C247&lt;TODAY(),"PAST DUE",IF($C247&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -9026,7 +9054,7 @@
         <v>5043.2</v>
       </c>
       <c r="J248" s="46" t="str">
-        <f aca="true">IF($B248="","",IF($F248&lt;&gt;"","PAID",IF($C248&lt;TODAY(),"PAST DUE",IF($C248&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B248="","",IF($F248&lt;&gt;"",IF($C248&gt;TODAY(),"ADJUSTED","PAID"),IF($C248&lt;TODAY(),"PAST DUE",IF($C248&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -9061,7 +9089,7 @@
         <v>5133.2</v>
       </c>
       <c r="J249" s="46" t="str">
-        <f aca="true">IF($B249="","",IF($F249&lt;&gt;"","PAID",IF($C249&lt;TODAY(),"PAST DUE",IF($C249&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B249="","",IF($F249&lt;&gt;"",IF($C249&gt;TODAY(),"ADJUSTED","PAID"),IF($C249&lt;TODAY(),"PAST DUE",IF($C249&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -9096,7 +9124,7 @@
         <v/>
       </c>
       <c r="J250" s="46" t="str">
-        <f aca="true">IF($B250="","",IF($F250&lt;&gt;"","PAID",IF($C250&lt;TODAY(),"PAST DUE",IF($C250&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B250="","",IF($F250&lt;&gt;"",IF($C250&gt;TODAY(),"ADJUSTED","PAID"),IF($C250&lt;TODAY(),"PAST DUE",IF($C250&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -9131,7 +9159,7 @@
         <v/>
       </c>
       <c r="J251" s="46" t="str">
-        <f aca="true">IF($B251="","",IF($F251&lt;&gt;"","PAID",IF($C251&lt;TODAY(),"PAST DUE",IF($C251&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B251="","",IF($F251&lt;&gt;"",IF($C251&gt;TODAY(),"ADJUSTED","PAID"),IF($C251&lt;TODAY(),"PAST DUE",IF($C251&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -9166,7 +9194,7 @@
         <v/>
       </c>
       <c r="J252" s="46" t="str">
-        <f aca="true">IF($B252="","",IF($F252&lt;&gt;"","PAID",IF($C252&lt;TODAY(),"PAST DUE",IF($C252&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B252="","",IF($F252&lt;&gt;"",IF($C252&gt;TODAY(),"ADJUSTED","PAID"),IF($C252&lt;TODAY(),"PAST DUE",IF($C252&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -9201,7 +9229,7 @@
         <v/>
       </c>
       <c r="J253" s="46" t="str">
-        <f aca="true">IF($B253="","",IF($F253&lt;&gt;"","PAID",IF($C253&lt;TODAY(),"PAST DUE",IF($C253&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B253="","",IF($F253&lt;&gt;"",IF($C253&gt;TODAY(),"ADJUSTED","PAID"),IF($C253&lt;TODAY(),"PAST DUE",IF($C253&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -9236,7 +9264,7 @@
         <v/>
       </c>
       <c r="J254" s="46" t="str">
-        <f aca="true">IF($B254="","",IF($F254&lt;&gt;"","PAID",IF($C254&lt;TODAY(),"PAST DUE",IF($C254&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B254="","",IF($F254&lt;&gt;"",IF($C254&gt;TODAY(),"ADJUSTED","PAID"),IF($C254&lt;TODAY(),"PAST DUE",IF($C254&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -9271,13 +9299,13 @@
         <v/>
       </c>
       <c r="J255" s="46" t="str">
-        <f aca="true">IF($B255="","",IF($F255&lt;&gt;"","PAID",IF($C255&lt;TODAY(),"PAST DUE",IF($C255&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B255="","",IF($F255&lt;&gt;"",IF($C255&gt;TODAY(),"ADJUSTED","PAID"),IF($C255&lt;TODAY(),"PAST DUE",IF($C255&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
     <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B256" s="47" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C256" s="48"/>
       <c r="D256" s="48"/>
@@ -9410,7 +9438,7 @@
     </row>
     <row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B263" s="52" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C263" s="53"/>
       <c r="D263" s="53"/>
@@ -9447,7 +9475,7 @@
       <c r="E265" s="32"/>
       <c r="F265" s="32"/>
       <c r="G265" s="33" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="H265" s="32"/>
       <c r="I265" s="34" t="n">
@@ -9462,19 +9490,19 @@
     </row>
     <row r="266" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B266" s="35" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C266" s="35" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D266" s="35" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E266" s="35" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F266" s="35" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G266" s="36" t="s">
         <v>18</v>
@@ -9483,10 +9511,10 @@
         <v>20</v>
       </c>
       <c r="I266" s="35" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="J266" s="35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="267" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9520,7 +9548,7 @@
         <v>5923.2</v>
       </c>
       <c r="J267" s="46" t="str">
-        <f aca="true">IF($B267="","",IF($F267&lt;&gt;"","PAID",IF($C267&lt;TODAY(),"PAST DUE",IF($C267&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B267="","",IF($F267&lt;&gt;"",IF($C267&gt;TODAY(),"ADJUSTED","PAID"),IF($C267&lt;TODAY(),"PAST DUE",IF($C267&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -9555,7 +9583,7 @@
         <v>5573.2</v>
       </c>
       <c r="J268" s="46" t="str">
-        <f aca="true">IF($B268="","",IF($F268&lt;&gt;"","PAID",IF($C268&lt;TODAY(),"PAST DUE",IF($C268&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B268="","",IF($F268&lt;&gt;"",IF($C268&gt;TODAY(),"ADJUSTED","PAID"),IF($C268&lt;TODAY(),"PAST DUE",IF($C268&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -9590,7 +9618,7 @@
         <v>5423.2</v>
       </c>
       <c r="J269" s="46" t="str">
-        <f aca="true">IF($B269="","",IF($F269&lt;&gt;"","PAID",IF($C269&lt;TODAY(),"PAST DUE",IF($C269&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B269="","",IF($F269&lt;&gt;"",IF($C269&gt;TODAY(),"ADJUSTED","PAID"),IF($C269&lt;TODAY(),"PAST DUE",IF($C269&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -9625,7 +9653,7 @@
         <v>5279.83</v>
       </c>
       <c r="J270" s="46" t="str">
-        <f aca="true">IF($B270="","",IF($F270&lt;&gt;"","PAID",IF($C270&lt;TODAY(),"PAST DUE",IF($C270&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B270="","",IF($F270&lt;&gt;"",IF($C270&gt;TODAY(),"ADJUSTED","PAID"),IF($C270&lt;TODAY(),"PAST DUE",IF($C270&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -9660,7 +9688,7 @@
         <v>5369.83</v>
       </c>
       <c r="J271" s="46" t="str">
-        <f aca="true">IF($B271="","",IF($F271&lt;&gt;"","PAID",IF($C271&lt;TODAY(),"PAST DUE",IF($C271&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B271="","",IF($F271&lt;&gt;"",IF($C271&gt;TODAY(),"ADJUSTED","PAID"),IF($C271&lt;TODAY(),"PAST DUE",IF($C271&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -9695,7 +9723,7 @@
         <v>5348.73</v>
       </c>
       <c r="J272" s="46" t="str">
-        <f aca="true">IF($B272="","",IF($F272&lt;&gt;"","PAID",IF($C272&lt;TODAY(),"PAST DUE",IF($C272&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B272="","",IF($F272&lt;&gt;"",IF($C272&gt;TODAY(),"ADJUSTED","PAID"),IF($C272&lt;TODAY(),"PAST DUE",IF($C272&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -9730,7 +9758,7 @@
         <v>5328.73</v>
       </c>
       <c r="J273" s="46" t="str">
-        <f aca="true">IF($B273="","",IF($F273&lt;&gt;"","PAID",IF($C273&lt;TODAY(),"PAST DUE",IF($C273&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B273="","",IF($F273&lt;&gt;"",IF($C273&gt;TODAY(),"ADJUSTED","PAID"),IF($C273&lt;TODAY(),"PAST DUE",IF($C273&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -9765,7 +9793,7 @@
         <v>5318.73</v>
       </c>
       <c r="J274" s="46" t="str">
-        <f aca="true">IF($B274="","",IF($F274&lt;&gt;"","PAID",IF($C274&lt;TODAY(),"PAST DUE",IF($C274&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B274="","",IF($F274&lt;&gt;"",IF($C274&gt;TODAY(),"ADJUSTED","PAID"),IF($C274&lt;TODAY(),"PAST DUE",IF($C274&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v>Upcoming</v>
       </c>
     </row>
@@ -9800,7 +9828,7 @@
         <v/>
       </c>
       <c r="J275" s="46" t="str">
-        <f aca="true">IF($B275="","",IF($F275&lt;&gt;"","PAID",IF($C275&lt;TODAY(),"PAST DUE",IF($C275&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B275="","",IF($F275&lt;&gt;"",IF($C275&gt;TODAY(),"ADJUSTED","PAID"),IF($C275&lt;TODAY(),"PAST DUE",IF($C275&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
@@ -9835,13 +9863,13 @@
         <v/>
       </c>
       <c r="J276" s="46" t="str">
-        <f aca="true">IF($B276="","",IF($F276&lt;&gt;"","PAID",IF($C276&lt;TODAY(),"PAST DUE",IF($C276&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
+        <f aca="true">IF($B276="","",IF($F276&lt;&gt;"",IF($C276&gt;TODAY(),"ADJUSTED","PAID"),IF($C276&lt;TODAY(),"PAST DUE",IF($C276&lt;=TODAY()+7,"DUE","Upcoming"))))</f>
         <v/>
       </c>
     </row>
     <row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B277" s="47" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C277" s="48"/>
       <c r="D277" s="48"/>
@@ -9974,7 +10002,7 @@
     </row>
     <row r="284" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B284" s="52" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C284" s="53"/>
       <c r="D284" s="53"/>
@@ -10060,17 +10088,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="57" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C4" s="57"/>
       <c r="D4" s="57"/>
@@ -10081,7 +10109,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="57" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C5" s="57"/>
       <c r="D5" s="57"/>
@@ -10096,7 +10124,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="57" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C6" s="57"/>
       <c r="D6" s="57"/>
@@ -10111,7 +10139,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="57" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="C7" s="57"/>
       <c r="D7" s="57"/>
@@ -10122,7 +10150,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="57" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C8" s="57"/>
       <c r="D8" s="57"/>
@@ -10133,7 +10161,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="57" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C9" s="57"/>
       <c r="D9" s="57"/>
@@ -10144,7 +10172,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="57" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C10" s="57"/>
       <c r="D10" s="57"/>
@@ -10155,34 +10183,34 @@
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="15" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="I12" s="15" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="J12" s="15" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="K12" s="15" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10720,10 +10748,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="56" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C26" s="71" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="D26" s="72" t="n">
         <f aca="false">$D$13</f>
@@ -10753,7 +10781,7 @@
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="73" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="C28" s="73"/>
       <c r="D28" s="73"/>
@@ -10823,47 +10851,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="74" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="75" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B3" s="75" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="C3" s="75" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D3" s="75" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E3" s="75" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F3" s="75" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="G3" s="75" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="H3" s="75" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="I3" s="75" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="J3" s="75" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="K3" s="75" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>